<commit_message>
Tableau actualisé avec graphique en sheet 2
</commit_message>
<xml_diff>
--- a/combined.xlsx
+++ b/combined.xlsx
@@ -218,11 +218,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
-    <numFmt numFmtId="167" formatCode="General"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -388,7 +387,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="28">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -409,10 +408,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -421,11 +416,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -437,7 +428,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -451,10 +442,6 @@
     </xf>
     <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -485,10 +472,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -501,11 +484,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -778,17 +757,16 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="1" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="15.07"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="18.25"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="18.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="10.41"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="14.58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="11.76"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16371" min="16336" style="1" width="10.16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16372" style="0" width="10.16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="10.41"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="14.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="11.76"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16336" style="1" width="10.16"/>
   </cols>
   <sheetData>
-    <row r="1" s="5" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -799,279 +777,168 @@
       <c r="F1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="4"/>
       <c r="H1" s="4" t="s">
         <v>2</v>
       </c>
       <c r="N1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="XDH1" s="4"/>
-      <c r="XDI1" s="4"/>
-      <c r="XDJ1" s="4"/>
-      <c r="XDK1" s="4"/>
-      <c r="XDL1" s="4"/>
-      <c r="XDM1" s="4"/>
-      <c r="XDN1" s="4"/>
-      <c r="XDO1" s="4"/>
-      <c r="XDP1" s="4"/>
-      <c r="XDQ1" s="4"/>
-      <c r="XDR1" s="4"/>
-      <c r="XDS1" s="4"/>
-      <c r="XDT1" s="4"/>
-      <c r="XDU1" s="4"/>
-      <c r="XDV1" s="4"/>
-      <c r="XDW1" s="4"/>
-      <c r="XDX1" s="4"/>
-      <c r="XDY1" s="4"/>
-      <c r="XDZ1" s="4"/>
-      <c r="XEA1" s="4"/>
-      <c r="XEB1" s="4"/>
-      <c r="XEC1" s="4"/>
-      <c r="XED1" s="4"/>
-      <c r="XEE1" s="4"/>
-      <c r="XEF1" s="4"/>
-      <c r="XEG1" s="4"/>
-      <c r="XEH1" s="4"/>
-      <c r="XEI1" s="4"/>
-      <c r="XEJ1" s="4"/>
-      <c r="XEK1" s="4"/>
-      <c r="XEL1" s="4"/>
-      <c r="XEM1" s="4"/>
-      <c r="XEN1" s="4"/>
-      <c r="XEO1" s="4"/>
-      <c r="XEP1" s="4"/>
-      <c r="XEQ1" s="4"/>
-      <c r="XFD1" s="0"/>
-    </row>
-    <row r="2" s="8" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="XFD1" s="1"/>
+    </row>
+    <row r="2" s="6" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2"/>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7" t="s">
+      <c r="H2" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="I2" s="7" t="s">
+      <c r="I2" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="L2" s="7" t="s">
+      <c r="L2" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="M2" s="7" t="s">
+      <c r="M2" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="N2" s="7" t="s">
+      <c r="N2" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="O2" s="7" t="s">
+      <c r="O2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="Q2" s="8" t="s">
+      <c r="Q2" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="XDH2" s="7"/>
-      <c r="XDI2" s="7"/>
-      <c r="XDJ2" s="7"/>
-      <c r="XDK2" s="7"/>
-      <c r="XDL2" s="7"/>
-      <c r="XDM2" s="7"/>
-      <c r="XDN2" s="7"/>
-      <c r="XDO2" s="7"/>
-      <c r="XDP2" s="7"/>
-      <c r="XDQ2" s="7"/>
-      <c r="XDR2" s="7"/>
-      <c r="XDS2" s="7"/>
-      <c r="XDT2" s="7"/>
-      <c r="XDU2" s="7"/>
-      <c r="XDV2" s="7"/>
-      <c r="XDW2" s="7"/>
-      <c r="XDX2" s="7"/>
-      <c r="XDY2" s="7"/>
-      <c r="XDZ2" s="7"/>
-      <c r="XEA2" s="7"/>
-      <c r="XEB2" s="7"/>
-      <c r="XEC2" s="7"/>
-      <c r="XED2" s="7"/>
-      <c r="XEE2" s="7"/>
-      <c r="XEF2" s="7"/>
-      <c r="XEG2" s="7"/>
-      <c r="XEH2" s="7"/>
-      <c r="XEI2" s="7"/>
-      <c r="XEJ2" s="7"/>
-      <c r="XEK2" s="7"/>
-      <c r="XEL2" s="7"/>
-      <c r="XEM2" s="7"/>
-      <c r="XEN2" s="7"/>
-      <c r="XEO2" s="7"/>
-      <c r="XEP2" s="7"/>
-      <c r="XEQ2" s="7"/>
-      <c r="XFD2" s="0"/>
-    </row>
-    <row r="3" s="8" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="XFD2" s="1"/>
+    </row>
+    <row r="3" s="6" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2"/>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6" t="s">
+      <c r="C3" s="5"/>
+      <c r="D3" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="6"/>
-      <c r="F3" s="7" t="s">
+      <c r="E3" s="5"/>
+      <c r="F3" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7" t="s">
+      <c r="H3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="I3" s="7" t="s">
+      <c r="I3" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="L3" s="7" t="s">
+      <c r="L3" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="N3" s="7" t="s">
+      <c r="N3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="O3" s="7" t="s">
+      <c r="O3" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="P3" s="8" t="s">
+      <c r="P3" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="Q3" s="9"/>
-      <c r="R3" s="8" t="s">
+      <c r="Q3" s="7"/>
+      <c r="R3" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="T3" s="8" t="s">
+      <c r="T3" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="XDH3" s="7"/>
-      <c r="XDI3" s="7"/>
-      <c r="XDJ3" s="7"/>
-      <c r="XDK3" s="7"/>
-      <c r="XDL3" s="7"/>
-      <c r="XDM3" s="7"/>
-      <c r="XDN3" s="7"/>
-      <c r="XDO3" s="7"/>
-      <c r="XDP3" s="7"/>
-      <c r="XDQ3" s="7"/>
-      <c r="XDR3" s="7"/>
-      <c r="XDS3" s="7"/>
-      <c r="XDT3" s="7"/>
-      <c r="XDU3" s="7"/>
-      <c r="XDV3" s="7"/>
-      <c r="XDW3" s="7"/>
-      <c r="XDX3" s="7"/>
-      <c r="XDY3" s="7"/>
-      <c r="XDZ3" s="7"/>
-      <c r="XEA3" s="7"/>
-      <c r="XEB3" s="7"/>
-      <c r="XEC3" s="7"/>
-      <c r="XED3" s="7"/>
-      <c r="XEE3" s="7"/>
-      <c r="XEF3" s="7"/>
-      <c r="XEG3" s="7"/>
-      <c r="XEH3" s="7"/>
-      <c r="XEI3" s="7"/>
-      <c r="XEJ3" s="7"/>
-      <c r="XEK3" s="7"/>
-      <c r="XEL3" s="7"/>
-      <c r="XEM3" s="7"/>
-      <c r="XEN3" s="7"/>
-      <c r="XEO3" s="7"/>
-      <c r="XEP3" s="7"/>
-      <c r="XEQ3" s="7"/>
-      <c r="XFD3" s="0"/>
-    </row>
-    <row r="4" s="12" customFormat="true" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10"/>
-      <c r="B4" s="11" t="s">
+      <c r="XFD3" s="1"/>
+    </row>
+    <row r="4" s="10" customFormat="true" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8"/>
+      <c r="B4" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E4" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="G4" s="11" t="s">
+      <c r="G4" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="J4" s="11" t="s">
+      <c r="J4" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="N4" s="11"/>
-      <c r="XDH4" s="11"/>
-      <c r="XDI4" s="11"/>
-      <c r="XDJ4" s="11"/>
-      <c r="XDK4" s="11"/>
-      <c r="XDL4" s="11"/>
-      <c r="XDM4" s="11"/>
-      <c r="XDN4" s="11"/>
-      <c r="XDO4" s="11"/>
-      <c r="XDP4" s="11"/>
-      <c r="XDQ4" s="11"/>
-      <c r="XDR4" s="11"/>
-      <c r="XDS4" s="11"/>
-      <c r="XDT4" s="11"/>
-      <c r="XDU4" s="11"/>
-      <c r="XDV4" s="11"/>
-      <c r="XDW4" s="11"/>
-      <c r="XDX4" s="11"/>
-      <c r="XDY4" s="11"/>
-      <c r="XDZ4" s="11"/>
-      <c r="XEA4" s="11"/>
-      <c r="XEB4" s="11"/>
-      <c r="XEC4" s="11"/>
-      <c r="XED4" s="11"/>
-      <c r="XEE4" s="11"/>
-      <c r="XEF4" s="11"/>
-      <c r="XEG4" s="11"/>
-      <c r="XEH4" s="11"/>
-      <c r="XEI4" s="11"/>
-      <c r="XEJ4" s="11"/>
-      <c r="XEK4" s="11"/>
-      <c r="XEL4" s="11"/>
-      <c r="XEM4" s="11"/>
-      <c r="XEN4" s="11"/>
-      <c r="XEO4" s="11"/>
-      <c r="XEP4" s="11"/>
-      <c r="XEQ4" s="11"/>
-      <c r="XFC4" s="0"/>
-      <c r="XFD4" s="0"/>
+      <c r="N4" s="9"/>
+      <c r="XDH4" s="9"/>
+      <c r="XDI4" s="9"/>
+      <c r="XDJ4" s="9"/>
+      <c r="XDK4" s="9"/>
+      <c r="XDL4" s="9"/>
+      <c r="XDM4" s="9"/>
+      <c r="XDN4" s="9"/>
+      <c r="XDO4" s="9"/>
+      <c r="XDP4" s="9"/>
+      <c r="XDQ4" s="9"/>
+      <c r="XDR4" s="9"/>
+      <c r="XDS4" s="9"/>
+      <c r="XDT4" s="9"/>
+      <c r="XDU4" s="9"/>
+      <c r="XDV4" s="9"/>
+      <c r="XDW4" s="9"/>
+      <c r="XDX4" s="9"/>
+      <c r="XDY4" s="9"/>
+      <c r="XDZ4" s="9"/>
+      <c r="XEA4" s="9"/>
+      <c r="XEB4" s="9"/>
+      <c r="XEC4" s="9"/>
+      <c r="XED4" s="9"/>
+      <c r="XEE4" s="9"/>
+      <c r="XEF4" s="9"/>
+      <c r="XEG4" s="9"/>
+      <c r="XEH4" s="9"/>
+      <c r="XEI4" s="9"/>
+      <c r="XEJ4" s="9"/>
+      <c r="XEK4" s="9"/>
+      <c r="XEL4" s="9"/>
+      <c r="XEM4" s="9"/>
+      <c r="XEN4" s="9"/>
+      <c r="XEO4" s="9"/>
+      <c r="XEP4" s="9"/>
+      <c r="XEQ4" s="9"/>
+      <c r="XFC4" s="1"/>
+      <c r="XFD4" s="1"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="B5" s="14" t="n">
+      <c r="B5" s="12" t="n">
         <v>141</v>
       </c>
-      <c r="C5" s="14" t="n">
+      <c r="C5" s="12" t="n">
         <v>446</v>
       </c>
-      <c r="D5" s="15" t="n">
+      <c r="D5" s="13" t="n">
         <v>26.4</v>
       </c>
-      <c r="E5" s="14" t="n">
+      <c r="E5" s="12" t="n">
         <v>920</v>
       </c>
       <c r="F5" s="1" t="n">
@@ -1106,37 +973,37 @@
       <c r="O5" s="1" t="n">
         <v>2.74</v>
       </c>
-      <c r="P5" s="16" t="n">
+      <c r="P5" s="1" t="n">
         <f aca="false">E5+D5+B5+0.8*C5+G5+J5</f>
         <v>4839.9</v>
       </c>
-      <c r="Q5" s="16" t="n">
+      <c r="Q5" s="1" t="n">
         <f aca="false">P5-$Q$34*O5/100</f>
         <v>3332.9</v>
       </c>
-      <c r="R5" s="16" t="n">
+      <c r="R5" s="1" t="n">
         <f aca="false">Q5/N5</f>
         <v>6.48045887614233</v>
       </c>
-      <c r="T5" s="16" t="n">
+      <c r="T5" s="1" t="n">
         <f aca="false">O5*50000/100</f>
         <v>1370</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="18" t="n">
+      <c r="B6" s="15" t="n">
         <v>200</v>
       </c>
-      <c r="C6" s="18" t="n">
+      <c r="C6" s="15" t="n">
         <v>248</v>
       </c>
-      <c r="D6" s="19" t="n">
+      <c r="D6" s="16" t="n">
         <v>61.1</v>
       </c>
-      <c r="E6" s="18" t="n">
+      <c r="E6" s="15" t="n">
         <v>722</v>
       </c>
       <c r="F6" s="1" t="n">
@@ -1171,37 +1038,37 @@
       <c r="O6" s="1" t="n">
         <v>3.42</v>
       </c>
-      <c r="P6" s="16" t="n">
+      <c r="P6" s="1" t="n">
         <f aca="false">E6+D6+B6+0.8*C6+G6+J6</f>
         <v>5758.3</v>
       </c>
-      <c r="Q6" s="16" t="n">
+      <c r="Q6" s="1" t="n">
         <f aca="false">P6-$Q$34*O6/100</f>
         <v>3877.3</v>
       </c>
-      <c r="R6" s="16" t="n">
+      <c r="R6" s="1" t="n">
         <f aca="false">Q6/N6</f>
         <v>6.03940809968847</v>
       </c>
-      <c r="T6" s="16" t="n">
+      <c r="T6" s="1" t="n">
         <f aca="false">O6*50000/100</f>
         <v>1710</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="14" t="n">
+      <c r="B7" s="12" t="n">
         <v>38</v>
       </c>
-      <c r="C7" s="14" t="n">
+      <c r="C7" s="12" t="n">
         <v>24</v>
       </c>
-      <c r="D7" s="15" t="n">
+      <c r="D7" s="13" t="n">
         <v>0.2</v>
       </c>
-      <c r="E7" s="14" t="n">
+      <c r="E7" s="12" t="n">
         <v>40</v>
       </c>
       <c r="F7" s="1" t="n">
@@ -1236,37 +1103,37 @@
       <c r="O7" s="1" t="n">
         <v>0.62</v>
       </c>
-      <c r="P7" s="16" t="n">
+      <c r="P7" s="1" t="n">
         <f aca="false">E7+D7+B7+0.8*C7+G7+J7</f>
         <v>689.4</v>
       </c>
-      <c r="Q7" s="16" t="n">
+      <c r="Q7" s="1" t="n">
         <f aca="false">P7-$Q$34*O7/100</f>
         <v>348.4</v>
       </c>
-      <c r="R7" s="16" t="n">
+      <c r="R7" s="1" t="n">
         <f aca="false">Q7/N7</f>
         <v>3.00344827586207</v>
       </c>
-      <c r="T7" s="16" t="n">
+      <c r="T7" s="1" t="n">
         <f aca="false">O7*50000/100</f>
         <v>310</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17" t="s">
+      <c r="A8" s="14" t="s">
         <v>30</v>
       </c>
-      <c r="B8" s="18" t="n">
+      <c r="B8" s="15" t="n">
         <v>46</v>
       </c>
-      <c r="C8" s="18" t="n">
+      <c r="C8" s="15" t="n">
         <v>36</v>
       </c>
-      <c r="D8" s="19" t="n">
+      <c r="D8" s="16" t="n">
         <v>0.3</v>
       </c>
-      <c r="E8" s="18" t="n">
+      <c r="E8" s="15" t="n">
         <v>36</v>
       </c>
       <c r="F8" s="1" t="n">
@@ -1301,35 +1168,35 @@
       <c r="O8" s="1" t="n">
         <v>0.49</v>
       </c>
-      <c r="P8" s="16" t="n">
+      <c r="P8" s="1" t="n">
         <f aca="false">E8+D8+B8+0.8*C8+G8+J8</f>
         <v>825.8</v>
       </c>
-      <c r="Q8" s="16" t="n">
+      <c r="Q8" s="1" t="n">
         <f aca="false">P8-$Q$34*O8/100</f>
         <v>556.3</v>
       </c>
-      <c r="R8" s="16" t="n">
+      <c r="R8" s="1" t="n">
         <f aca="false">ROUND(Q8/N8 *100/1000, 2)</f>
         <v>0.6</v>
       </c>
-      <c r="T8" s="16" t="n">
+      <c r="T8" s="1" t="n">
         <f aca="false">O8*50000/100</f>
         <v>245</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="13" t="s">
+      <c r="A9" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="B9" s="14" t="n">
+      <c r="B9" s="12" t="n">
         <v>16</v>
       </c>
-      <c r="C9" s="13"/>
-      <c r="D9" s="15" t="n">
+      <c r="C9" s="11"/>
+      <c r="D9" s="13" t="n">
         <v>0.8</v>
       </c>
-      <c r="E9" s="14" t="n">
+      <c r="E9" s="12" t="n">
         <v>46</v>
       </c>
       <c r="F9" s="1" t="n">
@@ -1364,37 +1231,37 @@
       <c r="O9" s="1" t="n">
         <v>0.19</v>
       </c>
-      <c r="P9" s="16" t="n">
+      <c r="P9" s="1" t="n">
         <f aca="false">E9+D9+B9+0.8*C9+G9+J9</f>
         <v>1026.8</v>
       </c>
-      <c r="Q9" s="16" t="n">
+      <c r="Q9" s="1" t="n">
         <f aca="false">P9-$Q$34*O9/100</f>
         <v>922.3</v>
       </c>
-      <c r="R9" s="16" t="n">
+      <c r="R9" s="1" t="n">
         <f aca="false">ROUND(Q9/N9 *100/1000, 2)</f>
         <v>2.53</v>
       </c>
-      <c r="T9" s="16" t="n">
+      <c r="T9" s="1" t="n">
         <f aca="false">O9*50000/100</f>
         <v>95</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="B10" s="18" t="n">
+      <c r="B10" s="15" t="n">
         <v>177</v>
       </c>
-      <c r="C10" s="18" t="n">
+      <c r="C10" s="15" t="n">
         <v>355</v>
       </c>
-      <c r="D10" s="19" t="n">
+      <c r="D10" s="16" t="n">
         <v>3.8</v>
       </c>
-      <c r="E10" s="18" t="n">
+      <c r="E10" s="15" t="n">
         <v>348</v>
       </c>
       <c r="F10" s="1" t="n">
@@ -1429,37 +1296,37 @@
       <c r="O10" s="1" t="n">
         <v>1.85</v>
       </c>
-      <c r="P10" s="16" t="n">
+      <c r="P10" s="1" t="n">
         <f aca="false">E10+D10+B10+0.8*C10+G10+J10</f>
         <v>2114.5</v>
       </c>
-      <c r="Q10" s="16" t="n">
+      <c r="Q10" s="1" t="n">
         <f aca="false">P10-$Q$34*O10/100</f>
         <v>1097</v>
       </c>
-      <c r="R10" s="16" t="n">
+      <c r="R10" s="1" t="n">
         <f aca="false">ROUND(Q10/N10 *100/1000, 2)</f>
         <v>0.32</v>
       </c>
-      <c r="T10" s="16" t="n">
+      <c r="T10" s="1" t="n">
         <f aca="false">O10*50000/100</f>
         <v>925</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="13" t="s">
+      <c r="A11" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="14" t="n">
+      <c r="B11" s="12" t="n">
         <v>106</v>
       </c>
-      <c r="C11" s="14" t="n">
+      <c r="C11" s="12" t="n">
         <v>350</v>
       </c>
-      <c r="D11" s="15" t="n">
+      <c r="D11" s="13" t="n">
         <v>113.8</v>
       </c>
-      <c r="E11" s="14" t="n">
+      <c r="E11" s="12" t="n">
         <v>533</v>
       </c>
       <c r="F11" s="1" t="n">
@@ -1494,37 +1361,37 @@
       <c r="O11" s="1" t="n">
         <v>2.22</v>
       </c>
-      <c r="P11" s="16" t="n">
+      <c r="P11" s="1" t="n">
         <f aca="false">E11+D11+B11+0.8*C11+G11+J11</f>
         <v>3369.3</v>
       </c>
-      <c r="Q11" s="16" t="n">
+      <c r="Q11" s="1" t="n">
         <f aca="false">P11-$Q$34*O11/100</f>
         <v>2148.3</v>
       </c>
-      <c r="R11" s="16" t="n">
+      <c r="R11" s="1" t="n">
         <f aca="false">ROUND(Q11/N11 *100/1000, 2)</f>
         <v>0.51</v>
       </c>
-      <c r="T11" s="16" t="n">
+      <c r="T11" s="1" t="n">
         <f aca="false">O11*50000/100</f>
         <v>1110</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17" t="s">
+      <c r="A12" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="18" t="n">
+      <c r="B12" s="15" t="n">
         <v>23</v>
       </c>
-      <c r="C12" s="18" t="n">
+      <c r="C12" s="15" t="n">
         <v>29</v>
       </c>
-      <c r="D12" s="19" t="n">
+      <c r="D12" s="16" t="n">
         <v>0.1</v>
       </c>
-      <c r="E12" s="18" t="n">
+      <c r="E12" s="15" t="n">
         <v>29</v>
       </c>
       <c r="F12" s="1" t="n">
@@ -1559,37 +1426,37 @@
       <c r="O12" s="1" t="n">
         <v>0.22</v>
       </c>
-      <c r="P12" s="16" t="n">
+      <c r="P12" s="1" t="n">
         <f aca="false">E12+D12+B12+0.8*C12+G12+J12</f>
         <v>256.3</v>
       </c>
-      <c r="Q12" s="16" t="n">
+      <c r="Q12" s="1" t="n">
         <f aca="false">P12-$Q$34*O12/100</f>
         <v>135.3</v>
       </c>
-      <c r="R12" s="16" t="n">
+      <c r="R12" s="1" t="n">
         <f aca="false">ROUND(Q12/N12 *100/1000, 2)</f>
         <v>0.32</v>
       </c>
-      <c r="T12" s="16" t="n">
+      <c r="T12" s="1" t="n">
         <f aca="false">O12*50000/100</f>
         <v>110</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="13" t="s">
+      <c r="A13" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="B13" s="14" t="n">
+      <c r="B13" s="12" t="n">
         <v>97</v>
       </c>
-      <c r="C13" s="14" t="n">
+      <c r="C13" s="12" t="n">
         <v>181</v>
       </c>
-      <c r="D13" s="15" t="n">
+      <c r="D13" s="13" t="n">
         <v>81.3</v>
       </c>
-      <c r="E13" s="14" t="n">
+      <c r="E13" s="12" t="n">
         <v>152</v>
       </c>
       <c r="F13" s="1" t="n">
@@ -1624,37 +1491,37 @@
       <c r="O13" s="1" t="n">
         <v>1.5</v>
       </c>
-      <c r="P13" s="16" t="n">
+      <c r="P13" s="1" t="n">
         <f aca="false">E13+D13+B13+0.8*C13+G13+J13</f>
         <v>2375.2</v>
       </c>
-      <c r="Q13" s="16" t="n">
+      <c r="Q13" s="1" t="n">
         <f aca="false">P13-$Q$34*O13/100</f>
         <v>1550.2</v>
       </c>
-      <c r="R13" s="16" t="n">
+      <c r="R13" s="1" t="n">
         <f aca="false">ROUND(Q13/N13 *100/1000, 2)</f>
         <v>0.55</v>
       </c>
-      <c r="T13" s="16" t="n">
+      <c r="T13" s="1" t="n">
         <f aca="false">O13*50000/100</f>
         <v>750</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="17" t="s">
+      <c r="A14" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="B14" s="18" t="n">
+      <c r="B14" s="15" t="n">
         <v>1078</v>
       </c>
-      <c r="C14" s="18" t="n">
+      <c r="C14" s="15" t="n">
         <v>2287</v>
       </c>
-      <c r="D14" s="18" t="n">
+      <c r="D14" s="15" t="n">
         <v>3100</v>
       </c>
-      <c r="E14" s="18" t="n">
+      <c r="E14" s="15" t="n">
         <v>6670</v>
       </c>
       <c r="F14" s="1" t="n">
@@ -1689,37 +1556,37 @@
       <c r="O14" s="1" t="n">
         <v>15.91</v>
       </c>
-      <c r="P14" s="16" t="n">
+      <c r="P14" s="1" t="n">
         <f aca="false">E14+D14+B14+0.8*C14+G14+J14</f>
         <v>37716.5</v>
       </c>
-      <c r="Q14" s="16" t="n">
+      <c r="Q14" s="1" t="n">
         <f aca="false">P14-$Q$34*O14/100</f>
         <v>28966</v>
       </c>
-      <c r="R14" s="16" t="n">
+      <c r="R14" s="1" t="n">
         <f aca="false">ROUND(Q14/N14 *100/1000, 2)</f>
         <v>0.97</v>
       </c>
-      <c r="T14" s="16" t="n">
+      <c r="T14" s="1" t="n">
         <f aca="false">O14*50000/100</f>
         <v>7955</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="13" t="s">
+      <c r="A15" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="B15" s="14" t="n">
+      <c r="B15" s="12" t="n">
         <v>973</v>
       </c>
-      <c r="C15" s="14" t="n">
+      <c r="C15" s="12" t="n">
         <v>3652</v>
       </c>
-      <c r="D15" s="15" t="n">
+      <c r="D15" s="13" t="n">
         <v>1595.2</v>
       </c>
-      <c r="E15" s="14" t="n">
+      <c r="E15" s="12" t="n">
         <v>8344</v>
       </c>
       <c r="F15" s="1" t="n">
@@ -1754,37 +1621,37 @@
       <c r="O15" s="1" t="n">
         <v>24.1</v>
       </c>
-      <c r="P15" s="16" t="n">
+      <c r="P15" s="1" t="n">
         <f aca="false">E15+D15+B15+0.8*C15+G15+J15</f>
         <v>41018.8</v>
       </c>
-      <c r="Q15" s="16" t="n">
+      <c r="Q15" s="1" t="n">
         <f aca="false">P15-$Q$34*O15/100</f>
         <v>27763.8</v>
       </c>
-      <c r="R15" s="16" t="n">
+      <c r="R15" s="1" t="n">
         <f aca="false">ROUND(Q15/N15 *100/1000, 2)</f>
         <v>0.61</v>
       </c>
-      <c r="T15" s="16" t="n">
+      <c r="T15" s="1" t="n">
         <f aca="false">O15*50000/100</f>
         <v>12050</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="17" t="s">
+      <c r="A16" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="B16" s="18" t="n">
+      <c r="B16" s="15" t="n">
         <v>91</v>
       </c>
-      <c r="C16" s="18" t="n">
+      <c r="C16" s="15" t="n">
         <v>74</v>
       </c>
-      <c r="D16" s="19" t="n">
+      <c r="D16" s="16" t="n">
         <v>22.7</v>
       </c>
-      <c r="E16" s="18" t="n">
+      <c r="E16" s="15" t="n">
         <v>118</v>
       </c>
       <c r="F16" s="1" t="n">
@@ -1819,37 +1686,37 @@
       <c r="O16" s="1" t="n">
         <v>1.32</v>
       </c>
-      <c r="P16" s="16" t="n">
+      <c r="P16" s="1" t="n">
         <f aca="false">E16+D16+B16+0.8*C16+G16+J16</f>
         <v>4088.6</v>
       </c>
-      <c r="Q16" s="16" t="n">
+      <c r="Q16" s="1" t="n">
         <f aca="false">P16-$Q$34*O16/100</f>
         <v>3362.6</v>
       </c>
-      <c r="R16" s="16" t="n">
+      <c r="R16" s="1" t="n">
         <f aca="false">ROUND(Q16/N16 *100/1000, 2)</f>
         <v>1.35</v>
       </c>
-      <c r="T16" s="16" t="n">
+      <c r="T16" s="1" t="n">
         <f aca="false">O16*50000/100</f>
         <v>660</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="13" t="s">
+      <c r="A17" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="B17" s="14" t="n">
+      <c r="B17" s="12" t="n">
         <v>139</v>
       </c>
-      <c r="C17" s="14" t="n">
+      <c r="C17" s="12" t="n">
         <v>153</v>
       </c>
-      <c r="D17" s="15" t="n">
+      <c r="D17" s="13" t="n">
         <v>5.9</v>
       </c>
-      <c r="E17" s="14" t="n">
+      <c r="E17" s="12" t="n">
         <v>208</v>
       </c>
       <c r="F17" s="1" t="n">
@@ -1884,37 +1751,37 @@
       <c r="O17" s="1" t="n">
         <v>1.16</v>
       </c>
-      <c r="P17" s="16" t="n">
+      <c r="P17" s="1" t="n">
         <f aca="false">E17+D17+B17+0.8*C17+G17+J17</f>
         <v>1578.1</v>
       </c>
-      <c r="Q17" s="16" t="n">
+      <c r="Q17" s="1" t="n">
         <f aca="false">P17-$Q$34*O17/100</f>
         <v>940.1</v>
       </c>
-      <c r="R17" s="16" t="n">
+      <c r="R17" s="1" t="n">
         <f aca="false">ROUND(Q17/N17 *100/1000, 2)</f>
         <v>0.43</v>
       </c>
-      <c r="T17" s="16" t="n">
+      <c r="T17" s="1" t="n">
         <f aca="false">O17*50000/100</f>
         <v>580</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="17" t="s">
+      <c r="A18" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="B18" s="18" t="n">
+      <c r="B18" s="15" t="n">
         <v>97</v>
       </c>
-      <c r="C18" s="18" t="n">
+      <c r="C18" s="15" t="n">
         <v>216</v>
       </c>
-      <c r="D18" s="19" t="n">
+      <c r="D18" s="16" t="n">
         <v>241.4</v>
       </c>
-      <c r="E18" s="18" t="n">
+      <c r="E18" s="15" t="n">
         <v>331</v>
       </c>
       <c r="F18" s="1" t="n">
@@ -1949,37 +1816,37 @@
       <c r="O18" s="1" t="n">
         <v>3.21</v>
       </c>
-      <c r="P18" s="16" t="n">
+      <c r="P18" s="1" t="n">
         <f aca="false">E18+D18+B18+0.8*C18+G18+J18</f>
         <v>3757.8</v>
       </c>
-      <c r="Q18" s="16" t="n">
+      <c r="Q18" s="1" t="n">
         <f aca="false">P18-$Q$34*O18/100</f>
         <v>1992.3</v>
       </c>
-      <c r="R18" s="16" t="n">
+      <c r="R18" s="1" t="n">
         <f aca="false">ROUND(Q18/N18 *100/1000, 2)</f>
         <v>0.33</v>
       </c>
-      <c r="T18" s="16" t="n">
+      <c r="T18" s="1" t="n">
         <f aca="false">O18*50000/100</f>
         <v>1605</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13" t="s">
+      <c r="A19" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="B19" s="14" t="n">
+      <c r="B19" s="12" t="n">
         <v>464</v>
       </c>
-      <c r="C19" s="14" t="n">
+      <c r="C19" s="12" t="n">
         <v>1205</v>
       </c>
-      <c r="D19" s="15" t="n">
+      <c r="D19" s="13" t="n">
         <v>544.5</v>
       </c>
-      <c r="E19" s="14" t="n">
+      <c r="E19" s="12" t="n">
         <v>2618</v>
       </c>
       <c r="F19" s="1" t="n">
@@ -2014,37 +1881,37 @@
       <c r="O19" s="1" t="n">
         <v>12.01</v>
       </c>
-      <c r="P19" s="16" t="n">
+      <c r="P19" s="1" t="n">
         <f aca="false">E19+D19+B19+0.8*C19+G19+J19</f>
         <v>22215.8</v>
       </c>
-      <c r="Q19" s="16" t="n">
+      <c r="Q19" s="1" t="n">
         <f aca="false">P19-$Q$34*O19/100</f>
         <v>15610.3</v>
       </c>
-      <c r="R19" s="16" t="n">
+      <c r="R19" s="1" t="n">
         <f aca="false">ROUND(Q19/N19 *100/1000, 2)</f>
         <v>0.69</v>
       </c>
-      <c r="T19" s="16" t="n">
+      <c r="T19" s="1" t="n">
         <f aca="false">O19*50000/100</f>
         <v>6005</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="17" t="s">
+      <c r="A20" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="B20" s="18" t="n">
+      <c r="B20" s="15" t="n">
         <v>27</v>
       </c>
-      <c r="C20" s="18" t="n">
+      <c r="C20" s="15" t="n">
         <v>27</v>
       </c>
-      <c r="D20" s="18" t="n">
+      <c r="D20" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="E20" s="18" t="n">
+      <c r="E20" s="15" t="n">
         <v>20</v>
       </c>
       <c r="F20" s="1" t="n">
@@ -2079,37 +1946,37 @@
       <c r="O20" s="1" t="n">
         <v>0.23</v>
       </c>
-      <c r="P20" s="16" t="n">
+      <c r="P20" s="1" t="n">
         <f aca="false">E20+D20+B20+0.8*C20+G20+J20</f>
         <v>407.7</v>
       </c>
-      <c r="Q20" s="16" t="n">
+      <c r="Q20" s="1" t="n">
         <f aca="false">P20-$Q$34*O20/100</f>
         <v>281.2</v>
       </c>
-      <c r="R20" s="16" t="n">
+      <c r="R20" s="1" t="n">
         <f aca="false">ROUND(Q20/N20 *100/1000, 2)</f>
         <v>0.65</v>
       </c>
-      <c r="T20" s="16" t="n">
+      <c r="T20" s="1" t="n">
         <f aca="false">O20*50000/100</f>
         <v>115</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="13" t="s">
+      <c r="A21" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="B21" s="14" t="n">
+      <c r="B21" s="12" t="n">
         <v>41</v>
       </c>
-      <c r="C21" s="14" t="n">
+      <c r="C21" s="12" t="n">
         <v>32</v>
       </c>
-      <c r="D21" s="15" t="n">
+      <c r="D21" s="13" t="n">
         <v>0.1</v>
       </c>
-      <c r="E21" s="14" t="n">
+      <c r="E21" s="12" t="n">
         <v>31</v>
       </c>
       <c r="F21" s="1" t="n">
@@ -2144,35 +2011,35 @@
       <c r="O21" s="1" t="n">
         <v>0.45</v>
       </c>
-      <c r="P21" s="16" t="n">
+      <c r="P21" s="1" t="n">
         <f aca="false">E21+D21+B21+0.8*C21+G21+J21</f>
         <v>425</v>
       </c>
-      <c r="Q21" s="16" t="n">
+      <c r="Q21" s="1" t="n">
         <f aca="false">P21-$Q$34*O21/100</f>
         <v>177.5</v>
       </c>
-      <c r="R21" s="16" t="n">
+      <c r="R21" s="1" t="n">
         <f aca="false">ROUND(Q21/N21 *100/1000, 2)</f>
         <v>0.21</v>
       </c>
-      <c r="T21" s="16" t="n">
+      <c r="T21" s="1" t="n">
         <f aca="false">O21*50000/100</f>
         <v>225</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="17" t="s">
+      <c r="A22" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="B22" s="18" t="n">
+      <c r="B22" s="15" t="n">
         <v>10</v>
       </c>
-      <c r="C22" s="17"/>
-      <c r="D22" s="18" t="n">
+      <c r="C22" s="14"/>
+      <c r="D22" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="E22" s="18" t="n">
+      <c r="E22" s="15" t="n">
         <v>208</v>
       </c>
       <c r="F22" s="1" t="n">
@@ -2207,35 +2074,35 @@
       <c r="O22" s="1" t="n">
         <v>0.48</v>
       </c>
-      <c r="P22" s="16" t="n">
+      <c r="P22" s="1" t="n">
         <f aca="false">E22+D22+B22+0.8*C22+G22+J22</f>
         <v>1923.5</v>
       </c>
-      <c r="Q22" s="16" t="n">
+      <c r="Q22" s="1" t="n">
         <f aca="false">P22-$Q$34*O22/100</f>
         <v>1659.5</v>
       </c>
-      <c r="R22" s="16" t="n">
+      <c r="R22" s="1" t="n">
         <f aca="false">ROUND(Q22/N22 *100/1000, 2)</f>
         <v>1.85</v>
       </c>
-      <c r="T22" s="16" t="n">
+      <c r="T22" s="1" t="n">
         <f aca="false">O22*50000/100</f>
         <v>240</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="13" t="s">
+      <c r="A23" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="B23" s="14" t="n">
+      <c r="B23" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="C23" s="13"/>
-      <c r="D23" s="14" t="n">
+      <c r="C23" s="11"/>
+      <c r="D23" s="12" t="n">
         <v>0</v>
       </c>
-      <c r="E23" s="14" t="n">
+      <c r="E23" s="12" t="n">
         <v>9</v>
       </c>
       <c r="F23" s="1" t="n">
@@ -2270,37 +2137,37 @@
       <c r="O23" s="1" t="n">
         <v>0.13</v>
       </c>
-      <c r="P23" s="16" t="n">
+      <c r="P23" s="1" t="n">
         <f aca="false">E23+D23+B23+0.8*C23+G23+J23</f>
         <v>417.7</v>
       </c>
-      <c r="Q23" s="16" t="n">
+      <c r="Q23" s="1" t="n">
         <f aca="false">P23-$Q$34*O23/100</f>
         <v>346.2</v>
       </c>
-      <c r="R23" s="16" t="n">
+      <c r="R23" s="1" t="n">
         <f aca="false">ROUND(Q23/N23 *100/1000, 2)</f>
         <v>1.41</v>
       </c>
-      <c r="T23" s="16" t="n">
+      <c r="T23" s="1" t="n">
         <f aca="false">O23*50000/100</f>
         <v>65</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="17" t="s">
+      <c r="A24" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="B24" s="18" t="n">
+      <c r="B24" s="15" t="n">
         <v>332</v>
       </c>
-      <c r="C24" s="18" t="n">
+      <c r="C24" s="15" t="n">
         <v>882</v>
       </c>
-      <c r="D24" s="18" t="n">
+      <c r="D24" s="15" t="n">
         <v>1961</v>
       </c>
-      <c r="E24" s="18" t="n">
+      <c r="E24" s="15" t="n">
         <v>913</v>
       </c>
       <c r="F24" s="1" t="n">
@@ -2335,37 +2202,37 @@
       <c r="O24" s="1" t="n">
         <v>6.23</v>
       </c>
-      <c r="P24" s="16" t="n">
+      <c r="P24" s="1" t="n">
         <f aca="false">E24+D24+B24+0.8*C24+G24+J24</f>
         <v>13742.2</v>
       </c>
-      <c r="Q24" s="16" t="n">
+      <c r="Q24" s="1" t="n">
         <f aca="false">P24-$Q$34*O24/100</f>
         <v>10315.7</v>
       </c>
-      <c r="R24" s="16" t="n">
+      <c r="R24" s="1" t="n">
         <f aca="false">ROUND(Q24/N24 *100/1000, 2)</f>
         <v>0.88</v>
       </c>
-      <c r="T24" s="16" t="n">
+      <c r="T24" s="1" t="n">
         <f aca="false">O24*50000/100</f>
         <v>3115</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="13" t="s">
+      <c r="A25" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="B25" s="14" t="n">
+      <c r="B25" s="12" t="n">
         <v>494</v>
       </c>
-      <c r="C25" s="14" t="n">
+      <c r="C25" s="12" t="n">
         <v>577</v>
       </c>
-      <c r="D25" s="14" t="n">
+      <c r="D25" s="12" t="n">
         <v>63</v>
       </c>
-      <c r="E25" s="14" t="n">
+      <c r="E25" s="12" t="n">
         <v>560</v>
       </c>
       <c r="F25" s="1" t="n">
@@ -2400,37 +2267,37 @@
       <c r="O25" s="1" t="n">
         <v>4.91</v>
       </c>
-      <c r="P25" s="16" t="n">
+      <c r="P25" s="1" t="n">
         <f aca="false">E25+D25+B25+0.8*C25+G25+J25</f>
         <v>4766.1</v>
       </c>
-      <c r="Q25" s="16" t="n">
+      <c r="Q25" s="1" t="n">
         <f aca="false">P25-$Q$34*O25/100</f>
         <v>2065.6</v>
       </c>
-      <c r="R25" s="16" t="n">
+      <c r="R25" s="1" t="n">
         <f aca="false">ROUND(Q25/N25 *100/1000, 2)</f>
         <v>0.22</v>
       </c>
-      <c r="T25" s="16" t="n">
+      <c r="T25" s="1" t="n">
         <f aca="false">O25*50000/100</f>
         <v>2455</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="17" t="s">
+      <c r="A26" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="B26" s="18" t="n">
+      <c r="B26" s="15" t="n">
         <v>136</v>
       </c>
-      <c r="C26" s="18" t="n">
+      <c r="C26" s="15" t="n">
         <v>114</v>
       </c>
-      <c r="D26" s="19" t="n">
+      <c r="D26" s="16" t="n">
         <v>24.9</v>
       </c>
-      <c r="E26" s="18" t="n">
+      <c r="E26" s="15" t="n">
         <v>330</v>
       </c>
       <c r="F26" s="1" t="n">
@@ -2465,37 +2332,37 @@
       <c r="O26" s="1" t="n">
         <v>1.63</v>
       </c>
-      <c r="P26" s="16" t="n">
+      <c r="P26" s="1" t="n">
         <f aca="false">E26+D26+B26+0.8*C26+G26+J26</f>
         <v>5356.3</v>
       </c>
-      <c r="Q26" s="16" t="n">
+      <c r="Q26" s="1" t="n">
         <f aca="false">P26-$Q$34*O26/100</f>
         <v>4459.8</v>
       </c>
-      <c r="R26" s="16" t="n">
+      <c r="R26" s="1" t="n">
         <f aca="false">ROUND(Q26/N26 *100/1000, 2)</f>
         <v>1.45</v>
       </c>
-      <c r="T26" s="16" t="n">
+      <c r="T26" s="1" t="n">
         <f aca="false">O26*50000/100</f>
         <v>815</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="13" t="s">
+      <c r="A27" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="B27" s="14" t="n">
+      <c r="B27" s="12" t="n">
         <v>133</v>
       </c>
-      <c r="C27" s="14" t="n">
+      <c r="C27" s="12" t="n">
         <v>40</v>
       </c>
-      <c r="D27" s="15" t="n">
+      <c r="D27" s="13" t="n">
         <v>1.9</v>
       </c>
-      <c r="E27" s="14" t="n">
+      <c r="E27" s="12" t="n">
         <v>121</v>
       </c>
       <c r="F27" s="1" t="n">
@@ -2530,37 +2397,37 @@
       <c r="O27" s="1" t="n">
         <v>2.02</v>
       </c>
-      <c r="P27" s="16" t="n">
+      <c r="P27" s="1" t="n">
         <f aca="false">E27+D27+B27+0.8*C27+G27+J27</f>
         <v>1581</v>
       </c>
-      <c r="Q27" s="16" t="n">
+      <c r="Q27" s="1" t="n">
         <f aca="false">P27-$Q$34*O27/100</f>
         <v>470</v>
       </c>
-      <c r="R27" s="16" t="n">
+      <c r="R27" s="1" t="n">
         <f aca="false">ROUND(Q27/N27 *100/1000, 2)</f>
         <v>0.12</v>
       </c>
-      <c r="T27" s="16" t="n">
+      <c r="T27" s="1" t="n">
         <f aca="false">O27*50000/100</f>
         <v>1010</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="17" t="s">
+      <c r="A28" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="B28" s="18" t="n">
+      <c r="B28" s="15" t="n">
         <v>76</v>
       </c>
-      <c r="C28" s="18" t="n">
+      <c r="C28" s="15" t="n">
         <v>51</v>
       </c>
-      <c r="D28" s="18" t="n">
+      <c r="D28" s="15" t="n">
         <v>0</v>
       </c>
-      <c r="E28" s="18" t="n">
+      <c r="E28" s="15" t="n">
         <v>19</v>
       </c>
       <c r="F28" s="1" t="n">
@@ -2595,37 +2462,37 @@
       <c r="O28" s="1" t="n">
         <v>0.73</v>
       </c>
-      <c r="P28" s="16" t="n">
+      <c r="P28" s="1" t="n">
         <f aca="false">E28+D28+B28+0.8*C28+G28+J28</f>
         <v>395.5</v>
       </c>
-      <c r="Q28" s="16" t="n">
+      <c r="Q28" s="1" t="n">
         <f aca="false">P28-$Q$34*O28/100</f>
         <v>-6</v>
       </c>
-      <c r="R28" s="16" t="n">
+      <c r="R28" s="1" t="n">
         <f aca="false">ROUND(Q28/N28 *100/1000, 2)</f>
         <v>-0</v>
       </c>
-      <c r="T28" s="16" t="n">
+      <c r="T28" s="1" t="n">
         <f aca="false">O28*50000/100</f>
         <v>365</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="13" t="s">
+      <c r="A29" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="B29" s="14" t="n">
+      <c r="B29" s="12" t="n">
         <v>33</v>
       </c>
-      <c r="C29" s="14" t="n">
+      <c r="C29" s="12" t="n">
         <v>18</v>
       </c>
-      <c r="D29" s="15" t="n">
+      <c r="D29" s="13" t="n">
         <v>0.4</v>
       </c>
-      <c r="E29" s="14" t="n">
+      <c r="E29" s="12" t="n">
         <v>75</v>
       </c>
       <c r="F29" s="1" t="n">
@@ -2660,37 +2527,37 @@
       <c r="O29" s="1" t="n">
         <v>0.38</v>
       </c>
-      <c r="P29" s="16" t="n">
+      <c r="P29" s="1" t="n">
         <f aca="false">E29+D29+B29+0.8*C29+G29+J29</f>
         <v>345.3</v>
       </c>
-      <c r="Q29" s="16" t="n">
+      <c r="Q29" s="1" t="n">
         <f aca="false">P29-$Q$34*O29/100</f>
         <v>136.3</v>
       </c>
-      <c r="R29" s="16" t="n">
+      <c r="R29" s="1" t="n">
         <f aca="false">ROUND(Q29/N29 *100/1000, 2)</f>
         <v>0.19</v>
       </c>
-      <c r="T29" s="16" t="n">
+      <c r="T29" s="1" t="n">
         <f aca="false">O29*50000/100</f>
         <v>190</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="17" t="s">
+      <c r="A30" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="B30" s="18" t="n">
+      <c r="B30" s="15" t="n">
         <v>683</v>
       </c>
-      <c r="C30" s="18" t="n">
+      <c r="C30" s="15" t="n">
         <v>1122</v>
       </c>
-      <c r="D30" s="19" t="n">
+      <c r="D30" s="16" t="n">
         <v>240.6</v>
       </c>
-      <c r="E30" s="18" t="n">
+      <c r="E30" s="15" t="n">
         <v>2151</v>
       </c>
       <c r="F30" s="1" t="n">
@@ -2725,37 +2592,37 @@
       <c r="O30" s="1" t="n">
         <v>8.98</v>
       </c>
-      <c r="P30" s="16" t="n">
+      <c r="P30" s="1" t="n">
         <f aca="false">E30+D30+B30+0.8*C30+G30+J30</f>
         <v>22621.6</v>
       </c>
-      <c r="Q30" s="16" t="n">
+      <c r="Q30" s="1" t="n">
         <f aca="false">P30-$Q$34*O30/100</f>
         <v>17682.6</v>
       </c>
-      <c r="R30" s="16" t="n">
+      <c r="R30" s="1" t="n">
         <f aca="false">ROUND(Q30/N30 *100/1000, 2)</f>
         <v>1.05</v>
       </c>
-      <c r="T30" s="16" t="n">
+      <c r="T30" s="1" t="n">
         <f aca="false">O30*50000/100</f>
         <v>4490</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="13" t="s">
+      <c r="A31" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="B31" s="14" t="n">
+      <c r="B31" s="12" t="n">
         <v>189</v>
       </c>
-      <c r="C31" s="14" t="n">
+      <c r="C31" s="12" t="n">
         <v>813</v>
       </c>
-      <c r="D31" s="15" t="n">
+      <c r="D31" s="13" t="n">
         <v>245.1</v>
       </c>
-      <c r="E31" s="14" t="n">
+      <c r="E31" s="12" t="n">
         <v>712</v>
       </c>
       <c r="F31" s="1" t="n">
@@ -2790,285 +2657,249 @@
       <c r="O31" s="1" t="n">
         <v>3.2</v>
       </c>
-      <c r="P31" s="16" t="n">
+      <c r="P31" s="1" t="n">
         <f aca="false">E31+D31+B31+0.8*C31+G31+J31</f>
         <v>4284.7</v>
       </c>
-      <c r="Q31" s="16" t="n">
+      <c r="Q31" s="1" t="n">
         <f aca="false">P31-$Q$34*O31/100</f>
         <v>2524.7</v>
       </c>
-      <c r="R31" s="16" t="n">
+      <c r="R31" s="1" t="n">
         <f aca="false">ROUND(Q31/N31 *100/1000, 2)</f>
         <v>0.42</v>
       </c>
-      <c r="T31" s="16" t="n">
+      <c r="T31" s="1" t="n">
         <f aca="false">O31*50000/100</f>
         <v>1600</v>
       </c>
     </row>
-    <row r="32" s="24" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="20" t="s">
+    <row r="32" s="20" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="B32" s="21" t="n">
+      <c r="B32" s="18" t="n">
         <v>5847</v>
       </c>
-      <c r="C32" s="21" t="n">
+      <c r="C32" s="18" t="n">
         <v>12930</v>
       </c>
-      <c r="D32" s="22" t="n">
+      <c r="D32" s="19" t="n">
         <v>8334.6</v>
       </c>
-      <c r="E32" s="21" t="n">
+      <c r="E32" s="18" t="n">
         <v>26264</v>
       </c>
-      <c r="F32" s="23" t="n">
+      <c r="F32" s="20" t="n">
         <v>100</v>
       </c>
-      <c r="G32" s="23" t="n">
+      <c r="G32" s="20" t="n">
         <f aca="false">F32*F$34*1000/100</f>
         <v>93000</v>
       </c>
-      <c r="H32" s="23" t="n">
+      <c r="H32" s="20" t="n">
         <v>299</v>
       </c>
-      <c r="I32" s="23" t="n">
+      <c r="I32" s="20" t="n">
         <v>100</v>
       </c>
-      <c r="J32" s="23" t="n">
+      <c r="J32" s="20" t="n">
         <f aca="false">I32*I$34/100*1000</f>
         <v>44000</v>
       </c>
-      <c r="K32" s="23" t="n">
+      <c r="K32" s="20" t="n">
         <v>44</v>
       </c>
-      <c r="L32" s="23" t="n">
+      <c r="L32" s="20" t="n">
         <v>100</v>
       </c>
-      <c r="N32" s="23" t="n">
+      <c r="N32" s="20" t="n">
         <v>18796</v>
       </c>
-      <c r="O32" s="23" t="n">
+      <c r="O32" s="20" t="n">
         <v>100</v>
       </c>
-      <c r="P32" s="24" t="n">
+      <c r="P32" s="20" t="n">
         <f aca="false">E32+D32+B32+0.8*C32+G32+J32</f>
         <v>187789.6</v>
       </c>
-      <c r="Q32" s="24" t="n">
+      <c r="Q32" s="20" t="n">
         <f aca="false">P32-$Q$34*O32/100</f>
         <v>132789.6</v>
       </c>
-      <c r="R32" s="24" t="n">
+      <c r="R32" s="20" t="n">
         <f aca="false">ROUND(Q32/N32 *100/1000, 2)</f>
         <v>0.71</v>
       </c>
-      <c r="T32" s="24" t="n">
+      <c r="T32" s="20" t="n">
         <f aca="false">O32*50000/100</f>
         <v>50000</v>
       </c>
-      <c r="XDH32" s="23"/>
-      <c r="XDI32" s="23"/>
-      <c r="XDJ32" s="23"/>
-      <c r="XDK32" s="23"/>
-      <c r="XDL32" s="23"/>
-      <c r="XDM32" s="23"/>
-      <c r="XDN32" s="23"/>
-      <c r="XDO32" s="23"/>
-      <c r="XDP32" s="23"/>
-      <c r="XDQ32" s="23"/>
-      <c r="XDR32" s="23"/>
-      <c r="XDS32" s="23"/>
-      <c r="XDT32" s="23"/>
-      <c r="XDU32" s="23"/>
-      <c r="XDV32" s="23"/>
-      <c r="XDW32" s="23"/>
-      <c r="XDX32" s="23"/>
-      <c r="XDY32" s="23"/>
-      <c r="XDZ32" s="23"/>
-      <c r="XEA32" s="23"/>
-      <c r="XEB32" s="23"/>
-      <c r="XEC32" s="23"/>
-      <c r="XED32" s="23"/>
-      <c r="XEE32" s="23"/>
-      <c r="XEF32" s="23"/>
-      <c r="XEG32" s="23"/>
-      <c r="XEH32" s="23"/>
-      <c r="XEI32" s="23"/>
-      <c r="XEJ32" s="23"/>
-      <c r="XEK32" s="23"/>
-      <c r="XEL32" s="23"/>
-      <c r="XEM32" s="23"/>
-      <c r="XEN32" s="23"/>
-      <c r="XEO32" s="23"/>
-      <c r="XEP32" s="23"/>
-      <c r="XEQ32" s="23"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="0" t="n">
+      <c r="B33" s="1" t="n">
         <f aca="false">SUM(B5:B31)</f>
         <v>5847</v>
       </c>
-      <c r="C33" s="0" t="n">
+      <c r="C33" s="1" t="n">
         <f aca="false">SUM(C5:C31)</f>
         <v>12932</v>
       </c>
-      <c r="D33" s="0" t="n">
+      <c r="D33" s="1" t="n">
         <f aca="false">SUM(D5:D31)</f>
         <v>8334.5</v>
       </c>
-      <c r="E33" s="0" t="n">
+      <c r="E33" s="1" t="n">
         <f aca="false">SUM(E5:E31)</f>
         <v>26264</v>
       </c>
-      <c r="G33" s="0" t="n">
+      <c r="G33" s="1" t="n">
         <f aca="false">SUM(G5:G31)</f>
         <v>93018.6</v>
       </c>
-      <c r="J33" s="0" t="n">
+      <c r="J33" s="1" t="n">
         <f aca="false">SUM(J5:J31)</f>
         <v>44088</v>
       </c>
-      <c r="P33" s="16" t="n">
+      <c r="P33" s="1" t="n">
         <f aca="false">SUM(P5:P31)</f>
         <v>187897.7</v>
       </c>
-      <c r="Q33" s="16" t="n">
+      <c r="Q33" s="1" t="n">
         <f aca="false">SUM(Q5:Q31)</f>
         <v>132716.2</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="F34" s="25" t="n">
+      <c r="F34" s="21" t="n">
         <v>93</v>
       </c>
-      <c r="I34" s="25" t="n">
+      <c r="I34" s="21" t="n">
         <v>44</v>
       </c>
-      <c r="Q34" s="0" t="n">
+      <c r="Q34" s="1" t="n">
         <v>55000</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N37" s="26" t="s">
+      <c r="N37" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="O37" s="27" t="n">
+      <c r="O37" s="23" t="n">
         <v>192.8</v>
       </c>
-      <c r="P37" s="28"/>
-      <c r="Q37" s="28"/>
+      <c r="P37" s="24"/>
+      <c r="Q37" s="24"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N38" s="26" t="s">
+      <c r="N38" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="O38" s="26" t="n">
+      <c r="O38" s="22" t="n">
         <f aca="false">O37*0.7</f>
         <v>134.96</v>
       </c>
-      <c r="P38" s="28"/>
-      <c r="Q38" s="28"/>
+      <c r="P38" s="24"/>
+      <c r="Q38" s="24"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N39" s="26"/>
-      <c r="O39" s="29"/>
-      <c r="P39" s="28"/>
-      <c r="Q39" s="28"/>
+      <c r="N39" s="22"/>
+      <c r="O39" s="22"/>
+      <c r="P39" s="24"/>
+      <c r="Q39" s="24"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N40" s="26" t="s">
+      <c r="N40" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="O40" s="29" t="n">
+      <c r="O40" s="22" t="n">
         <v>55</v>
       </c>
-      <c r="P40" s="28"/>
-      <c r="Q40" s="28"/>
+      <c r="P40" s="24"/>
+      <c r="Q40" s="24"/>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="N41" s="26" t="s">
+      <c r="N41" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="O41" s="29" t="n">
+      <c r="O41" s="22" t="n">
         <v>19</v>
       </c>
-      <c r="P41" s="28"/>
-      <c r="Q41" s="28"/>
+      <c r="P41" s="24"/>
+      <c r="Q41" s="24"/>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B42" s="30"/>
-      <c r="C42" s="30"/>
-      <c r="D42" s="30"/>
-      <c r="E42" s="30"/>
-      <c r="N42" s="26" t="s">
+      <c r="B42" s="25"/>
+      <c r="C42" s="25"/>
+      <c r="D42" s="25"/>
+      <c r="E42" s="25"/>
+      <c r="N42" s="22" t="s">
         <v>59</v>
       </c>
-      <c r="O42" s="26" t="n">
+      <c r="O42" s="22" t="n">
         <f aca="false">O37+O41</f>
         <v>211.8</v>
       </c>
-      <c r="P42" s="28"/>
-      <c r="Q42" s="28"/>
+      <c r="P42" s="24"/>
+      <c r="Q42" s="24"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="30"/>
-      <c r="C43" s="30" t="s">
+      <c r="B43" s="25"/>
+      <c r="C43" s="25" t="s">
         <v>60</v>
       </c>
-      <c r="D43" s="30"/>
-      <c r="E43" s="30"/>
-      <c r="N43" s="26" t="s">
+      <c r="D43" s="25"/>
+      <c r="E43" s="25"/>
+      <c r="N43" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="O43" s="26" t="n">
+      <c r="O43" s="22" t="n">
         <f aca="false">O38-O40</f>
         <v>79.96</v>
       </c>
-      <c r="P43" s="28"/>
-      <c r="Q43" s="28"/>
+      <c r="P43" s="24"/>
+      <c r="Q43" s="24"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="30"/>
-      <c r="C44" s="30"/>
-      <c r="D44" s="30"/>
-      <c r="E44" s="30"/>
-      <c r="N44" s="26" t="s">
+      <c r="B44" s="25"/>
+      <c r="C44" s="25"/>
+      <c r="D44" s="25"/>
+      <c r="E44" s="25"/>
+      <c r="N44" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="O44" s="26" t="n">
+      <c r="O44" s="22" t="n">
         <f aca="false">O43/O42</f>
         <v>0.37752596789424</v>
       </c>
-      <c r="P44" s="28"/>
-      <c r="Q44" s="28"/>
+      <c r="P44" s="24"/>
+      <c r="Q44" s="24"/>
     </row>
     <row r="47" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="31"/>
-      <c r="B47" s="32"/>
-      <c r="D47" s="32"/>
-      <c r="E47" s="32"/>
+      <c r="A47" s="26"/>
+      <c r="B47" s="27"/>
+      <c r="D47" s="27"/>
+      <c r="E47" s="27"/>
       <c r="J47" s="1"/>
-      <c r="Q47" s="16" t="s">
+      <c r="Q47" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="T47" s="16" t="s">
+      <c r="T47" s="1" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="31"/>
-      <c r="B49" s="32" t="s">
+      <c r="A49" s="26"/>
+      <c r="B49" s="27" t="s">
         <v>22</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D49" s="32" t="s">
+      <c r="D49" s="27" t="s">
         <v>24</v>
       </c>
-      <c r="E49" s="32" t="s">
+      <c r="E49" s="27" t="s">
         <v>25</v>
       </c>
       <c r="G49" s="1" t="s">

</xml_diff>

<commit_message>
Tableau avec valeurs pour jouer
</commit_message>
<xml_diff>
--- a/combined.xlsx
+++ b/combined.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="101">
   <si>
     <t xml:space="preserve">Country</t>
   </si>
@@ -79,7 +79,10 @@
     <t xml:space="preserve">Share s</t>
   </si>
   <si>
-    <t xml:space="preserve">With reduced share (55)</t>
+    <t xml:space="preserve">Our scenario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scenario 0</t>
   </si>
   <si>
     <t xml:space="preserve">proj.</t>
@@ -292,10 +295,22 @@
     <t xml:space="preserve">share GNI</t>
   </si>
   <si>
+    <t xml:space="preserve">Reward fund</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ajustable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOR</t>
+  </si>
+  <si>
     <t xml:space="preserve">GNI contrib reduction</t>
   </si>
   <si>
     <t xml:space="preserve">Ajout budg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Remboursement </t>
   </si>
   <si>
     <t xml:space="preserve">New budg</t>
@@ -314,10 +329,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0"/>
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
+    <numFmt numFmtId="167" formatCode="General"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -399,12 +415,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="14">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF8A65"/>
+        <bgColor rgb="FFFF9800"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -433,7 +455,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFB4C7DC"/>
-        <bgColor rgb="FF99CCFF"/>
+        <bgColor rgb="FFD1C4E9"/>
       </patternFill>
     </fill>
     <fill>
@@ -456,8 +478,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF333333"/>
-        <bgColor rgb="FF333300"/>
+        <fgColor rgb="FFD1C4E9"/>
+        <bgColor rgb="FFB4C7DC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCDD2"/>
+        <bgColor rgb="FFD1C4E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF9800"/>
+        <bgColor rgb="FFFFBF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -495,7 +529,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="40">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -504,16 +538,12 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -524,19 +554,31 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -556,19 +598,19 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -580,51 +622,67 @@
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="8" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="8" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="9" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="9" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="9" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="10" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="11" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -662,11 +720,11 @@
       <rgbColor rgb="FF729FCF"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFF2F7FF"/>
-      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFD9E1F2"/>
       <rgbColor rgb="FF650953"/>
-      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FFFF8A65"/>
       <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFD9E1F2"/>
+      <rgbColor rgb="FFD1C4E9"/>
       <rgbColor rgb="FF000080"/>
       <rgbColor rgb="FFFF00FF"/>
       <rgbColor rgb="FFFFFF00"/>
@@ -682,12 +740,12 @@
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FFFFCDD2"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>
       <rgbColor rgb="FFFFBF00"/>
-      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF9800"/>
       <rgbColor rgb="FFFF420E"/>
       <rgbColor rgb="FF5983B0"/>
       <rgbColor rgb="FFB3B3B3"/>
@@ -2115,11 +2173,11 @@
         </c:ser>
         <c:gapWidth val="100"/>
         <c:overlap val="100"/>
-        <c:axId val="10080540"/>
-        <c:axId val="73984353"/>
+        <c:axId val="36144290"/>
+        <c:axId val="94750663"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="10080540"/>
+        <c:axId val="36144290"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2151,7 +2209,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="73984353"/>
+        <c:crossAx val="94750663"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2159,7 +2217,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="73984353"/>
+        <c:axId val="94750663"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2189,7 +2247,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="10080540"/>
+        <c:crossAx val="36144290"/>
         <c:crossesAt val="0"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2245,14 +2303,14 @@
     <xdr:from>
       <xdr:col>1</xdr:col>
       <xdr:colOff>700560</xdr:colOff>
-      <xdr:row>38</xdr:row>
+      <xdr:row>40</xdr:row>
       <xdr:rowOff>97200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>7</xdr:col>
-      <xdr:colOff>1159200</xdr:colOff>
-      <xdr:row>70</xdr:row>
-      <xdr:rowOff>40320</xdr:rowOff>
+      <xdr:colOff>1158480</xdr:colOff>
+      <xdr:row>72</xdr:row>
+      <xdr:rowOff>39600</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2260,8 +2318,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="2460960" y="7635960"/>
-        <a:ext cx="10059840" cy="5658120"/>
+        <a:off x="2460960" y="7986600"/>
+        <a:ext cx="10059120" cy="5657400"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2385,7 +2443,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:XFD49"/>
+  <dimension ref="A1:XFD52"/>
   <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22"/>
@@ -2394,238 +2452,244 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="18.25"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="8.59"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="1" width="18.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="1" width="10.41"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="2" width="10.41"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="1" width="14.58"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="1" width="11.76"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="33" style="1" width="11.79"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16341" style="1" width="10.16"/>
   </cols>
   <sheetData>
-    <row r="1" s="4" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" s="5" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3" t="s">
+      <c r="B1" s="4"/>
+      <c r="C1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3" t="s">
+      <c r="D1" s="4"/>
+      <c r="E1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3" t="s">
+      <c r="F1" s="4"/>
+      <c r="G1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2" t="s">
+      <c r="H1" s="3"/>
+      <c r="I1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="J1" s="4" t="s">
+      <c r="J1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="4" t="s">
+      <c r="L1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="M1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="P1" s="4" t="s">
+      <c r="P1" s="5" t="s">
         <v>6</v>
       </c>
       <c r="S1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="AB1" s="4" t="s">
+      <c r="U1" s="6"/>
+      <c r="AB1" s="5" t="s">
         <v>8</v>
       </c>
       <c r="XFD1" s="1"/>
     </row>
-    <row r="2" s="6" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2"/>
-      <c r="B2" s="5" t="s">
+    <row r="2" s="8" customFormat="true" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3"/>
+      <c r="B2" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5" t="s">
+      <c r="C2" s="7"/>
+      <c r="D2" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5" t="s">
+      <c r="E2" s="7"/>
+      <c r="F2" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5" t="s">
+      <c r="G2" s="7"/>
+      <c r="H2" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="I2" s="5"/>
-      <c r="J2" s="6" t="s">
+      <c r="I2" s="7"/>
+      <c r="J2" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="M2" s="6" t="s">
+      <c r="M2" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="N2" s="6" t="s">
+      <c r="N2" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="Q2" s="6" t="s">
+      <c r="Q2" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="R2" s="6" t="s">
+      <c r="R2" s="8" t="s">
         <v>17</v>
       </c>
       <c r="S2" s="1"/>
-      <c r="T2" s="6" t="s">
+      <c r="T2" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="V2" s="6" t="s">
+      <c r="U2" s="6"/>
+      <c r="V2" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="AB2" s="6" t="s">
+      <c r="Y2" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="AB2" s="8" t="s">
         <v>16</v>
       </c>
       <c r="XFD2" s="1"/>
     </row>
-    <row r="3" s="6" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2"/>
-      <c r="B3" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5" t="s">
+    <row r="3" s="8" customFormat="true" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3"/>
+      <c r="B3" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
-      <c r="I3" s="5"/>
-      <c r="J3" s="6" t="s">
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="M3" s="6" t="s">
+      <c r="G3" s="7"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="7"/>
+      <c r="J3" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="N3" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="Q3" s="6" t="s">
-        <v>22</v>
+      <c r="M3" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="N3" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q3" s="8" t="s">
+        <v>23</v>
       </c>
       <c r="S3" s="1"/>
-      <c r="T3" s="6" t="s">
-        <v>22</v>
+      <c r="T3" s="8" t="s">
+        <v>23</v>
       </c>
       <c r="U3" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="V3" s="9"/>
+      <c r="W3" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y3" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB3" s="8" t="s">
         <v>24</v>
-      </c>
-      <c r="V3" s="7"/>
-      <c r="W3" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="Y3" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="AB3" s="6" t="s">
-        <v>23</v>
       </c>
       <c r="XFD3" s="1"/>
     </row>
-    <row r="4" s="10" customFormat="true" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8"/>
-      <c r="B4" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9" t="s">
+    <row r="4" s="12" customFormat="true" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="10"/>
+      <c r="B4" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9" t="s">
+      <c r="C4" s="11"/>
+      <c r="D4" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="G4" s="9"/>
-      <c r="H4" s="9" t="s">
+      <c r="E4" s="11"/>
+      <c r="F4" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="I4" s="9"/>
-      <c r="K4" s="9" t="s">
+      <c r="G4" s="11"/>
+      <c r="H4" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="I4" s="11"/>
+      <c r="K4" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="L4" s="9"/>
-      <c r="O4" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="P4" s="9"/>
+      <c r="L4" s="11"/>
+      <c r="O4" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="P4" s="11"/>
       <c r="S4" s="1"/>
-      <c r="AB4" s="9"/>
-      <c r="XDM4" s="9"/>
-      <c r="XDN4" s="9"/>
-      <c r="XDO4" s="9"/>
-      <c r="XDP4" s="9"/>
-      <c r="XDQ4" s="9"/>
-      <c r="XDR4" s="9"/>
-      <c r="XDS4" s="9"/>
-      <c r="XDT4" s="9"/>
-      <c r="XDU4" s="9"/>
-      <c r="XDV4" s="9"/>
-      <c r="XDW4" s="9"/>
-      <c r="XDX4" s="9"/>
-      <c r="XDY4" s="9"/>
-      <c r="XDZ4" s="9"/>
-      <c r="XEA4" s="9"/>
-      <c r="XEB4" s="9"/>
-      <c r="XEC4" s="9"/>
-      <c r="XED4" s="9"/>
-      <c r="XEE4" s="9"/>
-      <c r="XEF4" s="9"/>
-      <c r="XEG4" s="9"/>
-      <c r="XEH4" s="9"/>
-      <c r="XEI4" s="9"/>
-      <c r="XEJ4" s="9"/>
-      <c r="XEK4" s="9"/>
-      <c r="XEL4" s="9"/>
-      <c r="XEM4" s="9"/>
-      <c r="XEN4" s="9"/>
-      <c r="XEO4" s="9"/>
-      <c r="XEP4" s="9"/>
-      <c r="XEQ4" s="9"/>
-      <c r="XER4" s="9"/>
-      <c r="XES4" s="9"/>
-      <c r="XET4" s="9"/>
-      <c r="XEU4" s="9"/>
-      <c r="XEV4" s="9"/>
+      <c r="U4" s="2"/>
+      <c r="AB4" s="11"/>
+      <c r="XDM4" s="11"/>
+      <c r="XDN4" s="11"/>
+      <c r="XDO4" s="11"/>
+      <c r="XDP4" s="11"/>
+      <c r="XDQ4" s="11"/>
+      <c r="XDR4" s="11"/>
+      <c r="XDS4" s="11"/>
+      <c r="XDT4" s="11"/>
+      <c r="XDU4" s="11"/>
+      <c r="XDV4" s="11"/>
+      <c r="XDW4" s="11"/>
+      <c r="XDX4" s="11"/>
+      <c r="XDY4" s="11"/>
+      <c r="XDZ4" s="11"/>
+      <c r="XEA4" s="11"/>
+      <c r="XEB4" s="11"/>
+      <c r="XEC4" s="11"/>
+      <c r="XED4" s="11"/>
+      <c r="XEE4" s="11"/>
+      <c r="XEF4" s="11"/>
+      <c r="XEG4" s="11"/>
+      <c r="XEH4" s="11"/>
+      <c r="XEI4" s="11"/>
+      <c r="XEJ4" s="11"/>
+      <c r="XEK4" s="11"/>
+      <c r="XEL4" s="11"/>
+      <c r="XEM4" s="11"/>
+      <c r="XEN4" s="11"/>
+      <c r="XEO4" s="11"/>
+      <c r="XEP4" s="11"/>
+      <c r="XEQ4" s="11"/>
+      <c r="XER4" s="11"/>
+      <c r="XES4" s="11"/>
+      <c r="XET4" s="11"/>
+      <c r="XEU4" s="11"/>
+      <c r="XEV4" s="11"/>
       <c r="XFD4" s="1"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="B5" s="12" t="n">
+      <c r="A5" s="13" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="14" t="n">
         <v>141</v>
       </c>
-      <c r="C5" s="12" t="n">
+      <c r="C5" s="14" t="n">
         <f aca="false">1000*B5/$S5</f>
         <v>345.61025947732</v>
       </c>
-      <c r="D5" s="13" t="n">
+      <c r="D5" s="15" t="n">
         <v>330</v>
       </c>
-      <c r="E5" s="12" t="n">
+      <c r="E5" s="14" t="n">
         <f aca="false">1000*D5/$S5</f>
         <v>808.87507537245</v>
       </c>
-      <c r="F5" s="14" t="n">
+      <c r="F5" s="16" t="n">
         <v>26.4</v>
       </c>
-      <c r="G5" s="12" t="n">
+      <c r="G5" s="14" t="n">
         <f aca="false">1000*F5/$S5</f>
         <v>64.710006029796</v>
       </c>
-      <c r="H5" s="12" t="n">
+      <c r="H5" s="14" t="n">
         <v>920</v>
       </c>
-      <c r="I5" s="12" t="n">
+      <c r="I5" s="14" t="n">
         <f aca="false">1000*H5/$S5</f>
         <v>2255.04566467471</v>
       </c>
@@ -2635,7 +2699,7 @@
       <c r="K5" s="1" t="n">
         <v>1900</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="L5" s="14" t="n">
         <f aca="false">1000*K5/$S5</f>
         <v>4657.15952487168</v>
       </c>
@@ -2649,7 +2713,7 @@
         <f aca="false">N5*N$34/100*1000</f>
         <v>1452</v>
       </c>
-      <c r="P5" s="12" t="n">
+      <c r="P5" s="14" t="n">
         <f aca="false">1000*O5/$S5</f>
         <v>3559.05033163878</v>
       </c>
@@ -2665,17 +2729,17 @@
       <c r="T5" s="1" t="n">
         <v>2.74</v>
       </c>
-      <c r="U5" s="1" t="n">
+      <c r="U5" s="2" t="n">
         <f aca="false">H5+F5+B5+0.8*D5+K5+O5</f>
         <v>4703.4</v>
       </c>
       <c r="V5" s="1" t="n">
-        <f aca="false">U5-$V$34*T5/100</f>
-        <v>3196.4</v>
+        <f aca="false">U5-$T$42*1000*T5/100</f>
+        <v>3043.28606</v>
       </c>
       <c r="W5" s="1" t="n">
         <f aca="false">V5/S5</f>
-        <v>7.83481300278939</v>
+        <v>7.45950982170432</v>
       </c>
       <c r="Y5" s="1" t="n">
         <f aca="false">T5*50000/100</f>
@@ -2685,7 +2749,7 @@
         <v>514.3</v>
       </c>
       <c r="AG5" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="AH5" s="1" t="n">
         <v>1</v>
@@ -2703,34 +2767,34 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="B6" s="16" t="n">
+      <c r="A6" s="17" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" s="18" t="n">
         <v>200</v>
       </c>
-      <c r="C6" s="12" t="n">
+      <c r="C6" s="14" t="n">
         <f aca="false">1000*B6/$S6</f>
         <v>394.508442480669</v>
       </c>
-      <c r="D6" s="17" t="n">
+      <c r="D6" s="19" t="n">
         <v>184</v>
       </c>
-      <c r="E6" s="12" t="n">
+      <c r="E6" s="14" t="n">
         <f aca="false">1000*D6/$S6</f>
         <v>362.947767082216</v>
       </c>
-      <c r="F6" s="18" t="n">
+      <c r="F6" s="20" t="n">
         <v>61.1</v>
       </c>
-      <c r="G6" s="12" t="n">
+      <c r="G6" s="14" t="n">
         <f aca="false">1000*F6/$S6</f>
         <v>120.522329177844</v>
       </c>
-      <c r="H6" s="16" t="n">
+      <c r="H6" s="18" t="n">
         <v>722</v>
       </c>
-      <c r="I6" s="12" t="n">
+      <c r="I6" s="14" t="n">
         <f aca="false">1000*H6/$S6</f>
         <v>1424.17547735522</v>
       </c>
@@ -2740,7 +2804,7 @@
       <c r="K6" s="1" t="n">
         <v>1100</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="L6" s="14" t="n">
         <f aca="false">1000*K6/$S6</f>
         <v>2169.79643364368</v>
       </c>
@@ -2754,7 +2818,7 @@
         <f aca="false">N6*N$34/100*1000</f>
         <v>1452</v>
       </c>
-      <c r="P6" s="12" t="n">
+      <c r="P6" s="14" t="n">
         <f aca="false">1000*O6/$S6</f>
         <v>2864.13129240966</v>
       </c>
@@ -2770,17 +2834,17 @@
       <c r="T6" s="1" t="n">
         <v>3.42</v>
       </c>
-      <c r="U6" s="1" t="n">
+      <c r="U6" s="2" t="n">
         <f aca="false">H6+F6+B6+0.8*D6+K6+O6</f>
         <v>3682.3</v>
       </c>
       <c r="V6" s="1" t="n">
-        <f aca="false">U6-$V$34*T6/100</f>
-        <v>1801.3</v>
+        <f aca="false">U6-$T$42*1000*T6/100</f>
+        <v>1610.18698</v>
       </c>
       <c r="W6" s="1" t="n">
         <f aca="false">V6/S6</f>
-        <v>3.55314028720215</v>
+        <v>3.17616178791226</v>
       </c>
       <c r="Y6" s="1" t="n">
         <f aca="false">T6*50000/100</f>
@@ -2790,7 +2854,7 @@
         <v>642</v>
       </c>
       <c r="AG6" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="AH6" s="1" t="n">
         <v>1</v>
@@ -2808,34 +2872,34 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="B7" s="12" t="n">
+      <c r="A7" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="B7" s="14" t="n">
         <v>38</v>
       </c>
-      <c r="C7" s="12" t="n">
+      <c r="C7" s="14" t="n">
         <f aca="false">1000*B7/$S7</f>
         <v>726.008291778911</v>
       </c>
-      <c r="D7" s="13" t="n">
+      <c r="D7" s="15" t="n">
         <v>18</v>
       </c>
-      <c r="E7" s="12" t="n">
+      <c r="E7" s="14" t="n">
         <f aca="false">1000*D7/$S7</f>
         <v>343.898664526853</v>
       </c>
-      <c r="F7" s="14" t="n">
+      <c r="F7" s="16" t="n">
         <v>0.2</v>
       </c>
-      <c r="G7" s="12" t="n">
+      <c r="G7" s="14" t="n">
         <f aca="false">1000*F7/$S7</f>
         <v>3.82109627252059</v>
       </c>
-      <c r="H7" s="12" t="n">
+      <c r="H7" s="14" t="n">
         <v>40</v>
       </c>
-      <c r="I7" s="12" t="n">
+      <c r="I7" s="14" t="n">
         <f aca="false">1000*H7/$S7</f>
         <v>764.219254504117</v>
       </c>
@@ -2845,7 +2909,7 @@
       <c r="K7" s="1" t="n">
         <v>270</v>
       </c>
-      <c r="L7" s="12" t="n">
+      <c r="L7" s="14" t="n">
         <f aca="false">1000*K7/$S7</f>
         <v>5158.47996790279</v>
       </c>
@@ -2859,7 +2923,7 @@
         <f aca="false">N7*N$34/100*1000</f>
         <v>220</v>
       </c>
-      <c r="P7" s="12" t="n">
+      <c r="P7" s="14" t="n">
         <f aca="false">1000*O7/$S7</f>
         <v>4203.20589977264</v>
       </c>
@@ -2875,17 +2939,17 @@
       <c r="T7" s="1" t="n">
         <v>0.62</v>
       </c>
-      <c r="U7" s="1" t="n">
+      <c r="U7" s="2" t="n">
         <f aca="false">H7+F7+B7+0.8*D7+K7+O7</f>
         <v>582.6</v>
       </c>
       <c r="V7" s="1" t="n">
-        <f aca="false">U7-$V$34*T7/100</f>
-        <v>241.6</v>
+        <f aca="false">U7-$T$42*1000*T7/100</f>
+        <v>206.95378</v>
       </c>
       <c r="W7" s="1" t="n">
         <f aca="false">V7/S7</f>
-        <v>4.61588429720487</v>
+        <v>3.95395158671023</v>
       </c>
       <c r="Y7" s="1" t="n">
         <f aca="false">T7*50000/100</f>
@@ -2895,7 +2959,7 @@
         <v>116</v>
       </c>
       <c r="AG7" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="AH7" s="1" t="n">
         <v>0</v>
@@ -2913,34 +2977,34 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="B8" s="16" t="n">
+      <c r="A8" s="17" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" s="18" t="n">
         <v>46</v>
       </c>
-      <c r="C8" s="12" t="n">
+      <c r="C8" s="14" t="n">
         <f aca="false">1000*B8/$S8</f>
         <v>786.755148115208</v>
       </c>
-      <c r="D8" s="17" t="n">
+      <c r="D8" s="19" t="n">
         <v>26</v>
       </c>
-      <c r="E8" s="12" t="n">
+      <c r="E8" s="14" t="n">
         <f aca="false">1000*D8/$S8</f>
         <v>444.687692412944</v>
       </c>
-      <c r="F8" s="18" t="n">
+      <c r="F8" s="20" t="n">
         <v>0.3</v>
       </c>
-      <c r="G8" s="12" t="n">
+      <c r="G8" s="14" t="n">
         <f aca="false">1000*F8/$S8</f>
         <v>5.13101183553397</v>
       </c>
-      <c r="H8" s="16" t="n">
+      <c r="H8" s="18" t="n">
         <v>36</v>
       </c>
-      <c r="I8" s="12" t="n">
+      <c r="I8" s="14" t="n">
         <f aca="false">1000*H8/$S8</f>
         <v>615.721420264076</v>
       </c>
@@ -2950,7 +3014,7 @@
       <c r="K8" s="1" t="n">
         <v>380</v>
       </c>
-      <c r="L8" s="12" t="n">
+      <c r="L8" s="14" t="n">
         <f aca="false">1000*K8/$S8</f>
         <v>6499.28165834303</v>
       </c>
@@ -2964,7 +3028,7 @@
         <f aca="false">N8*N$34/100*1000</f>
         <v>352</v>
       </c>
-      <c r="P8" s="12" t="n">
+      <c r="P8" s="14" t="n">
         <f aca="false">1000*O8/$S8</f>
         <v>6020.38722035986</v>
       </c>
@@ -2980,17 +3044,17 @@
       <c r="T8" s="1" t="n">
         <v>0.49</v>
       </c>
-      <c r="U8" s="1" t="n">
-        <f aca="false">H8+F8+B8+0.8*D8+K8+O8</f>
-        <v>835.1</v>
+      <c r="U8" s="2" t="n">
+        <f aca="false">H8+F8+B8+D8+K8+O8</f>
+        <v>840.3</v>
       </c>
       <c r="V8" s="1" t="n">
-        <f aca="false">U8-$V$34*T8/100</f>
-        <v>565.6</v>
+        <f aca="false">U8-$T$42*1000*T8/100</f>
+        <v>543.41831</v>
       </c>
       <c r="W8" s="1" t="n">
         <f aca="false">ROUND(V8/S8 *100/1000, 2)</f>
-        <v>0.97</v>
+        <v>0.93</v>
       </c>
       <c r="Y8" s="1" t="n">
         <f aca="false">T8*50000/100</f>
@@ -3000,7 +3064,7 @@
         <v>93</v>
       </c>
       <c r="AG8" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="AH8" s="1" t="n">
         <v>0</v>
@@ -3018,32 +3082,32 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="B9" s="12" t="n">
+      <c r="A9" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="C9" s="12" t="n">
+      <c r="C9" s="14" t="n">
         <f aca="false">1000*B9/$S9</f>
         <v>727.603456116417</v>
       </c>
-      <c r="D9" s="19"/>
-      <c r="E9" s="12" t="n">
+      <c r="D9" s="21"/>
+      <c r="E9" s="14" t="n">
         <f aca="false">1000*D9/$S9</f>
         <v>0</v>
       </c>
-      <c r="F9" s="14" t="n">
+      <c r="F9" s="16" t="n">
         <v>0.8</v>
       </c>
-      <c r="G9" s="12" t="n">
+      <c r="G9" s="14" t="n">
         <f aca="false">1000*F9/$S9</f>
         <v>36.3801728058208</v>
       </c>
-      <c r="H9" s="12" t="n">
+      <c r="H9" s="14" t="n">
         <v>46</v>
       </c>
-      <c r="I9" s="12" t="n">
+      <c r="I9" s="14" t="n">
         <f aca="false">1000*H9/$S9</f>
         <v>2091.8599363347</v>
       </c>
@@ -3053,7 +3117,7 @@
       <c r="K9" s="1" t="n">
         <v>290</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="L9" s="14" t="n">
         <f aca="false">1000*K9/$S9</f>
         <v>13187.8126421101</v>
       </c>
@@ -3067,7 +3131,7 @@
         <f aca="false">N9*N$34/100*1000</f>
         <v>220</v>
       </c>
-      <c r="P9" s="12" t="n">
+      <c r="P9" s="14" t="n">
         <f aca="false">1000*O9/$S9</f>
         <v>10004.5475216007</v>
       </c>
@@ -3083,17 +3147,17 @@
       <c r="T9" s="1" t="n">
         <v>0.19</v>
       </c>
-      <c r="U9" s="1" t="n">
-        <f aca="false">H9+F9+B9+0.8*D9+K9+O9</f>
+      <c r="U9" s="2" t="n">
+        <f aca="false">H9+F9+B9+D9+K9+O9</f>
         <v>572.8</v>
       </c>
       <c r="V9" s="1" t="n">
-        <f aca="false">U9-$V$34*T9/100</f>
-        <v>468.3</v>
+        <f aca="false">U9-$T$42*1000*T9/100</f>
+        <v>457.68261</v>
       </c>
       <c r="W9" s="1" t="n">
         <f aca="false">ROUND(V9/S9 *100/1000, 2)</f>
-        <v>2.13</v>
+        <v>2.08</v>
       </c>
       <c r="Y9" s="1" t="n">
         <f aca="false">T9*50000/100</f>
@@ -3103,7 +3167,7 @@
         <v>36.5</v>
       </c>
       <c r="AG9" s="1" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="AH9" s="1" t="n">
         <v>0</v>
@@ -3121,34 +3185,34 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="B10" s="16" t="n">
+      <c r="A10" s="17" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10" s="18" t="n">
         <v>177</v>
       </c>
-      <c r="C10" s="12" t="n">
+      <c r="C10" s="14" t="n">
         <f aca="false">1000*B10/$S10</f>
         <v>777.772407095745</v>
       </c>
-      <c r="D10" s="17" t="n">
+      <c r="D10" s="19" t="n">
         <v>263</v>
       </c>
-      <c r="E10" s="12" t="n">
+      <c r="E10" s="14" t="n">
         <f aca="false">1000*D10/$S10</f>
         <v>1155.67312466769</v>
       </c>
-      <c r="F10" s="18" t="n">
+      <c r="F10" s="20" t="n">
         <v>3.8</v>
       </c>
-      <c r="G10" s="12" t="n">
+      <c r="G10" s="14" t="n">
         <f aca="false">1000*F10/$S10</f>
         <v>16.6979386834115</v>
       </c>
-      <c r="H10" s="16" t="n">
+      <c r="H10" s="18" t="n">
         <v>348</v>
       </c>
-      <c r="I10" s="12" t="n">
+      <c r="I10" s="14" t="n">
         <f aca="false">1000*H10/$S10</f>
         <v>1529.17964784926</v>
       </c>
@@ -3158,7 +3222,7 @@
       <c r="K10" s="1" t="n">
         <v>440</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="L10" s="14" t="n">
         <f aca="false">1000*K10/$S10</f>
         <v>1933.44553176343</v>
       </c>
@@ -3172,7 +3236,7 @@
         <f aca="false">N10*N$34/100*1000</f>
         <v>660</v>
       </c>
-      <c r="P10" s="12" t="n">
+      <c r="P10" s="14" t="n">
         <f aca="false">1000*O10/$S10</f>
         <v>2900.16829764515</v>
       </c>
@@ -3188,17 +3252,17 @@
       <c r="T10" s="1" t="n">
         <v>1.85</v>
       </c>
-      <c r="U10" s="1" t="n">
-        <f aca="false">H10+F10+B10+0.8*D10+K10+O10</f>
-        <v>1839.2</v>
+      <c r="U10" s="2" t="n">
+        <f aca="false">H10+F10+B10+D10+K10+O10</f>
+        <v>1891.8</v>
       </c>
       <c r="V10" s="1" t="n">
-        <f aca="false">U10-$V$34*T10/100</f>
-        <v>821.7</v>
+        <f aca="false">U10-$T$42*1000*T10/100</f>
+        <v>770.92015</v>
       </c>
       <c r="W10" s="1" t="n">
         <f aca="false">ROUND(V10/S10 *100/1000, 2)</f>
-        <v>0.36</v>
+        <v>0.34</v>
       </c>
       <c r="Y10" s="1" t="n">
         <f aca="false">T10*50000/100</f>
@@ -3208,7 +3272,7 @@
         <v>347.3</v>
       </c>
       <c r="AG10" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="AH10" s="1" t="n">
         <v>0</v>
@@ -3226,34 +3290,34 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="B11" s="12" t="n">
+      <c r="A11" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" s="14" t="n">
         <v>106</v>
       </c>
-      <c r="C11" s="12" t="n">
+      <c r="C11" s="14" t="n">
         <f aca="false">1000*B11/$S11</f>
         <v>304.277684963515</v>
       </c>
-      <c r="D11" s="13" t="n">
+      <c r="D11" s="15" t="n">
         <v>258</v>
       </c>
-      <c r="E11" s="12" t="n">
+      <c r="E11" s="14" t="n">
         <f aca="false">1000*D11/$S11</f>
         <v>740.600403024405</v>
       </c>
-      <c r="F11" s="14" t="n">
+      <c r="F11" s="16" t="n">
         <v>113.8</v>
       </c>
-      <c r="G11" s="12" t="n">
+      <c r="G11" s="14" t="n">
         <f aca="false">1000*F11/$S11</f>
         <v>326.667929706114</v>
       </c>
-      <c r="H11" s="12" t="n">
+      <c r="H11" s="14" t="n">
         <v>533</v>
       </c>
-      <c r="I11" s="12" t="n">
+      <c r="I11" s="14" t="n">
         <f aca="false">1000*H11/$S11</f>
         <v>1530.00005741088</v>
       </c>
@@ -3263,7 +3327,7 @@
       <c r="K11" s="1" t="n">
         <v>1130</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="L11" s="14" t="n">
         <f aca="false">1000*K11/$S11</f>
         <v>3243.71494347899</v>
       </c>
@@ -3277,7 +3341,7 @@
         <f aca="false">N11*N$34/100*1000</f>
         <v>616</v>
       </c>
-      <c r="P11" s="12" t="n">
+      <c r="P11" s="14" t="n">
         <f aca="false">1000*O11/$S11</f>
         <v>1768.25522582571</v>
       </c>
@@ -3293,17 +3357,17 @@
       <c r="T11" s="1" t="n">
         <v>2.22</v>
       </c>
-      <c r="U11" s="1" t="n">
-        <f aca="false">H11+F11+B11+0.8*D11+K11+O11</f>
-        <v>2705.2</v>
+      <c r="U11" s="2" t="n">
+        <f aca="false">H11+F11+B11+D11+K11+O11</f>
+        <v>2756.8</v>
       </c>
       <c r="V11" s="1" t="n">
-        <f aca="false">U11-$V$34*T11/100</f>
-        <v>1484.2</v>
+        <f aca="false">U11-$T$42*1000*T11/100</f>
+        <v>1411.74418</v>
       </c>
       <c r="W11" s="1" t="n">
         <f aca="false">ROUND(V11/S11 *100/1000, 2)</f>
-        <v>0.43</v>
+        <v>0.41</v>
       </c>
       <c r="Y11" s="1" t="n">
         <f aca="false">T11*50000/100</f>
@@ -3313,7 +3377,7 @@
         <v>417.8</v>
       </c>
       <c r="AG11" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="AH11" s="1" t="n">
         <v>1</v>
@@ -3331,34 +3395,34 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="B12" s="16" t="n">
+      <c r="A12" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" s="18" t="n">
         <v>23</v>
       </c>
-      <c r="C12" s="12" t="n">
+      <c r="C12" s="14" t="n">
         <f aca="false">1000*B12/$S12</f>
         <v>744.360658921001</v>
       </c>
-      <c r="D12" s="17" t="n">
+      <c r="D12" s="19" t="n">
         <v>21</v>
       </c>
-      <c r="E12" s="12" t="n">
+      <c r="E12" s="14" t="n">
         <f aca="false">1000*D12/$S12</f>
         <v>679.633645101783</v>
       </c>
-      <c r="F12" s="18" t="n">
+      <c r="F12" s="20" t="n">
         <v>0.1</v>
       </c>
-      <c r="G12" s="12" t="n">
+      <c r="G12" s="14" t="n">
         <f aca="false">1000*F12/$S12</f>
         <v>3.23635069096087</v>
       </c>
-      <c r="H12" s="16" t="n">
+      <c r="H12" s="18" t="n">
         <v>29</v>
       </c>
-      <c r="I12" s="12" t="n">
+      <c r="I12" s="14" t="n">
         <f aca="false">1000*H12/$S12</f>
         <v>938.541700378653</v>
       </c>
@@ -3368,7 +3432,7 @@
       <c r="K12" s="1" t="n">
         <v>900</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="L12" s="14" t="n">
         <f aca="false">1000*K12/$S12</f>
         <v>29127.1562186479</v>
       </c>
@@ -3382,7 +3446,7 @@
         <f aca="false">N12*N$34/100*1000</f>
         <v>88</v>
       </c>
-      <c r="P12" s="12" t="n">
+      <c r="P12" s="14" t="n">
         <f aca="false">1000*O12/$S12</f>
         <v>2847.98860804557</v>
       </c>
@@ -3398,17 +3462,17 @@
       <c r="T12" s="1" t="n">
         <v>0.22</v>
       </c>
-      <c r="U12" s="1" t="n">
-        <f aca="false">H12+F12+B12+0.8*D12+K12+O12</f>
-        <v>1056.9</v>
+      <c r="U12" s="2" t="n">
+        <f aca="false">H12+F12+B12+D12+K12+O12</f>
+        <v>1061.1</v>
       </c>
       <c r="V12" s="1" t="n">
-        <f aca="false">U12-$V$34*T12/100</f>
-        <v>935.9</v>
+        <f aca="false">U12-$T$42*1000*T12/100</f>
+        <v>927.80618</v>
       </c>
       <c r="W12" s="1" t="n">
         <f aca="false">ROUND(V12/S12 *100/1000, 2)</f>
-        <v>3.03</v>
+        <v>3</v>
       </c>
       <c r="Y12" s="1" t="n">
         <f aca="false">T12*50000/100</f>
@@ -3418,7 +3482,7 @@
         <v>41.9</v>
       </c>
       <c r="AG12" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="AH12" s="1" t="n">
         <v>0</v>
@@ -3436,34 +3500,34 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="B13" s="12" t="n">
+      <c r="A13" s="13" t="s">
+        <v>49</v>
+      </c>
+      <c r="B13" s="14" t="n">
         <v>97</v>
       </c>
-      <c r="C13" s="12" t="n">
+      <c r="C13" s="14" t="n">
         <f aca="false">1000*B13/$S13</f>
         <v>379.785988637743</v>
       </c>
-      <c r="D13" s="13" t="n">
+      <c r="D13" s="15" t="n">
         <v>133</v>
       </c>
-      <c r="E13" s="12" t="n">
+      <c r="E13" s="14" t="n">
         <f aca="false">1000*D13/$S13</f>
         <v>520.737489575462</v>
       </c>
-      <c r="F13" s="14" t="n">
+      <c r="F13" s="16" t="n">
         <v>81.3</v>
       </c>
-      <c r="G13" s="12" t="n">
+      <c r="G13" s="14" t="n">
         <f aca="false">1000*F13/$S13</f>
         <v>318.315472951015</v>
       </c>
-      <c r="H13" s="12" t="n">
+      <c r="H13" s="14" t="n">
         <v>152</v>
       </c>
-      <c r="I13" s="12" t="n">
+      <c r="I13" s="14" t="n">
         <f aca="false">1000*H13/$S13</f>
         <v>595.128559514814</v>
       </c>
@@ -3473,7 +3537,7 @@
       <c r="K13" s="1" t="n">
         <v>720</v>
       </c>
-      <c r="L13" s="12" t="n">
+      <c r="L13" s="14" t="n">
         <f aca="false">1000*K13/$S13</f>
         <v>2819.03001875438</v>
       </c>
@@ -3487,7 +3551,7 @@
         <f aca="false">N13*N$34/100*1000</f>
         <v>440</v>
       </c>
-      <c r="P13" s="12" t="n">
+      <c r="P13" s="14" t="n">
         <f aca="false">1000*O13/$S13</f>
         <v>1722.74056701657</v>
       </c>
@@ -3503,17 +3567,17 @@
       <c r="T13" s="1" t="n">
         <v>1.5</v>
       </c>
-      <c r="U13" s="1" t="n">
-        <f aca="false">H13+F13+B13+0.8*D13+K13+O13</f>
-        <v>1596.7</v>
+      <c r="U13" s="2" t="n">
+        <f aca="false">H13+F13+B13+D13+K13+O13</f>
+        <v>1623.3</v>
       </c>
       <c r="V13" s="1" t="n">
-        <f aca="false">U13-$V$34*T13/100</f>
-        <v>771.7</v>
+        <f aca="false">U13-$T$42*1000*T13/100</f>
+        <v>714.4785</v>
       </c>
       <c r="W13" s="1" t="n">
         <f aca="false">ROUND(V13/S13 *100/1000, 2)</f>
-        <v>0.3</v>
+        <v>0.28</v>
       </c>
       <c r="Y13" s="1" t="n">
         <f aca="false">T13*50000/100</f>
@@ -3523,7 +3587,7 @@
         <v>281.7</v>
       </c>
       <c r="AG13" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="AH13" s="1" t="n">
         <v>0</v>
@@ -3541,34 +3605,34 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="15" t="s">
-        <v>50</v>
-      </c>
-      <c r="B14" s="16" t="n">
+      <c r="A14" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="B14" s="18" t="n">
         <v>1078</v>
       </c>
-      <c r="C14" s="12" t="n">
+      <c r="C14" s="14" t="n">
         <f aca="false">1000*B14/$S14</f>
         <v>418.692157950257</v>
       </c>
-      <c r="D14" s="17" t="n">
+      <c r="D14" s="19" t="n">
         <v>1691</v>
       </c>
-      <c r="E14" s="12" t="n">
+      <c r="E14" s="14" t="n">
         <f aca="false">1000*D14/$S14</f>
         <v>656.779628101934</v>
       </c>
-      <c r="F14" s="16" t="n">
+      <c r="F14" s="18" t="n">
         <v>3100</v>
       </c>
-      <c r="G14" s="12" t="n">
+      <c r="G14" s="14" t="n">
         <f aca="false">1000*F14/$S14</f>
         <v>1204.03125199054</v>
       </c>
-      <c r="H14" s="16" t="n">
+      <c r="H14" s="18" t="n">
         <v>6670</v>
       </c>
-      <c r="I14" s="12" t="n">
+      <c r="I14" s="14" t="n">
         <f aca="false">1000*H14/$S14</f>
         <v>2590.60917766996</v>
       </c>
@@ -3578,7 +3642,7 @@
       <c r="K14" s="1" t="n">
         <v>5380</v>
       </c>
-      <c r="L14" s="12" t="n">
+      <c r="L14" s="14" t="n">
         <f aca="false">1000*K14/$S14</f>
         <v>2089.57681797067</v>
       </c>
@@ -3592,7 +3656,7 @@
         <f aca="false">N14*N$34/100*1000</f>
         <v>9108</v>
       </c>
-      <c r="P14" s="12" t="n">
+      <c r="P14" s="14" t="n">
         <f aca="false">1000*O14/$S14</f>
         <v>3537.5214977838</v>
       </c>
@@ -3608,17 +3672,17 @@
       <c r="T14" s="1" t="n">
         <v>15.91</v>
       </c>
-      <c r="U14" s="1" t="n">
-        <f aca="false">H14+F14+B14+0.8*D14+K14+O14</f>
-        <v>26688.8</v>
+      <c r="U14" s="2" t="n">
+        <f aca="false">H14+F14+B14+D14+K14+O14</f>
+        <v>27027</v>
       </c>
       <c r="V14" s="1" t="n">
-        <f aca="false">U14-$V$34*T14/100</f>
-        <v>17938.3</v>
+        <f aca="false">U14-$T$42*1000*T14/100</f>
+        <v>17387.43329</v>
       </c>
       <c r="W14" s="1" t="n">
         <f aca="false">ROUND(V14/S14 *100/1000, 2)</f>
-        <v>0.7</v>
+        <v>0.68</v>
       </c>
       <c r="Y14" s="1" t="n">
         <f aca="false">T14*50000/100</f>
@@ -3628,7 +3692,7 @@
         <v>2991.1</v>
       </c>
       <c r="AG14" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="AH14" s="1" t="n">
         <v>5</v>
@@ -3646,34 +3710,34 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="B15" s="12" t="n">
+      <c r="A15" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="B15" s="14" t="n">
         <v>973</v>
       </c>
-      <c r="C15" s="12" t="n">
+      <c r="C15" s="14" t="n">
         <f aca="false">1000*B15/$S15</f>
         <v>260.893020991029</v>
       </c>
-      <c r="D15" s="20" t="n">
+      <c r="D15" s="22" t="n">
         <v>2700</v>
       </c>
-      <c r="E15" s="12" t="n">
+      <c r="E15" s="14" t="n">
         <f aca="false">1000*D15/$S15</f>
         <v>723.958023305013</v>
       </c>
-      <c r="F15" s="14" t="n">
+      <c r="F15" s="16" t="n">
         <v>1595.2</v>
       </c>
-      <c r="G15" s="12" t="n">
+      <c r="G15" s="14" t="n">
         <f aca="false">1000*F15/$S15</f>
         <v>427.725125472651</v>
       </c>
-      <c r="H15" s="12" t="n">
+      <c r="H15" s="14" t="n">
         <v>8344</v>
       </c>
-      <c r="I15" s="12" t="n">
+      <c r="I15" s="14" t="n">
         <f aca="false">1000*H15/$S15</f>
         <v>2237.29842461372</v>
       </c>
@@ -3683,7 +3747,7 @@
       <c r="K15" s="1" t="n">
         <v>6400</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="L15" s="14" t="n">
         <f aca="false">1000*K15/$S15</f>
         <v>1716.04864783411</v>
       </c>
@@ -3697,7 +3761,7 @@
         <f aca="false">N15*N$34/100*1000</f>
         <v>8492</v>
       </c>
-      <c r="P15" s="12" t="n">
+      <c r="P15" s="14" t="n">
         <f aca="false">1000*O15/$S15</f>
         <v>2276.98204959488</v>
       </c>
@@ -3713,17 +3777,17 @@
       <c r="T15" s="1" t="n">
         <v>24.1</v>
       </c>
-      <c r="U15" s="1" t="n">
-        <f aca="false">H15+F15+B15+0.8*D15+K15+O15</f>
-        <v>27964.2</v>
+      <c r="U15" s="2" t="n">
+        <f aca="false">H15+F15+B15+D15+K15+O15</f>
+        <v>28504.2</v>
       </c>
       <c r="V15" s="1" t="n">
-        <f aca="false">U15-$V$34*T15/100</f>
-        <v>14709.2</v>
+        <f aca="false">U15-$T$42*1000*T15/100</f>
+        <v>13902.4679</v>
       </c>
       <c r="W15" s="1" t="n">
         <f aca="false">ROUND(V15/S15 *100/1000, 2)</f>
-        <v>0.39</v>
+        <v>0.37</v>
       </c>
       <c r="Y15" s="1" t="n">
         <f aca="false">T15*50000/100</f>
@@ -3733,7 +3797,7 @@
         <v>4529.7</v>
       </c>
       <c r="AG15" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="AH15" s="1" t="n">
         <v>6</v>
@@ -3751,34 +3815,34 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="15" t="s">
-        <v>54</v>
-      </c>
-      <c r="B16" s="16" t="n">
+      <c r="A16" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="B16" s="18" t="n">
         <v>91</v>
       </c>
-      <c r="C16" s="12" t="n">
+      <c r="C16" s="14" t="n">
         <f aca="false">1000*B16/$S16</f>
         <v>503.093193867792</v>
       </c>
-      <c r="D16" s="17" t="n">
+      <c r="D16" s="19" t="n">
         <v>54</v>
       </c>
-      <c r="E16" s="12" t="n">
+      <c r="E16" s="14" t="n">
         <f aca="false">1000*D16/$S16</f>
         <v>298.538818339129</v>
       </c>
-      <c r="F16" s="18" t="n">
+      <c r="F16" s="20" t="n">
         <v>22.7</v>
       </c>
-      <c r="G16" s="12" t="n">
+      <c r="G16" s="14" t="n">
         <f aca="false">1000*F16/$S16</f>
         <v>125.496873635152</v>
       </c>
-      <c r="H16" s="16" t="n">
+      <c r="H16" s="18" t="n">
         <v>118</v>
       </c>
-      <c r="I16" s="12" t="n">
+      <c r="I16" s="14" t="n">
         <f aca="false">1000*H16/$S16</f>
         <v>652.362603037356</v>
       </c>
@@ -3788,7 +3852,7 @@
       <c r="K16" s="1" t="n">
         <v>2540</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="L16" s="14" t="n">
         <f aca="false">1000*K16/$S16</f>
         <v>14042.3814552109</v>
       </c>
@@ -3802,7 +3866,7 @@
         <f aca="false">N16*N$34/100*1000</f>
         <v>924</v>
       </c>
-      <c r="P16" s="12" t="n">
+      <c r="P16" s="14" t="n">
         <f aca="false">1000*O16/$S16</f>
         <v>5108.33089158065</v>
       </c>
@@ -3818,17 +3882,17 @@
       <c r="T16" s="1" t="n">
         <v>1.32</v>
       </c>
-      <c r="U16" s="1" t="n">
-        <f aca="false">H16+F16+B16+0.8*D16+K16+O16</f>
-        <v>3738.9</v>
+      <c r="U16" s="2" t="n">
+        <f aca="false">H16+F16+B16+D16+K16+O16</f>
+        <v>3749.7</v>
       </c>
       <c r="V16" s="1" t="n">
-        <f aca="false">U16-$V$34*T16/100</f>
-        <v>3012.9</v>
+        <f aca="false">U16-$T$42*1000*T16/100</f>
+        <v>2949.93708</v>
       </c>
       <c r="W16" s="1" t="n">
         <f aca="false">ROUND(V16/S16 *100/1000, 2)</f>
-        <v>1.67</v>
+        <v>1.63</v>
       </c>
       <c r="Y16" s="1" t="n">
         <f aca="false">T16*50000/100</f>
@@ -3838,7 +3902,7 @@
         <v>248.4</v>
       </c>
       <c r="AG16" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="AH16" s="1" t="n">
         <v>2</v>
@@ -3856,34 +3920,34 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11" t="s">
-        <v>56</v>
-      </c>
-      <c r="B17" s="12" t="n">
+      <c r="A17" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="B17" s="14" t="n">
         <v>139</v>
       </c>
-      <c r="C17" s="12" t="n">
+      <c r="C17" s="14" t="n">
         <f aca="false">1000*B17/$S17</f>
         <v>933.361983293492</v>
       </c>
-      <c r="D17" s="13" t="n">
+      <c r="D17" s="15" t="n">
         <v>113</v>
       </c>
-      <c r="E17" s="12" t="n">
+      <c r="E17" s="14" t="n">
         <f aca="false">1000*D17/$S17</f>
         <v>758.776288576724</v>
       </c>
-      <c r="F17" s="14" t="n">
+      <c r="F17" s="16" t="n">
         <v>5.9</v>
       </c>
-      <c r="G17" s="12" t="n">
+      <c r="G17" s="14" t="n">
         <f aca="false">1000*F17/$S17</f>
         <v>39.617523031882</v>
       </c>
-      <c r="H17" s="12" t="n">
+      <c r="H17" s="14" t="n">
         <v>208</v>
       </c>
-      <c r="I17" s="12" t="n">
+      <c r="I17" s="14" t="n">
         <f aca="false">1000*H17/$S17</f>
         <v>1396.68555773415</v>
       </c>
@@ -3893,7 +3957,7 @@
       <c r="K17" s="1" t="n">
         <v>370</v>
       </c>
-      <c r="L17" s="12" t="n">
+      <c r="L17" s="14" t="n">
         <f aca="false">1000*K17/$S17</f>
         <v>2484.48873250786</v>
       </c>
@@ -3907,7 +3971,7 @@
         <f aca="false">N17*N$34/100*1000</f>
         <v>396</v>
       </c>
-      <c r="P17" s="12" t="n">
+      <c r="P17" s="14" t="n">
         <f aca="false">1000*O17/$S17</f>
         <v>2659.07442722462</v>
       </c>
@@ -3923,17 +3987,17 @@
       <c r="T17" s="1" t="n">
         <v>1.16</v>
       </c>
-      <c r="U17" s="1" t="n">
-        <f aca="false">H17+F17+B17+0.8*D17+K17+O17</f>
-        <v>1209.3</v>
+      <c r="U17" s="2" t="n">
+        <f aca="false">H17+F17+B17+D17+K17+O17</f>
+        <v>1231.9</v>
       </c>
       <c r="V17" s="1" t="n">
-        <f aca="false">U17-$V$34*T17/100</f>
-        <v>571.3</v>
+        <f aca="false">U17-$T$42*1000*T17/100</f>
+        <v>529.07804</v>
       </c>
       <c r="W17" s="1" t="n">
         <f aca="false">ROUND(V17/S17 *100/1000, 2)</f>
-        <v>0.38</v>
+        <v>0.36</v>
       </c>
       <c r="Y17" s="1" t="n">
         <f aca="false">T17*50000/100</f>
@@ -3943,7 +4007,7 @@
         <v>218.8</v>
       </c>
       <c r="AG17" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="AH17" s="1" t="n">
         <v>0</v>
@@ -3961,34 +4025,34 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="15" t="s">
-        <v>58</v>
-      </c>
-      <c r="B18" s="16" t="n">
+      <c r="A18" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="B18" s="18" t="n">
         <v>97</v>
       </c>
-      <c r="C18" s="12" t="n">
+      <c r="C18" s="14" t="n">
         <f aca="false">1000*B18/$S18</f>
         <v>299.863052234907</v>
       </c>
-      <c r="D18" s="17" t="n">
+      <c r="D18" s="19" t="n">
         <v>160</v>
       </c>
-      <c r="E18" s="12" t="n">
+      <c r="E18" s="14" t="n">
         <f aca="false">1000*D18/$S18</f>
         <v>494.619467603971</v>
       </c>
-      <c r="F18" s="18" t="n">
+      <c r="F18" s="20" t="n">
         <v>241.4</v>
       </c>
-      <c r="G18" s="12" t="n">
+      <c r="G18" s="14" t="n">
         <f aca="false">1000*F18/$S18</f>
         <v>746.257121747491</v>
       </c>
-      <c r="H18" s="16" t="n">
+      <c r="H18" s="18" t="n">
         <v>331</v>
       </c>
-      <c r="I18" s="12" t="n">
+      <c r="I18" s="14" t="n">
         <f aca="false">1000*H18/$S18</f>
         <v>1023.24402360571</v>
       </c>
@@ -3998,7 +4062,7 @@
       <c r="K18" s="1" t="n">
         <v>940</v>
       </c>
-      <c r="L18" s="12" t="n">
+      <c r="L18" s="14" t="n">
         <f aca="false">1000*K18/$S18</f>
         <v>2905.88937217333</v>
       </c>
@@ -4012,7 +4076,7 @@
         <f aca="false">N18*N$34/100*1000</f>
         <v>572</v>
       </c>
-      <c r="P18" s="12" t="n">
+      <c r="P18" s="14" t="n">
         <f aca="false">1000*O18/$S18</f>
         <v>1768.2645966842</v>
       </c>
@@ -4028,17 +4092,17 @@
       <c r="T18" s="1" t="n">
         <v>3.21</v>
       </c>
-      <c r="U18" s="1" t="n">
-        <f aca="false">H18+F18+B18+0.8*D18+K18+O18</f>
-        <v>2309.4</v>
+      <c r="U18" s="2" t="n">
+        <f aca="false">H18+F18+B18+D18+K18+O18</f>
+        <v>2341.4</v>
       </c>
       <c r="V18" s="1" t="n">
-        <f aca="false">U18-$V$34*T18/100</f>
-        <v>543.9</v>
+        <f aca="false">U18-$T$42*1000*T18/100</f>
+        <v>396.52199</v>
       </c>
       <c r="W18" s="1" t="n">
         <f aca="false">ROUND(V18/S18 *100/1000, 2)</f>
-        <v>0.17</v>
+        <v>0.12</v>
       </c>
       <c r="Y18" s="1" t="n">
         <f aca="false">T18*50000/100</f>
@@ -4048,7 +4112,7 @@
         <v>602.4</v>
       </c>
       <c r="AG18" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="AH18" s="1" t="n">
         <v>0</v>
@@ -4066,34 +4130,34 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11" t="s">
-        <v>60</v>
-      </c>
-      <c r="B19" s="12" t="n">
+      <c r="A19" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="B19" s="14" t="n">
         <v>464</v>
       </c>
-      <c r="C19" s="12" t="n">
+      <c r="C19" s="14" t="n">
         <f aca="false">1000*B19/$S19</f>
         <v>255.791133309077</v>
       </c>
-      <c r="D19" s="13" t="n">
+      <c r="D19" s="15" t="n">
         <v>891</v>
       </c>
-      <c r="E19" s="12" t="n">
+      <c r="E19" s="14" t="n">
         <f aca="false">1000*D19/$S19</f>
         <v>491.185128832732</v>
       </c>
-      <c r="F19" s="14" t="n">
+      <c r="F19" s="16" t="n">
         <v>544.5</v>
       </c>
-      <c r="G19" s="12" t="n">
+      <c r="G19" s="14" t="n">
         <f aca="false">1000*F19/$S19</f>
         <v>300.168689842225</v>
       </c>
-      <c r="H19" s="12" t="n">
+      <c r="H19" s="14" t="n">
         <v>2618</v>
       </c>
-      <c r="I19" s="12" t="n">
+      <c r="I19" s="14" t="n">
         <f aca="false">1000*H19/$S19</f>
         <v>1443.23531681716</v>
       </c>
@@ -4103,7 +4167,7 @@
       <c r="K19" s="1" t="n">
         <v>7110</v>
       </c>
-      <c r="L19" s="12" t="n">
+      <c r="L19" s="14" t="n">
         <f aca="false">1000*K19/$S19</f>
         <v>3919.55809876625</v>
       </c>
@@ -4117,7 +4181,7 @@
         <f aca="false">N19*N$34/100*1000</f>
         <v>8316</v>
       </c>
-      <c r="P19" s="12" t="n">
+      <c r="P19" s="14" t="n">
         <f aca="false">1000*O19/$S19</f>
         <v>4584.39453577217</v>
       </c>
@@ -4133,17 +4197,17 @@
       <c r="T19" s="1" t="n">
         <v>12.01</v>
       </c>
-      <c r="U19" s="1" t="n">
-        <f aca="false">H19+F19+B19+0.8*D19+K19+O19</f>
-        <v>19765.3</v>
+      <c r="U19" s="2" t="n">
+        <f aca="false">H19+F19+B19+D19+K19+O19</f>
+        <v>19943.5</v>
       </c>
       <c r="V19" s="1" t="n">
-        <f aca="false">U19-$V$34*T19/100</f>
-        <v>13159.8</v>
+        <f aca="false">U19-$T$42*1000*T19/100</f>
+        <v>12666.86919</v>
       </c>
       <c r="W19" s="1" t="n">
         <f aca="false">ROUND(V19/S19 *100/1000, 2)</f>
-        <v>0.73</v>
+        <v>0.7</v>
       </c>
       <c r="Y19" s="1" t="n">
         <f aca="false">T19*50000/100</f>
@@ -4153,7 +4217,7 @@
         <v>2258</v>
       </c>
       <c r="AG19" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="AH19" s="1" t="n">
         <v>7</v>
@@ -4171,34 +4235,34 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="15" t="s">
-        <v>62</v>
-      </c>
-      <c r="B20" s="16" t="n">
+      <c r="A20" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="B20" s="18" t="n">
         <v>27</v>
       </c>
-      <c r="C20" s="12" t="n">
+      <c r="C20" s="14" t="n">
         <f aca="false">1000*B20/$S20</f>
         <v>816.326530612245</v>
       </c>
-      <c r="D20" s="17" t="n">
+      <c r="D20" s="19" t="n">
         <v>20</v>
       </c>
-      <c r="E20" s="12" t="n">
+      <c r="E20" s="14" t="n">
         <f aca="false">1000*D20/$S20</f>
         <v>604.686318972033</v>
       </c>
-      <c r="F20" s="16" t="n">
+      <c r="F20" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="G20" s="12" t="n">
+      <c r="G20" s="14" t="n">
         <f aca="false">1000*F20/$S20</f>
         <v>0</v>
       </c>
-      <c r="H20" s="16" t="n">
+      <c r="H20" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="I20" s="12" t="n">
+      <c r="I20" s="14" t="n">
         <f aca="false">1000*H20/$S20</f>
         <v>604.686318972033</v>
       </c>
@@ -4208,7 +4272,7 @@
       <c r="K20" s="1" t="n">
         <v>180</v>
       </c>
-      <c r="L20" s="12" t="n">
+      <c r="L20" s="14" t="n">
         <f aca="false">1000*K20/$S20</f>
         <v>5442.1768707483</v>
       </c>
@@ -4222,7 +4286,7 @@
         <f aca="false">N20*N$34/100*1000</f>
         <v>88</v>
       </c>
-      <c r="P20" s="12" t="n">
+      <c r="P20" s="14" t="n">
         <f aca="false">1000*O20/$S20</f>
         <v>2660.61980347695</v>
       </c>
@@ -4238,17 +4302,17 @@
       <c r="T20" s="1" t="n">
         <v>0.23</v>
       </c>
-      <c r="U20" s="1" t="n">
-        <f aca="false">H20+F20+B20+0.8*D20+K20+O20</f>
-        <v>331</v>
+      <c r="U20" s="2" t="n">
+        <f aca="false">H20+F20+B20+D20+K20+O20</f>
+        <v>335</v>
       </c>
       <c r="V20" s="1" t="n">
-        <f aca="false">U20-$V$34*T20/100</f>
-        <v>204.5</v>
+        <f aca="false">U20-$T$42*1000*T20/100</f>
+        <v>195.64737</v>
       </c>
       <c r="W20" s="1" t="n">
         <f aca="false">ROUND(V20/S20 *100/1000, 2)</f>
-        <v>0.62</v>
+        <v>0.59</v>
       </c>
       <c r="Y20" s="1" t="n">
         <f aca="false">T20*50000/100</f>
@@ -4258,7 +4322,7 @@
         <v>43</v>
       </c>
       <c r="AG20" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="AH20" s="1" t="n">
         <v>0</v>
@@ -4276,34 +4340,34 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="B21" s="12" t="n">
+      <c r="A21" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="B21" s="14" t="n">
         <v>41</v>
       </c>
-      <c r="C21" s="12" t="n">
+      <c r="C21" s="14" t="n">
         <f aca="false">1000*B21/$S21</f>
         <v>759.034360189574</v>
       </c>
-      <c r="D21" s="13" t="n">
+      <c r="D21" s="15" t="n">
         <v>24</v>
       </c>
-      <c r="E21" s="12" t="n">
+      <c r="E21" s="14" t="n">
         <f aca="false">1000*D21/$S21</f>
         <v>444.312796208531</v>
       </c>
-      <c r="F21" s="14" t="n">
+      <c r="F21" s="16" t="n">
         <v>0.1</v>
       </c>
-      <c r="G21" s="12" t="n">
+      <c r="G21" s="14" t="n">
         <f aca="false">1000*F21/$S21</f>
         <v>1.85130331753555</v>
       </c>
-      <c r="H21" s="12" t="n">
+      <c r="H21" s="14" t="n">
         <v>31</v>
       </c>
-      <c r="I21" s="12" t="n">
+      <c r="I21" s="14" t="n">
         <f aca="false">1000*H21/$S21</f>
         <v>573.904028436019</v>
       </c>
@@ -4313,7 +4377,7 @@
       <c r="K21" s="1" t="n">
         <v>140</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="L21" s="14" t="n">
         <f aca="false">1000*K21/$S21</f>
         <v>2591.82464454976</v>
       </c>
@@ -4327,7 +4391,7 @@
         <f aca="false">N21*N$34/100*1000</f>
         <v>132</v>
       </c>
-      <c r="P21" s="12" t="n">
+      <c r="P21" s="14" t="n">
         <f aca="false">1000*O21/$S21</f>
         <v>2443.72037914692</v>
       </c>
@@ -4343,17 +4407,17 @@
       <c r="T21" s="1" t="n">
         <v>0.45</v>
       </c>
-      <c r="U21" s="1" t="n">
-        <f aca="false">H21+F21+B21+0.8*D21+K21+O21</f>
-        <v>363.3</v>
+      <c r="U21" s="2" t="n">
+        <f aca="false">H21+F21+B21+D21+K21+O21</f>
+        <v>368.1</v>
       </c>
       <c r="V21" s="1" t="n">
-        <f aca="false">U21-$V$34*T21/100</f>
-        <v>115.8</v>
+        <f aca="false">U21-$T$42*1000*T21/100</f>
+        <v>95.45355</v>
       </c>
       <c r="W21" s="1" t="n">
         <f aca="false">ROUND(V21/S21 *100/1000, 2)</f>
-        <v>0.21</v>
+        <v>0.18</v>
       </c>
       <c r="Y21" s="1" t="n">
         <f aca="false">T21*50000/100</f>
@@ -4363,7 +4427,7 @@
         <v>84.3</v>
       </c>
       <c r="AG21" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="AH21" s="1" t="n">
         <v>0</v>
@@ -4381,32 +4445,32 @@
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="15" t="s">
-        <v>66</v>
-      </c>
-      <c r="B22" s="16" t="n">
+      <c r="A22" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="B22" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="C22" s="12" t="n">
+      <c r="C22" s="14" t="n">
         <f aca="false">1000*B22/$S22</f>
         <v>198.137507430157</v>
       </c>
-      <c r="D22" s="21"/>
-      <c r="E22" s="12" t="n">
+      <c r="D22" s="23"/>
+      <c r="E22" s="14" t="n">
         <f aca="false">1000*D22/$S22</f>
         <v>0</v>
       </c>
-      <c r="F22" s="16" t="n">
+      <c r="F22" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="G22" s="12" t="n">
+      <c r="G22" s="14" t="n">
         <f aca="false">1000*F22/$S22</f>
         <v>0</v>
       </c>
-      <c r="H22" s="16" t="n">
+      <c r="H22" s="18" t="n">
         <v>208</v>
       </c>
-      <c r="I22" s="12" t="n">
+      <c r="I22" s="14" t="n">
         <f aca="false">1000*H22/$S22</f>
         <v>4121.26015454726</v>
       </c>
@@ -4416,7 +4480,7 @@
       <c r="K22" s="1" t="n">
         <v>210</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="L22" s="14" t="n">
         <f aca="false">1000*K22/$S22</f>
         <v>4160.88765603329</v>
       </c>
@@ -4430,7 +4494,7 @@
         <f aca="false">N22*N$34/100*1000</f>
         <v>264</v>
       </c>
-      <c r="P22" s="12" t="n">
+      <c r="P22" s="14" t="n">
         <f aca="false">1000*O22/$S22</f>
         <v>5230.83019615613</v>
       </c>
@@ -4446,17 +4510,17 @@
       <c r="T22" s="1" t="n">
         <v>0.48</v>
       </c>
-      <c r="U22" s="1" t="n">
-        <f aca="false">H22+F22+B22+0.8*D22+K22+O22</f>
+      <c r="U22" s="2" t="n">
+        <f aca="false">H22+F22+B22+D22+K22+O22</f>
         <v>692</v>
       </c>
       <c r="V22" s="1" t="n">
-        <f aca="false">U22-$V$34*T22/100</f>
-        <v>428</v>
+        <f aca="false">U22-$T$42*1000*T22/100</f>
+        <v>401.17712</v>
       </c>
       <c r="W22" s="1" t="n">
         <f aca="false">ROUND(V22/S22 *100/1000, 2)</f>
-        <v>0.85</v>
+        <v>0.79</v>
       </c>
       <c r="Y22" s="1" t="n">
         <f aca="false">T22*50000/100</f>
@@ -4466,7 +4530,7 @@
         <v>89.5</v>
       </c>
       <c r="AG22" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="AH22" s="1" t="n">
         <v>0</v>
@@ -4484,32 +4548,32 @@
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="B23" s="12" t="n">
+      <c r="A23" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="B23" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="C23" s="12" t="n">
+      <c r="C23" s="14" t="n">
         <f aca="false">1000*B23/$S23</f>
         <v>510.538983298082</v>
       </c>
-      <c r="D23" s="19"/>
-      <c r="E23" s="12" t="n">
+      <c r="D23" s="21"/>
+      <c r="E23" s="14" t="n">
         <f aca="false">1000*D23/$S23</f>
         <v>0</v>
       </c>
-      <c r="F23" s="12" t="n">
+      <c r="F23" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="G23" s="12" t="n">
+      <c r="G23" s="14" t="n">
         <f aca="false">1000*F23/$S23</f>
         <v>0</v>
       </c>
-      <c r="H23" s="12" t="n">
+      <c r="H23" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="I23" s="12" t="n">
+      <c r="I23" s="14" t="n">
         <f aca="false">1000*H23/$S23</f>
         <v>656.407264240391</v>
       </c>
@@ -4519,7 +4583,7 @@
       <c r="K23" s="1" t="n">
         <v>270</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="L23" s="14" t="n">
         <f aca="false">1000*K23/$S23</f>
         <v>19692.2179272117</v>
       </c>
@@ -4533,7 +4597,7 @@
         <f aca="false">N23*N$34/100*1000</f>
         <v>132</v>
       </c>
-      <c r="P23" s="12" t="n">
+      <c r="P23" s="14" t="n">
         <f aca="false">1000*O23/$S23</f>
         <v>9627.3065421924</v>
       </c>
@@ -4549,17 +4613,17 @@
       <c r="T23" s="1" t="n">
         <v>0.13</v>
       </c>
-      <c r="U23" s="1" t="n">
-        <f aca="false">H23+F23+B23+0.8*D23+K23+O23</f>
+      <c r="U23" s="2" t="n">
+        <f aca="false">H23+F23+B23+D23+K23+O23</f>
         <v>418</v>
       </c>
       <c r="V23" s="1" t="n">
-        <f aca="false">U23-$V$34*T23/100</f>
-        <v>346.5</v>
+        <f aca="false">U23-$T$42*1000*T23/100</f>
+        <v>339.23547</v>
       </c>
       <c r="W23" s="1" t="n">
         <f aca="false">ROUND(V23/S23 *100/1000, 2)</f>
-        <v>2.53</v>
+        <v>2.47</v>
       </c>
       <c r="Y23" s="1" t="n">
         <f aca="false">T23*50000/100</f>
@@ -4569,7 +4633,7 @@
         <v>24.6</v>
       </c>
       <c r="AG23" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="AH23" s="1" t="n">
         <v>0</v>
@@ -4587,34 +4651,34 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="15" t="s">
-        <v>70</v>
-      </c>
-      <c r="B24" s="16" t="n">
+      <c r="A24" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="B24" s="18" t="n">
         <v>332</v>
       </c>
-      <c r="C24" s="12" t="n">
+      <c r="C24" s="14" t="n">
         <f aca="false">1000*B24/$S24</f>
         <v>396.580804533444</v>
       </c>
-      <c r="D24" s="17" t="n">
+      <c r="D24" s="19" t="n">
         <v>652</v>
       </c>
-      <c r="E24" s="12" t="n">
+      <c r="E24" s="14" t="n">
         <f aca="false">1000*D24/$S24</f>
         <v>778.827363119896</v>
       </c>
-      <c r="F24" s="16" t="n">
+      <c r="F24" s="18" t="n">
         <v>1961</v>
       </c>
-      <c r="G24" s="12" t="n">
+      <c r="G24" s="14" t="n">
         <f aca="false">1000*F24/$S24</f>
         <v>2342.4546918376</v>
       </c>
-      <c r="H24" s="16" t="n">
+      <c r="H24" s="18" t="n">
         <v>913</v>
       </c>
-      <c r="I24" s="12" t="n">
+      <c r="I24" s="14" t="n">
         <f aca="false">1000*H24/$S24</f>
         <v>1090.59721246697</v>
       </c>
@@ -4624,7 +4688,7 @@
       <c r="K24" s="1" t="n">
         <v>1980</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="L24" s="14" t="n">
         <f aca="false">1000*K24/$S24</f>
         <v>2365.15058125367</v>
       </c>
@@ -4638,7 +4702,7 @@
         <f aca="false">N24*N$34/100*1000</f>
         <v>1628</v>
       </c>
-      <c r="P24" s="12" t="n">
+      <c r="P24" s="14" t="n">
         <f aca="false">1000*O24/$S24</f>
         <v>1944.67936680858</v>
       </c>
@@ -4654,17 +4718,17 @@
       <c r="T24" s="1" t="n">
         <v>6.23</v>
       </c>
-      <c r="U24" s="1" t="n">
-        <f aca="false">H24+F24+B24+0.8*D24+K24+O24</f>
-        <v>7335.6</v>
+      <c r="U24" s="2" t="n">
+        <f aca="false">H24+F24+B24+D24+K24+O24</f>
+        <v>7466</v>
       </c>
       <c r="V24" s="1" t="n">
-        <f aca="false">U24-$V$34*T24/100</f>
-        <v>3909.1</v>
+        <f aca="false">U24-$T$42*1000*T24/100</f>
+        <v>3691.36137</v>
       </c>
       <c r="W24" s="1" t="n">
         <f aca="false">ROUND(V24/S24 *100/1000, 2)</f>
-        <v>0.47</v>
+        <v>0.44</v>
       </c>
       <c r="Y24" s="1" t="n">
         <f aca="false">T24*50000/100</f>
@@ -4674,7 +4738,7 @@
         <v>1170.6</v>
       </c>
       <c r="AG24" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="AH24" s="1" t="n">
         <v>1</v>
@@ -4692,34 +4756,34 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="B25" s="12" t="n">
+      <c r="A25" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="B25" s="14" t="n">
         <v>494</v>
       </c>
-      <c r="C25" s="12" t="n">
+      <c r="C25" s="14" t="n">
         <f aca="false">1000*B25/$S25</f>
         <v>901.606282772202</v>
       </c>
-      <c r="D25" s="13" t="n">
+      <c r="D25" s="15" t="n">
         <v>427</v>
       </c>
-      <c r="E25" s="12" t="n">
+      <c r="E25" s="14" t="n">
         <f aca="false">1000*D25/$S25</f>
         <v>779.323649278806</v>
       </c>
-      <c r="F25" s="12" t="n">
+      <c r="F25" s="14" t="n">
         <v>63</v>
       </c>
-      <c r="G25" s="12" t="n">
+      <c r="G25" s="14" t="n">
         <f aca="false">1000*F25/$S25</f>
         <v>114.982177762447</v>
       </c>
-      <c r="H25" s="12" t="n">
+      <c r="H25" s="14" t="n">
         <v>560</v>
       </c>
-      <c r="I25" s="12" t="n">
+      <c r="I25" s="14" t="n">
         <f aca="false">1000*H25/$S25</f>
         <v>1022.06380233286</v>
       </c>
@@ -4729,7 +4793,7 @@
       <c r="K25" s="1" t="n">
         <v>1190</v>
       </c>
-      <c r="L25" s="12" t="n">
+      <c r="L25" s="14" t="n">
         <f aca="false">1000*K25/$S25</f>
         <v>2171.88557995733</v>
       </c>
@@ -4743,7 +4807,7 @@
         <f aca="false">N25*N$34/100*1000</f>
         <v>1188</v>
       </c>
-      <c r="P25" s="12" t="n">
+      <c r="P25" s="14" t="n">
         <f aca="false">1000*O25/$S25</f>
         <v>2168.23535209186</v>
       </c>
@@ -4759,17 +4823,17 @@
       <c r="T25" s="1" t="n">
         <v>4.91</v>
       </c>
-      <c r="U25" s="1" t="n">
-        <f aca="false">H25+F25+B25+0.8*D25+K25+O25</f>
-        <v>3836.6</v>
+      <c r="U25" s="2" t="n">
+        <f aca="false">H25+F25+B25+D25+K25+O25</f>
+        <v>3922</v>
       </c>
       <c r="V25" s="1" t="n">
-        <f aca="false">U25-$V$34*T25/100</f>
-        <v>1136.1</v>
+        <f aca="false">U25-$T$42*1000*T25/100</f>
+        <v>947.12429</v>
       </c>
       <c r="W25" s="1" t="n">
         <f aca="false">ROUND(V25/S25 *100/1000, 2)</f>
-        <v>0.21</v>
+        <v>0.17</v>
       </c>
       <c r="Y25" s="1" t="n">
         <f aca="false">T25*50000/100</f>
@@ -4779,7 +4843,7 @@
         <v>922.9</v>
       </c>
       <c r="AG25" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="AH25" s="1" t="n">
         <v>1</v>
@@ -4797,34 +4861,34 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="15" t="s">
-        <v>74</v>
-      </c>
-      <c r="B26" s="16" t="n">
+      <c r="A26" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="B26" s="18" t="n">
         <v>136</v>
       </c>
-      <c r="C26" s="12" t="n">
+      <c r="C26" s="14" t="n">
         <f aca="false">1000*B26/$S26</f>
         <v>641.88790560472</v>
       </c>
-      <c r="D26" s="17" t="n">
+      <c r="D26" s="19" t="n">
         <v>84</v>
       </c>
-      <c r="E26" s="12" t="n">
+      <c r="E26" s="14" t="n">
         <f aca="false">1000*D26/$S26</f>
         <v>396.46017699115</v>
       </c>
-      <c r="F26" s="18" t="n">
+      <c r="F26" s="20" t="n">
         <v>24.9</v>
       </c>
-      <c r="G26" s="12" t="n">
+      <c r="G26" s="14" t="n">
         <f aca="false">1000*F26/$S26</f>
         <v>117.522123893805</v>
       </c>
-      <c r="H26" s="16" t="n">
+      <c r="H26" s="18" t="n">
         <v>330</v>
       </c>
-      <c r="I26" s="12" t="n">
+      <c r="I26" s="14" t="n">
         <f aca="false">1000*H26/$S26</f>
         <v>1557.52212389381</v>
       </c>
@@ -4834,7 +4898,7 @@
       <c r="K26" s="1" t="n">
         <v>1950</v>
       </c>
-      <c r="L26" s="12" t="n">
+      <c r="L26" s="14" t="n">
         <f aca="false">1000*K26/$S26</f>
         <v>9203.53982300885</v>
       </c>
@@ -4848,7 +4912,7 @@
         <f aca="false">N26*N$34/100*1000</f>
         <v>924</v>
       </c>
-      <c r="P26" s="12" t="n">
+      <c r="P26" s="14" t="n">
         <f aca="false">1000*O26/$S26</f>
         <v>4361.06194690266</v>
       </c>
@@ -4864,17 +4928,17 @@
       <c r="T26" s="1" t="n">
         <v>1.63</v>
       </c>
-      <c r="U26" s="1" t="n">
-        <f aca="false">H26+F26+B26+0.8*D26+K26+O26</f>
-        <v>3432.1</v>
+      <c r="U26" s="2" t="n">
+        <f aca="false">H26+F26+B26+D26+K26+O26</f>
+        <v>3448.9</v>
       </c>
       <c r="V26" s="1" t="n">
-        <f aca="false">U26-$V$34*T26/100</f>
-        <v>2535.6</v>
+        <f aca="false">U26-$T$42*1000*T26/100</f>
+        <v>2461.31397</v>
       </c>
       <c r="W26" s="1" t="n">
         <f aca="false">ROUND(V26/S26 *100/1000, 2)</f>
-        <v>1.2</v>
+        <v>1.16</v>
       </c>
       <c r="Y26" s="1" t="n">
         <f aca="false">T26*50000/100</f>
@@ -4884,7 +4948,7 @@
         <v>306.8</v>
       </c>
       <c r="AG26" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="AH26" s="1" t="n">
         <v>1</v>
@@ -4902,34 +4966,34 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="11" t="s">
-        <v>76</v>
-      </c>
-      <c r="B27" s="12" t="n">
+      <c r="A27" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="B27" s="14" t="n">
         <v>133</v>
       </c>
-      <c r="C27" s="12" t="n">
+      <c r="C27" s="14" t="n">
         <f aca="false">1000*B27/$S27</f>
         <v>617.708255926284</v>
       </c>
-      <c r="D27" s="13" t="n">
+      <c r="D27" s="15" t="n">
         <v>30</v>
       </c>
-      <c r="E27" s="12" t="n">
+      <c r="E27" s="14" t="n">
         <f aca="false">1000*D27/$S27</f>
         <v>139.332689306681</v>
       </c>
-      <c r="F27" s="14" t="n">
+      <c r="F27" s="16" t="n">
         <v>1.9</v>
       </c>
-      <c r="G27" s="12" t="n">
+      <c r="G27" s="14" t="n">
         <f aca="false">1000*F27/$S27</f>
         <v>8.82440365608977</v>
       </c>
-      <c r="H27" s="12" t="n">
+      <c r="H27" s="14" t="n">
         <v>121</v>
       </c>
-      <c r="I27" s="12" t="n">
+      <c r="I27" s="14" t="n">
         <f aca="false">1000*H27/$S27</f>
         <v>561.975180203611</v>
       </c>
@@ -4939,7 +5003,7 @@
       <c r="K27" s="1" t="n">
         <v>620</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="L27" s="14" t="n">
         <f aca="false">1000*K27/$S27</f>
         <v>2879.5422456714</v>
       </c>
@@ -4953,7 +5017,7 @@
         <f aca="false">N27*N$34/100*1000</f>
         <v>484</v>
       </c>
-      <c r="P27" s="12" t="n">
+      <c r="P27" s="14" t="n">
         <f aca="false">1000*O27/$S27</f>
         <v>2247.90072081445</v>
       </c>
@@ -4969,17 +5033,17 @@
       <c r="T27" s="1" t="n">
         <v>2.02</v>
       </c>
-      <c r="U27" s="1" t="n">
-        <f aca="false">H27+F27+B27+0.8*D27+K27+O27</f>
-        <v>1383.9</v>
+      <c r="U27" s="2" t="n">
+        <f aca="false">H27+F27+B27+D27+K27+O27</f>
+        <v>1389.9</v>
       </c>
       <c r="V27" s="1" t="n">
-        <f aca="false">U27-$V$34*T27/100</f>
-        <v>272.9</v>
+        <f aca="false">U27-$T$42*1000*T27/100</f>
+        <v>166.02038</v>
       </c>
       <c r="W27" s="1" t="n">
         <f aca="false">ROUND(V27/S27 *100/1000, 2)</f>
-        <v>0.13</v>
+        <v>0.08</v>
       </c>
       <c r="Y27" s="1" t="n">
         <f aca="false">T27*50000/100</f>
@@ -4989,7 +5053,7 @@
         <v>380.1</v>
       </c>
       <c r="AG27" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="AH27" s="1" t="n">
         <v>0</v>
@@ -5007,34 +5071,34 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="15" t="s">
-        <v>78</v>
-      </c>
-      <c r="B28" s="16" t="n">
+      <c r="A28" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="B28" s="18" t="n">
         <v>76</v>
       </c>
-      <c r="C28" s="12" t="n">
+      <c r="C28" s="14" t="n">
         <f aca="false">1000*B28/$S28</f>
         <v>781.105469793829</v>
       </c>
-      <c r="D28" s="17" t="n">
+      <c r="D28" s="19" t="n">
         <v>37</v>
       </c>
-      <c r="E28" s="12" t="n">
+      <c r="E28" s="14" t="n">
         <f aca="false">1000*D28/$S28</f>
         <v>380.275031346996</v>
       </c>
-      <c r="F28" s="16" t="n">
+      <c r="F28" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="G28" s="12" t="n">
+      <c r="G28" s="14" t="n">
         <f aca="false">1000*F28/$S28</f>
         <v>0</v>
       </c>
-      <c r="H28" s="16" t="n">
+      <c r="H28" s="18" t="n">
         <v>19</v>
       </c>
-      <c r="I28" s="12" t="n">
+      <c r="I28" s="14" t="n">
         <f aca="false">1000*H28/$S28</f>
         <v>195.276367448457</v>
       </c>
@@ -5044,7 +5108,7 @@
       <c r="K28" s="1" t="n">
         <v>400</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="L28" s="14" t="n">
         <f aca="false">1000*K28/$S28</f>
         <v>4111.08141996752</v>
       </c>
@@ -5058,7 +5122,7 @@
         <f aca="false">N28*N$34/100*1000</f>
         <v>176</v>
       </c>
-      <c r="P28" s="12" t="n">
+      <c r="P28" s="14" t="n">
         <f aca="false">1000*O28/$S28</f>
         <v>1808.87582478571</v>
       </c>
@@ -5074,17 +5138,17 @@
       <c r="T28" s="1" t="n">
         <v>0.73</v>
       </c>
-      <c r="U28" s="1" t="n">
-        <f aca="false">H28+F28+B28+0.8*D28+K28+O28</f>
-        <v>700.6</v>
+      <c r="U28" s="2" t="n">
+        <f aca="false">H28+F28+B28+D28+K28+O28</f>
+        <v>708</v>
       </c>
       <c r="V28" s="1" t="n">
-        <f aca="false">U28-$V$34*T28/100</f>
-        <v>299.1</v>
+        <f aca="false">U28-$T$42*1000*T28/100</f>
+        <v>265.70687</v>
       </c>
       <c r="W28" s="1" t="n">
         <f aca="false">ROUND(V28/S28 *100/1000, 2)</f>
-        <v>0.31</v>
+        <v>0.27</v>
       </c>
       <c r="Y28" s="1" t="n">
         <f aca="false">T28*50000/100</f>
@@ -5094,7 +5158,7 @@
         <v>136.8</v>
       </c>
       <c r="AG28" s="1" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="AH28" s="1" t="n">
         <v>0</v>
@@ -5112,34 +5176,34 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="B29" s="12" t="n">
+      <c r="A29" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="B29" s="14" t="n">
         <v>33</v>
       </c>
-      <c r="C29" s="12" t="n">
+      <c r="C29" s="14" t="n">
         <f aca="false">1000*B29/$S29</f>
         <v>641.137728041033</v>
       </c>
-      <c r="D29" s="13" t="n">
+      <c r="D29" s="15" t="n">
         <v>14</v>
       </c>
-      <c r="E29" s="12" t="n">
+      <c r="E29" s="14" t="n">
         <f aca="false">1000*D29/$S29</f>
         <v>271.997824017408</v>
       </c>
-      <c r="F29" s="14" t="n">
+      <c r="F29" s="16" t="n">
         <v>0.4</v>
       </c>
-      <c r="G29" s="12" t="n">
+      <c r="G29" s="14" t="n">
         <f aca="false">1000*F29/$S29</f>
         <v>7.77136640049737</v>
       </c>
-      <c r="H29" s="12" t="n">
+      <c r="H29" s="14" t="n">
         <v>75</v>
       </c>
-      <c r="I29" s="12" t="n">
+      <c r="I29" s="14" t="n">
         <f aca="false">1000*H29/$S29</f>
         <v>1457.13120009326</v>
       </c>
@@ -5149,7 +5213,7 @@
       <c r="K29" s="1" t="n">
         <v>300</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="L29" s="14" t="n">
         <f aca="false">1000*K29/$S29</f>
         <v>5828.52480037303</v>
       </c>
@@ -5163,7 +5227,7 @@
         <f aca="false">N29*N$34/100*1000</f>
         <v>176</v>
       </c>
-      <c r="P29" s="12" t="n">
+      <c r="P29" s="14" t="n">
         <f aca="false">1000*O29/$S29</f>
         <v>3419.40121621884</v>
       </c>
@@ -5179,17 +5243,17 @@
       <c r="T29" s="1" t="n">
         <v>0.38</v>
       </c>
-      <c r="U29" s="1" t="n">
-        <f aca="false">H29+F29+B29+0.8*D29+K29+O29</f>
-        <v>595.6</v>
+      <c r="U29" s="2" t="n">
+        <f aca="false">H29+F29+B29+D29+K29+O29</f>
+        <v>598.4</v>
       </c>
       <c r="V29" s="1" t="n">
-        <f aca="false">U29-$V$34*T29/100</f>
-        <v>386.6</v>
+        <f aca="false">U29-$T$42*1000*T29/100</f>
+        <v>368.16522</v>
       </c>
       <c r="W29" s="1" t="n">
         <f aca="false">ROUND(V29/S29 *100/1000, 2)</f>
-        <v>0.75</v>
+        <v>0.72</v>
       </c>
       <c r="Y29" s="1" t="n">
         <f aca="false">T29*50000/100</f>
@@ -5199,7 +5263,7 @@
         <v>70.5</v>
       </c>
       <c r="AG29" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="AH29" s="1" t="n">
         <v>0</v>
@@ -5217,34 +5281,34 @@
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="15" t="s">
-        <v>82</v>
-      </c>
-      <c r="B30" s="16" t="n">
+      <c r="A30" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="B30" s="18" t="n">
         <v>683</v>
       </c>
-      <c r="C30" s="12" t="n">
+      <c r="C30" s="14" t="n">
         <f aca="false">1000*B30/$S30</f>
         <v>562.985554433614</v>
       </c>
-      <c r="D30" s="17" t="n">
+      <c r="D30" s="19" t="n">
         <v>830</v>
       </c>
-      <c r="E30" s="12" t="n">
+      <c r="E30" s="14" t="n">
         <f aca="false">1000*D30/$S30</f>
         <v>684.155212562079</v>
       </c>
-      <c r="F30" s="18" t="n">
+      <c r="F30" s="20" t="n">
         <v>240.6</v>
       </c>
-      <c r="G30" s="12" t="n">
+      <c r="G30" s="14" t="n">
         <f aca="false">1000*F30/$S30</f>
         <v>198.32258330414</v>
       </c>
-      <c r="H30" s="16" t="n">
+      <c r="H30" s="18" t="n">
         <v>2151</v>
       </c>
-      <c r="I30" s="12" t="n">
+      <c r="I30" s="14" t="n">
         <f aca="false">1000*H30/$S30</f>
         <v>1773.033568941</v>
       </c>
@@ -5254,7 +5318,7 @@
       <c r="K30" s="1" t="n">
         <v>9330</v>
       </c>
-      <c r="L30" s="12" t="n">
+      <c r="L30" s="14" t="n">
         <f aca="false">1000*K30/$S30</f>
         <v>7690.56401590867</v>
       </c>
@@ -5268,7 +5332,7 @@
         <f aca="false">N30*N$34/100*1000</f>
         <v>4532</v>
       </c>
-      <c r="P30" s="12" t="n">
+      <c r="P30" s="14" t="n">
         <f aca="false">1000*O30/$S30</f>
         <v>3735.65231726668</v>
       </c>
@@ -5284,17 +5348,17 @@
       <c r="T30" s="1" t="n">
         <v>8.98</v>
       </c>
-      <c r="U30" s="1" t="n">
-        <f aca="false">H30+F30+B30+0.8*D30+K30+O30</f>
-        <v>17600.6</v>
+      <c r="U30" s="2" t="n">
+        <f aca="false">H30+F30+B30+D30+K30+O30</f>
+        <v>17766.6</v>
       </c>
       <c r="V30" s="1" t="n">
-        <f aca="false">U30-$V$34*T30/100</f>
-        <v>12661.6</v>
+        <f aca="false">U30-$T$42*1000*T30/100</f>
+        <v>12325.78862</v>
       </c>
       <c r="W30" s="1" t="n">
         <f aca="false">ROUND(V30/S30 *100/1000, 2)</f>
-        <v>1.04</v>
+        <v>1.02</v>
       </c>
       <c r="Y30" s="1" t="n">
         <f aca="false">T30*50000/100</f>
@@ -5304,7 +5368,7 @@
         <v>1687.2</v>
       </c>
       <c r="AG30" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="AH30" s="1" t="n">
         <v>9</v>
@@ -5322,34 +5386,34 @@
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="B31" s="12" t="n">
+      <c r="A31" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="B31" s="14" t="n">
         <v>189</v>
       </c>
-      <c r="C31" s="12" t="n">
+      <c r="C31" s="14" t="n">
         <f aca="false">1000*B31/$S31</f>
         <v>341.958899796996</v>
       </c>
-      <c r="D31" s="13" t="n">
+      <c r="D31" s="15" t="n">
         <v>601</v>
       </c>
-      <c r="E31" s="12" t="n">
+      <c r="E31" s="14" t="n">
         <f aca="false">1000*D31/$S31</f>
         <v>1087.39311522748</v>
       </c>
-      <c r="F31" s="14" t="n">
+      <c r="F31" s="16" t="n">
         <v>245.1</v>
       </c>
-      <c r="G31" s="12" t="n">
+      <c r="G31" s="14" t="n">
         <f aca="false">1000*F31/$S31</f>
         <v>443.460985927215</v>
       </c>
-      <c r="H31" s="12" t="n">
+      <c r="H31" s="14" t="n">
         <v>712</v>
       </c>
-      <c r="I31" s="12" t="n">
+      <c r="I31" s="14" t="n">
         <f aca="false">1000*H31/$S31</f>
         <v>1288.22611987016</v>
       </c>
@@ -5359,7 +5423,7 @@
       <c r="K31" s="1" t="n">
         <v>1160</v>
       </c>
-      <c r="L31" s="12" t="n">
+      <c r="L31" s="14" t="n">
         <f aca="false">1000*K31/$S31</f>
         <v>2098.79536383341</v>
       </c>
@@ -5373,7 +5437,7 @@
         <f aca="false">N31*N$34/100*1000</f>
         <v>1056</v>
       </c>
-      <c r="P31" s="12" t="n">
+      <c r="P31" s="14" t="n">
         <f aca="false">1000*O31/$S31</f>
         <v>1910.62750362766</v>
       </c>
@@ -5389,17 +5453,17 @@
       <c r="T31" s="1" t="n">
         <v>3.2</v>
       </c>
-      <c r="U31" s="1" t="n">
-        <f aca="false">H31+F31+B31+0.8*D31+K31+O31</f>
-        <v>3842.9</v>
+      <c r="U31" s="2" t="n">
+        <f aca="false">H31+F31+B31+D31+K31+O31</f>
+        <v>3963.1</v>
       </c>
       <c r="V31" s="1" t="n">
-        <f aca="false">U31-$V$34*T31/100</f>
-        <v>2082.9</v>
+        <f aca="false">U31-$T$42*1000*T31/100</f>
+        <v>2024.2808</v>
       </c>
       <c r="W31" s="1" t="n">
         <f aca="false">ROUND(V31/S31 *100/1000, 2)</f>
-        <v>0.38</v>
+        <v>0.37</v>
       </c>
       <c r="Y31" s="1" t="n">
         <f aca="false">T31*50000/100</f>
@@ -5409,7 +5473,7 @@
         <v>601.2</v>
       </c>
       <c r="AG31" s="1" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="AH31" s="1" t="n">
         <v>1</v>
@@ -5426,70 +5490,61 @@
         <v>1160</v>
       </c>
     </row>
-    <row r="32" s="26" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="22" t="s">
-        <v>86</v>
-      </c>
-      <c r="B32" s="23" t="n">
+    <row r="32" s="28" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="24" t="s">
+        <v>87</v>
+      </c>
+      <c r="B32" s="25" t="n">
         <v>5847</v>
       </c>
-      <c r="C32" s="23"/>
-      <c r="D32" s="24" t="n">
+      <c r="C32" s="25"/>
+      <c r="D32" s="26" t="n">
         <v>9557</v>
       </c>
-      <c r="E32" s="23"/>
-      <c r="F32" s="25" t="n">
+      <c r="E32" s="25"/>
+      <c r="F32" s="27" t="n">
         <v>8334.6</v>
       </c>
-      <c r="G32" s="25"/>
-      <c r="H32" s="23" t="n">
+      <c r="G32" s="27"/>
+      <c r="H32" s="25" t="n">
         <v>26264</v>
       </c>
-      <c r="I32" s="23"/>
-      <c r="J32" s="26" t="n">
+      <c r="I32" s="25"/>
+      <c r="K32" s="1" t="n">
+        <f aca="false">SUM(K5:K31)</f>
+        <v>47600</v>
+      </c>
+      <c r="O32" s="1" t="n">
+        <f aca="false">SUM(O5:O31)</f>
+        <v>44088</v>
+      </c>
+      <c r="Q32" s="28" t="n">
         <v>100</v>
       </c>
-      <c r="K32" s="26" t="n">
-        <f aca="false">J32*J$34*1000/100</f>
-        <v>93000</v>
-      </c>
-      <c r="M32" s="26" t="n">
-        <v>299</v>
-      </c>
-      <c r="N32" s="26" t="n">
+      <c r="S32" s="1"/>
+      <c r="T32" s="28" t="n">
         <v>100</v>
       </c>
-      <c r="O32" s="26" t="n">
-        <f aca="false">N32*N$34/100*1000</f>
-        <v>44000</v>
-      </c>
-      <c r="Q32" s="26" t="n">
-        <v>100</v>
-      </c>
-      <c r="S32" s="1"/>
-      <c r="T32" s="26" t="n">
-        <v>100</v>
-      </c>
-      <c r="U32" s="26" t="n">
-        <f aca="false">H32+F32+B32+0.8*D32+K32+O32</f>
-        <v>185091.2</v>
-      </c>
-      <c r="V32" s="26" t="n">
-        <f aca="false">U32-$V$34*T32/100</f>
-        <v>130091.2</v>
-      </c>
-      <c r="W32" s="26" t="e">
+      <c r="U32" s="2" t="n">
+        <f aca="false">H32+F32+B32+D32+K32+O32</f>
+        <v>141690.6</v>
+      </c>
+      <c r="V32" s="1" t="n">
+        <f aca="false">U32-$T$42*1000*T32/100</f>
+        <v>81102.5</v>
+      </c>
+      <c r="W32" s="28" t="e">
         <f aca="false">ROUND(V32/S32 *100/1000, 2)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="Y32" s="26" t="n">
+      <c r="Y32" s="28" t="n">
         <f aca="false">T32*50000/100</f>
         <v>50000</v>
       </c>
-      <c r="AB32" s="26" t="n">
+      <c r="AB32" s="28" t="n">
         <v>18796</v>
       </c>
-      <c r="AK32" s="26" t="n">
+      <c r="AK32" s="28" t="n">
         <f aca="false">SUM(AK5:AK31)</f>
         <v>47600</v>
       </c>
@@ -5520,170 +5575,203 @@
         <f aca="false">SUM(O5:O31)</f>
         <v>44088</v>
       </c>
-      <c r="U33" s="1" t="n">
+      <c r="U33" s="2" t="n">
         <f aca="false">SUM(U5:U31)</f>
-        <v>139782.3</v>
+        <v>141588.1</v>
       </c>
       <c r="V33" s="1" t="n">
         <f aca="false">SUM(V5:V31)</f>
-        <v>84600.8</v>
+        <v>80800.05927</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="J34" s="27" t="n">
+      <c r="J34" s="29" t="n">
         <v>93</v>
       </c>
-      <c r="N34" s="27" t="n">
+      <c r="N34" s="29" t="n">
         <v>44</v>
-      </c>
-      <c r="V34" s="1" t="n">
-        <v>55000</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="28" t="s">
-        <v>87</v>
-      </c>
-      <c r="C35" s="29" t="n">
-        <v>103453.5</v>
-      </c>
-      <c r="D35" s="29"/>
-      <c r="E35" s="29"/>
+      <c r="B35" s="30" t="s">
+        <v>88</v>
+      </c>
+      <c r="C35" s="31" t="n">
+        <f aca="false">SUM(B32:O32)</f>
+        <v>141690.6</v>
+      </c>
+      <c r="D35" s="31"/>
+      <c r="E35" s="31"/>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="28"/>
-      <c r="C36" s="29"/>
-      <c r="D36" s="29"/>
-      <c r="E36" s="29"/>
+      <c r="B36" s="30"/>
+      <c r="C36" s="31"/>
+      <c r="D36" s="31"/>
+      <c r="E36" s="31"/>
     </row>
     <row r="37" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="28"/>
-      <c r="C37" s="29"/>
-      <c r="D37" s="29"/>
-      <c r="E37" s="29"/>
-      <c r="S37" s="30" t="s">
-        <v>88</v>
-      </c>
-      <c r="T37" s="31" t="n">
+      <c r="B37" s="30"/>
+      <c r="C37" s="31"/>
+      <c r="D37" s="31"/>
+      <c r="E37" s="31"/>
+      <c r="S37" s="32" t="s">
+        <v>89</v>
+      </c>
+      <c r="T37" s="33" t="n">
         <v>192.8</v>
       </c>
-      <c r="U37" s="32"/>
-      <c r="V37" s="32"/>
+      <c r="U37" s="34"/>
+      <c r="V37" s="35"/>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="S38" s="30" t="s">
-        <v>89</v>
-      </c>
-      <c r="T38" s="30" t="n">
+      <c r="S38" s="32" t="s">
+        <v>90</v>
+      </c>
+      <c r="T38" s="32" t="n">
         <f aca="false">T37*0.7</f>
         <v>134.96</v>
       </c>
-      <c r="U38" s="32"/>
-      <c r="V38" s="32"/>
+      <c r="U38" s="34"/>
+      <c r="V38" s="35"/>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="S39" s="30"/>
-      <c r="T39" s="30"/>
-      <c r="U39" s="32"/>
-      <c r="V39" s="32"/>
+      <c r="S39" s="32"/>
+      <c r="T39" s="32"/>
+      <c r="U39" s="34"/>
+      <c r="V39" s="35"/>
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="S40" s="30" t="s">
-        <v>90</v>
-      </c>
-      <c r="T40" s="30" t="n">
-        <v>55</v>
-      </c>
-      <c r="U40" s="32"/>
-      <c r="V40" s="32"/>
+      <c r="S40" s="36" t="s">
+        <v>91</v>
+      </c>
+      <c r="T40" s="37" t="n">
+        <v>20</v>
+      </c>
+      <c r="U40" s="34"/>
+      <c r="V40" s="35"/>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="S41" s="30" t="s">
-        <v>91</v>
-      </c>
-      <c r="T41" s="30" t="n">
-        <v>19</v>
-      </c>
-      <c r="U41" s="32"/>
-      <c r="V41" s="32"/>
+      <c r="Q41" s="38" t="s">
+        <v>92</v>
+      </c>
+      <c r="S41" s="36" t="s">
+        <v>93</v>
+      </c>
+      <c r="T41" s="36" t="n">
+        <f aca="false">U33/1000 -T40</f>
+        <v>121.5881</v>
+      </c>
+      <c r="U41" s="34"/>
+      <c r="V41" s="35"/>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B42" s="32"/>
-      <c r="C42" s="32"/>
-      <c r="D42" s="32"/>
-      <c r="E42" s="32"/>
-      <c r="F42" s="32"/>
-      <c r="G42" s="32"/>
-      <c r="H42" s="32"/>
-      <c r="I42" s="32"/>
-      <c r="S42" s="30" t="s">
-        <v>92</v>
-      </c>
-      <c r="T42" s="30" t="n">
-        <f aca="false">T37+T41</f>
-        <v>211.8</v>
-      </c>
-      <c r="U42" s="32"/>
-      <c r="V42" s="32"/>
+      <c r="S42" s="36" t="s">
+        <v>94</v>
+      </c>
+      <c r="T42" s="36" t="n">
+        <f aca="false">T41-T43-T44</f>
+        <v>60.5881</v>
+      </c>
+      <c r="U42" s="34"/>
+      <c r="V42" s="35"/>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="32"/>
-      <c r="C43" s="32"/>
-      <c r="D43" s="32"/>
-      <c r="E43" s="32"/>
-      <c r="F43" s="32"/>
-      <c r="G43" s="32"/>
-      <c r="H43" s="32"/>
-      <c r="I43" s="32"/>
-      <c r="S43" s="30" t="s">
-        <v>89</v>
-      </c>
-      <c r="T43" s="30" t="n">
-        <f aca="false">T38-T40</f>
-        <v>79.96</v>
-      </c>
-      <c r="U43" s="32"/>
-      <c r="V43" s="32"/>
+      <c r="S43" s="36" t="s">
+        <v>95</v>
+      </c>
+      <c r="T43" s="37" t="n">
+        <v>35</v>
+      </c>
+      <c r="U43" s="34"/>
+      <c r="V43" s="35"/>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="32"/>
-      <c r="C44" s="32"/>
-      <c r="D44" s="32"/>
-      <c r="E44" s="32"/>
-      <c r="F44" s="32"/>
-      <c r="G44" s="32"/>
-      <c r="H44" s="32"/>
-      <c r="I44" s="32"/>
-      <c r="S44" s="30" t="s">
-        <v>93</v>
-      </c>
-      <c r="T44" s="30" t="n">
-        <f aca="false">T43/T42</f>
-        <v>0.37752596789424</v>
-      </c>
-      <c r="U44" s="32"/>
-      <c r="V44" s="32"/>
+      <c r="S44" s="36" t="s">
+        <v>96</v>
+      </c>
+      <c r="T44" s="37" t="n">
+        <v>26</v>
+      </c>
+      <c r="U44" s="34"/>
+      <c r="V44" s="35"/>
     </row>
-    <row r="47" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="33"/>
-      <c r="O47" s="1"/>
-      <c r="P47" s="1"/>
-      <c r="V47" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="Y47" s="1" t="s">
-        <v>95</v>
-      </c>
+    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B45" s="35"/>
+      <c r="C45" s="35"/>
+      <c r="D45" s="35"/>
+      <c r="E45" s="35"/>
+      <c r="F45" s="35"/>
+      <c r="G45" s="35"/>
+      <c r="H45" s="35"/>
+      <c r="I45" s="35"/>
+      <c r="S45" s="36" t="s">
+        <v>97</v>
+      </c>
+      <c r="T45" s="36" t="n">
+        <f aca="false">T37+T43</f>
+        <v>227.8</v>
+      </c>
+      <c r="U45" s="34"/>
+      <c r="V45" s="35"/>
     </row>
-    <row r="49" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="33"/>
-      <c r="K49" s="1" t="s">
+    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B46" s="35"/>
+      <c r="C46" s="35"/>
+      <c r="D46" s="35"/>
+      <c r="E46" s="35"/>
+      <c r="F46" s="35"/>
+      <c r="G46" s="35"/>
+      <c r="H46" s="35"/>
+      <c r="I46" s="35"/>
+      <c r="S46" s="36" t="s">
+        <v>90</v>
+      </c>
+      <c r="T46" s="36" t="n">
+        <f aca="false">T38-T42</f>
+        <v>74.3719</v>
+      </c>
+      <c r="U46" s="34"/>
+      <c r="V46" s="35"/>
+    </row>
+    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B47" s="35"/>
+      <c r="C47" s="35"/>
+      <c r="D47" s="35"/>
+      <c r="E47" s="35"/>
+      <c r="F47" s="35"/>
+      <c r="G47" s="35"/>
+      <c r="H47" s="35"/>
+      <c r="I47" s="35"/>
+      <c r="S47" s="36" t="s">
+        <v>98</v>
+      </c>
+      <c r="T47" s="36" t="n">
+        <f aca="false">T46/T45</f>
+        <v>0.326478928884987</v>
+      </c>
+      <c r="U47" s="34"/>
+      <c r="V47" s="35"/>
+    </row>
+    <row r="50" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="39"/>
+      <c r="O50" s="1"/>
+      <c r="P50" s="1"/>
+      <c r="V50" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="Y50" s="1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="39"/>
+      <c r="K52" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="O49" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="P49" s="1"/>
+      <c r="O52" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="P52" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
report final, table et grpahique
</commit_message>
<xml_diff>
--- a/combined.xlsx
+++ b/combined.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="220">
   <si>
     <t xml:space="preserve">Country</t>
   </si>
@@ -124,7 +124,7 @@
     <t xml:space="preserve">table_scenario</t>
   </si>
   <si>
-    <t xml:space="preserve">New revenue </t>
+    <t xml:space="preserve">New revenues </t>
   </si>
   <si>
     <t xml:space="preserve">Foregone revenues</t>
@@ -133,529 +133,532 @@
     <t xml:space="preserve">New Funds</t>
   </si>
   <si>
+    <t xml:space="preserve">Net new ressources</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Domestic budget gain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relative gain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">table_sscenario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6 NOR scenario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status-quo scenario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tax base </t>
+  </si>
+  <si>
+    <t xml:space="preserve">share of </t>
+  </si>
+  <si>
+    <t xml:space="preserve">passenger flow preserving reform</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Austria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Austria        </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Austria     </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  3,73 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Austria              </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 124$^{a}$       </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.57 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Belgium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Belgium        </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Belgium     </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  3,08 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Belgium              </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ---       </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.25 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bulgaria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bulgaria       </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  4,73 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bulgaria             </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.15 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Croatia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Croatia        </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  7,63 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Croatia              </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.28 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cyprus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cyprus         </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 16,92 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cyprus               </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> ---$^{b}$ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cyprus$^{a}$   </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.45 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Czechia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Czechia        </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Czechia     </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  2,52 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Czech Republic       </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Czech Republic </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.72 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Denmark</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Denmark        </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Denmark     </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  4,77 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Denmark              </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.53 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estonia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estonia        </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  4,16 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Estonia              </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.44 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finland</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finland        </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  4,34 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Finland              </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.40 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">France</t>
+  </si>
+  <si>
+    <t xml:space="preserve">France         </t>
+  </si>
+  <si>
+    <t xml:space="preserve">France      </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  3,12 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">France               </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 760$^{c}$ </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.48 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Germany</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Germany        </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Germany     </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  2,34 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Germany              </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 1{,}213   </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.54 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Greece</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Greece         </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Greece      </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 18,82 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Greece               </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.20 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hungary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hungary        </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  3,04 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hungary              </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.50 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ireland</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ireland        </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ireland     </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  3,90 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ireland              </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.33 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Italy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Italy          </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Italy       </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  5,68 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Italy                </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 637$^{d}$ </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.36 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Latvia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Latvia         </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  7,24 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Latvia               </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lithuania</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lithuania      </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  3,21 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lithuania            </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.26 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Luxembourg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Luxembourg     </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  6,42 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Luxembourg           </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Luxembourg$^{a}$ </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.43 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Malta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Malta          </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 24,29 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Malta                </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Malta$^{a}$    </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.46 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Netherlands</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Netherlands    </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Netherlands </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  3,17 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Netherlands          </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Poland</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Poland         </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Poland      </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  2,43 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Poland               </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.49 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Portugal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Portugal       </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Portugal    </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 12,14 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Portugal             </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Romania</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Romania        </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  2,95 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Romania              </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.08 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slovakia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slovakia       </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  0,61 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slovakia             </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slovenia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slovenia       </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  0,69 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Slovenia             </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.17 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spain          </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spain       </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 10,37 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spain                </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 373$^{c}$ </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sweden</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sweden         </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sweden      </t>
+  </si>
+  <si>
+    <t xml:space="preserve">  3,47 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sweden               </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 0.83 \\</t>
+  </si>
+  <si>
+    <t xml:space="preserve">European Union</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Taux effectif (inclus elasticité)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Taux effectif</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Autriche </t>
+  </si>
+  <si>
+    <t xml:space="preserve">124 M en 2024 a 5 % pub</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Budget 2026 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">8 % de croissance du secteur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">share GNI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reward fund</t>
+  </si>
+  <si>
     <t xml:space="preserve">NOR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Domestic budget gain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Relative gain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">table_sscenario</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6 NOR scenario</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Status-quo scenario</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tax base </t>
-  </si>
-  <si>
-    <t xml:space="preserve">share of </t>
-  </si>
-  <si>
-    <t xml:space="preserve">passenger flow preserving reform</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Austria</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Austria        </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Austria     </t>
-  </si>
-  <si>
-    <t xml:space="preserve">  3,73 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Austria              </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 124$^{a}$       </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 0.57 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Belgium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Belgium        </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Belgium     </t>
-  </si>
-  <si>
-    <t xml:space="preserve">  3,08 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Belgium              </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> ---       </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 0.25 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bulgaria</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bulgaria       </t>
-  </si>
-  <si>
-    <t xml:space="preserve">  4,73 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bulgaria             </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 0.15 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Croatia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Croatia        </t>
-  </si>
-  <si>
-    <t xml:space="preserve">  7,63 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Croatia              </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 0.28 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cyprus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cyprus         </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 16,92 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cyprus               </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> ---$^{b}$ </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cyprus$^{a}$   </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 0.45 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Czechia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Czechia        </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Czechia     </t>
-  </si>
-  <si>
-    <t xml:space="preserve">  2,52 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Czech Republic       </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Czech Republic </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 0.72 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Denmark</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Denmark        </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Denmark     </t>
-  </si>
-  <si>
-    <t xml:space="preserve">  4,77 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Denmark              </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 0.53 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estonia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estonia        </t>
-  </si>
-  <si>
-    <t xml:space="preserve">  4,16 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Estonia              </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 0.44 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finland</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finland        </t>
-  </si>
-  <si>
-    <t xml:space="preserve">  4,34 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Finland              </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 0.40 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">France</t>
-  </si>
-  <si>
-    <t xml:space="preserve">France         </t>
-  </si>
-  <si>
-    <t xml:space="preserve">France      </t>
-  </si>
-  <si>
-    <t xml:space="preserve">  3,12 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">France               </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 760$^{c}$ </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 0.48 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Germany</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Germany        </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Germany     </t>
-  </si>
-  <si>
-    <t xml:space="preserve">  2,34 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Germany              </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 1{,}213   </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 0.54 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Greece</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Greece         </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Greece      </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 18,82 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Greece               </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 0.20 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hungary</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hungary        </t>
-  </si>
-  <si>
-    <t xml:space="preserve">  3,04 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hungary              </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 0.50 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ireland</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ireland        </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ireland     </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
-    <t xml:space="preserve">  3,90 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ireland              </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 0.33 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Italy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Italy          </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Italy       </t>
-  </si>
-  <si>
-    <t xml:space="preserve">  5,68 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Italy                </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 637$^{d}$ </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 0.36 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Latvia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Latvia         </t>
-  </si>
-  <si>
-    <t xml:space="preserve">  7,24 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Latvia               </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lithuania</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lithuania      </t>
-  </si>
-  <si>
-    <t xml:space="preserve">  3,21 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lithuania            </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 0.26 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Luxembourg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Luxembourg     </t>
-  </si>
-  <si>
-    <t xml:space="preserve">  6,42 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Luxembourg           </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Luxembourg$^{a}$ </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 0.43 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Malta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Malta          </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 24,29 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Malta                </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Malta$^{a}$    </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 0.46 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Netherlands</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Netherlands    </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Netherlands </t>
-  </si>
-  <si>
-    <t xml:space="preserve">  3,17 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Netherlands          </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Poland</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Poland         </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Poland      </t>
-  </si>
-  <si>
-    <t xml:space="preserve">  2,43 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Poland               </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 0.49 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Portugal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Portugal       </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Portugal    </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 12,14 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Portugal             </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Romania</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Romania        </t>
-  </si>
-  <si>
-    <t xml:space="preserve">  2,95 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Romania              </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 0.08 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Slovakia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Slovakia       </t>
-  </si>
-  <si>
-    <t xml:space="preserve">  0,61 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Slovakia             </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Slovenia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Slovenia       </t>
-  </si>
-  <si>
-    <t xml:space="preserve">  0,69 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Slovenia             </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 0.17 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spain</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spain          </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spain       </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 10,37 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spain                </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 373$^{c}$ </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sweden</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sweden         </t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sweden      </t>
-  </si>
-  <si>
-    <t xml:space="preserve">  3,47 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sweden               </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 0.83 \\</t>
-  </si>
-  <si>
-    <t xml:space="preserve">European Union</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Taux effectif (inclus elasticité)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Taux effectif</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Autriche </t>
-  </si>
-  <si>
-    <t xml:space="preserve">124 M en 2024 a 5 % pub</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Budget 2026 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">8 % de croissance du secteur</t>
-  </si>
-  <si>
-    <t xml:space="preserve">share GNI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reward fund</t>
   </si>
   <si>
     <t xml:space="preserve">GNI contrib reduction</t>
@@ -2595,11 +2598,11 @@
         </c:ser>
         <c:gapWidth val="100"/>
         <c:overlap val="100"/>
-        <c:axId val="51947549"/>
-        <c:axId val="798835"/>
+        <c:axId val="31036089"/>
+        <c:axId val="65090437"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="51947549"/>
+        <c:axId val="31036089"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2631,7 +2634,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="798835"/>
+        <c:crossAx val="65090437"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2639,7 +2642,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="798835"/>
+        <c:axId val="65090437"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2680,7 +2683,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="51947549"/>
+        <c:crossAx val="31036089"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -9031,7 +9034,7 @@
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="P44" s="47" t="s">
-        <v>37</v>
+        <v>212</v>
       </c>
       <c r="Q44" s="47" t="n">
         <f aca="false">R36/1000 -Q43</f>
@@ -9051,7 +9054,7 @@
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="P45" s="47" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="Q45" s="47" t="n">
         <f aca="false">Q44-Q46-Q47</f>
@@ -9071,7 +9074,7 @@
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="P46" s="47" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="Q46" s="48" t="n">
         <v>14</v>
@@ -9090,7 +9093,7 @@
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="P47" s="47" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="Q47" s="48" t="n">
         <v>24</v>
@@ -9117,7 +9120,7 @@
       <c r="H48" s="43"/>
       <c r="I48" s="43"/>
       <c r="P48" s="47" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="Q48" s="47" t="n">
         <f aca="false">Q40+Q46</f>
@@ -9173,7 +9176,7 @@
       <c r="H50" s="43"/>
       <c r="I50" s="43"/>
       <c r="P50" s="47" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="Q50" s="49" t="n">
         <f aca="false">Q49/Q48</f>
@@ -9194,10 +9197,10 @@
     <row r="53" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="50"/>
       <c r="AA53" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="AE53" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AF53" s="1"/>
     </row>

</xml_diff>

<commit_message>
header tables dans fichier report, xlsx2tex renvoies juste les valeurs, update a 102 et modifs review GC
</commit_message>
<xml_diff>
--- a/combined.xlsx
+++ b/combined.xlsx
@@ -2493,85 +2493,85 @@
                 <c:formatCode>#,##0.00</c:formatCode>
                 <c:ptCount val="27"/>
                 <c:pt idx="0">
-                  <c:v>0.356975983763671</c:v>
+                  <c:v>0.340749802683504</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.284373204986587</c:v>
+                  <c:v>0.271447150214469</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.449691064366367</c:v>
+                  <c:v>0.429250561440623</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.57868988164466</c:v>
+                  <c:v>0.552385796115358</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.00346521145975</c:v>
+                  <c:v>0.957853156393402</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.297353728254231</c:v>
+                  <c:v>0.28383764969722</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.17735760665507</c:v>
+                  <c:v>0.169295897261657</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.238046538722936</c:v>
+                  <c:v>0.227226241508257</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.167032696832898</c:v>
+                  <c:v>0.159440301522312</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.354245258835647</c:v>
+                  <c:v>0.338143201615845</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.22759448054403</c:v>
+                  <c:v>0.217249276882938</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0.512370232362714</c:v>
+                  <c:v>0.489080676346227</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0.246951465176869</c:v>
+                  <c:v>0.23572639857792</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.172810891520677</c:v>
+                  <c:v>0.16495585099701</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.458197003274568</c:v>
+                  <c:v>0.437369866762087</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.222385487528345</c:v>
+                  <c:v>0.212277056277056</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.217873222748815</c:v>
+                  <c:v>0.207969894442051</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.524657023974638</c:v>
+                  <c:v>0.500808977430337</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0.965627598278754</c:v>
+                  <c:v>0.921735434720629</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0.193295873170592</c:v>
+                  <c:v>0.184509697117383</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0.214791088333689</c:v>
+                  <c:v>0.205027857045794</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0.444361628318584</c:v>
+                  <c:v>0.424163372485921</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0.218634168090956</c:v>
+                  <c:v>0.208696251359549</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>0.196551213796789</c:v>
+                  <c:v>0.187617067715117</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>0.314388296322201</c:v>
+                  <c:v>0.300097919216646</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>0.374689323469409</c:v>
+                  <c:v>0.357657990584436</c:v>
                 </c:pt>
                 <c:pt idx="26">
-                  <c:v>0.188976041165338</c:v>
+                  <c:v>0.180386221112368</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2579,11 +2579,11 @@
         </c:ser>
         <c:gapWidth val="100"/>
         <c:overlap val="100"/>
-        <c:axId val="49219474"/>
-        <c:axId val="88960972"/>
+        <c:axId val="49272629"/>
+        <c:axId val="47809847"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="49219474"/>
+        <c:axId val="49272629"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2615,7 +2615,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="88960972"/>
+        <c:crossAx val="47809847"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2623,7 +2623,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="88960972"/>
+        <c:axId val="47809847"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2664,7 +2664,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="49219474"/>
+        <c:crossAx val="49272629"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2881,6 +2881,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="2" width="13.76"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="11.27"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="18.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="11.02"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="14.37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="19" style="1" width="17.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="33" min="21" style="1" width="14.58"/>
@@ -3416,11 +3417,11 @@
       </c>
       <c r="M8" s="23" t="n">
         <f aca="false">O8*$M$37/100</f>
-        <v>1456.3692</v>
+        <v>1390.1706</v>
       </c>
       <c r="N8" s="24" t="n">
         <f aca="false">M8/$P8/10</f>
-        <v>0.356975983763671</v>
+        <v>0.340749802683504</v>
       </c>
       <c r="O8" s="23" t="n">
         <v>9900</v>
@@ -3434,31 +3435,31 @@
       </c>
       <c r="R8" s="23" t="n">
         <f aca="false">H8+F8+B8+D8+J8+M8</f>
-        <v>3130.1098</v>
+        <v>3063.9112</v>
       </c>
       <c r="S8" s="26" t="n">
         <f aca="false">R8/$P8/1000*100</f>
-        <v>0.76723266678759</v>
+        <v>0.751006485707423</v>
       </c>
       <c r="T8" s="26" t="n">
         <f aca="false">R8/P8</f>
-        <v>7.6723266678759</v>
+        <v>7.51006485707423</v>
       </c>
       <c r="U8" s="2" t="n">
         <f aca="false">3/5*H8+M8/3</f>
-        <v>1037.4564</v>
+        <v>1015.3902</v>
       </c>
       <c r="V8" s="26" t="n">
         <f aca="false">U8/$P8/1000*100</f>
-        <v>0.254294734468373</v>
+        <v>0.248886007441651</v>
       </c>
       <c r="W8" s="2" t="n">
         <f aca="false">R8-U8</f>
-        <v>2092.6534</v>
+        <v>2048.521</v>
       </c>
       <c r="X8" s="26" t="n">
         <f aca="false">W8/$P8/1000*100</f>
-        <v>0.512937932319217</v>
+        <v>0.502120478265772</v>
       </c>
       <c r="Y8" s="23" t="n">
         <f aca="false">124*(1.08)^4*3/5</f>
@@ -3475,31 +3476,31 @@
       </c>
       <c r="AC8" s="2" t="n">
         <f aca="false">1000/100*Q8*($Q$41+$Q$47-$Q$49)-AA8</f>
-        <v>1584.90627054526</v>
+        <v>1547.54496995203</v>
       </c>
       <c r="AD8" s="26" t="n">
         <f aca="false">AC8/$P8/1000*100</f>
-        <v>0.388482175468353</v>
+        <v>0.379324410367336</v>
       </c>
       <c r="AE8" s="2" t="n">
         <f aca="false">AC8+Q8/100*1000 *($Q$46+$Q$43)</f>
-        <v>2829.73991968701</v>
+        <v>2773.69796879718</v>
       </c>
       <c r="AF8" s="26" t="n">
         <f aca="false">AE8/$P8/1000*100</f>
-        <v>0.693607906309474</v>
+        <v>0.679871258657948</v>
       </c>
       <c r="AG8" s="26" t="n">
         <f aca="false">-Y8+($Q$45 + $Q$46)*1000*Q8/100</f>
-        <v>1304.6965339276</v>
+        <v>1267.33523333438</v>
       </c>
       <c r="AH8" s="26" t="n">
         <f aca="false">AG8/P8/10</f>
-        <v>0.319798941581474</v>
+        <v>0.310641176480456</v>
       </c>
       <c r="AI8" s="26" t="n">
         <f aca="false">AG8/P8</f>
-        <v>3.19798941581474</v>
+        <v>3.10641176480456</v>
       </c>
       <c r="AK8" s="26" t="n">
         <f aca="false">-Q8*($Q$47)*10</f>
@@ -3645,11 +3646,11 @@
       </c>
       <c r="M9" s="23" t="n">
         <f aca="false">O9*$M$37/100</f>
-        <v>1441.6584</v>
+        <v>1376.12847272727</v>
       </c>
       <c r="N9" s="24" t="n">
         <f aca="false">M9/$P9/10</f>
-        <v>0.284373204986587</v>
+        <v>0.271447150214469</v>
       </c>
       <c r="O9" s="23" t="n">
         <v>9800</v>
@@ -3663,31 +3664,31 @@
       </c>
       <c r="R9" s="23" t="n">
         <f aca="false">H9+F9+B9+D9+J9+M9</f>
-        <v>2866.4324</v>
+        <v>2800.90247272727</v>
       </c>
       <c r="S9" s="26" t="n">
         <f aca="false">R9/$P9/1000*100</f>
-        <v>0.565415890800063</v>
+        <v>0.552489836027946</v>
       </c>
       <c r="T9" s="26" t="n">
         <f aca="false">R9/P9</f>
-        <v>5.65415890800063</v>
+        <v>5.52489836027946</v>
       </c>
       <c r="U9" s="2" t="n">
         <f aca="false">3/5*H9+M9/3</f>
-        <v>913.7528</v>
+        <v>891.909490909091</v>
       </c>
       <c r="V9" s="26" t="n">
         <f aca="false">U9/$P9/1000*100</f>
-        <v>0.180241596970175</v>
+        <v>0.175932912046136</v>
       </c>
       <c r="W9" s="2" t="n">
         <f aca="false">R9-U9</f>
-        <v>1952.6796</v>
+        <v>1908.99298181818</v>
       </c>
       <c r="X9" s="26" t="n">
         <f aca="false">W9/$P9/1000*100</f>
-        <v>0.385174293829888</v>
+        <v>0.37655692398181</v>
       </c>
       <c r="Y9" s="26"/>
       <c r="Z9" s="30" t="n">
@@ -3704,31 +3705,31 @@
       </c>
       <c r="AC9" s="2" t="n">
         <f aca="false">1000/100*Q9*($Q$41+$Q$47-$Q$49)-AA9</f>
-        <v>2034.12853432534</v>
+        <v>1987.70232836922</v>
       </c>
       <c r="AD9" s="26" t="n">
         <f aca="false">AC9/$P9/1000*100</f>
-        <v>0.401240439941088</v>
+        <v>0.392082674840071</v>
       </c>
       <c r="AE9" s="2" t="n">
         <f aca="false">AC9+Q9/100*1000 *($Q$46+$Q$43)</f>
-        <v>3580.99393939749</v>
+        <v>3511.35463046331</v>
       </c>
       <c r="AF9" s="26" t="n">
         <f aca="false">AE9/$P9/1000*100</f>
-        <v>0.70636617078221</v>
+        <v>0.692629523130684</v>
       </c>
       <c r="AG9" s="26" t="n">
         <f aca="false">-Z9+($Q$45 + $Q$46)*1000*Q9/100</f>
-        <v>1685.93201181242</v>
+        <v>1639.5058058563</v>
       </c>
       <c r="AH9" s="26" t="n">
         <f aca="false">AG9/P9/10</f>
-        <v>0.332557206054209</v>
+        <v>0.323399440953192</v>
       </c>
       <c r="AI9" s="26" t="n">
         <f aca="false">AG9/P9</f>
-        <v>3.32557206054209</v>
+        <v>3.23399440953192</v>
       </c>
       <c r="AK9" s="26" t="n">
         <f aca="false">-Q9*($Q$47)*10</f>
@@ -3874,11 +3875,11 @@
       </c>
       <c r="M10" s="23" t="n">
         <f aca="false">O10*$M$37/100</f>
-        <v>235.3728</v>
+        <v>224.674036363636</v>
       </c>
       <c r="N10" s="24" t="n">
         <f aca="false">M10/$P10/10</f>
-        <v>0.449691064366367</v>
+        <v>0.429250561440623</v>
       </c>
       <c r="O10" s="23" t="n">
         <v>1600</v>
@@ -3892,31 +3893,31 @@
       </c>
       <c r="R10" s="23" t="n">
         <f aca="false">H10+F10+B10+D10+J10+M10</f>
-        <v>394.5746</v>
+        <v>383.875836363636</v>
       </c>
       <c r="S10" s="26" t="n">
         <f aca="false">R10/$P10/1000*100</f>
-        <v>0.753853766645651</v>
+        <v>0.733413263719907</v>
       </c>
       <c r="T10" s="26" t="n">
         <f aca="false">R10/P10</f>
-        <v>7.53853766645651</v>
+        <v>7.33413263719907</v>
       </c>
       <c r="U10" s="2" t="n">
         <f aca="false">3/5*H10+M10/3</f>
-        <v>102.4576</v>
+        <v>98.8913454545455</v>
       </c>
       <c r="V10" s="26" t="n">
         <f aca="false">U10/$P10/1000*100</f>
-        <v>0.195750176725703</v>
+        <v>0.188936675750455</v>
       </c>
       <c r="W10" s="2" t="n">
         <f aca="false">R10-U10</f>
-        <v>292.117</v>
+        <v>284.984490909091</v>
       </c>
       <c r="X10" s="26" t="n">
         <f aca="false">W10/$P10/1000*100</f>
-        <v>0.558103589919948</v>
+        <v>0.544476587969452</v>
       </c>
       <c r="Y10" s="26"/>
       <c r="Z10" s="26"/>
@@ -3930,31 +3931,31 @@
       </c>
       <c r="AC10" s="2" t="n">
         <f aca="false">1000/100*Q10*($Q$41+$Q$47-$Q$49)-AA10</f>
-        <v>216.321517901062</v>
+        <v>211.528252069539</v>
       </c>
       <c r="AD10" s="26" t="n">
         <f aca="false">AC10/$P10/1000*100</f>
-        <v>0.413292672858872</v>
+        <v>0.404134907757855</v>
       </c>
       <c r="AE10" s="2" t="n">
         <f aca="false">AC10+Q10/100*1000 *($Q$46+$Q$43)</f>
-        <v>376.027376680613</v>
+        <v>368.837477933328</v>
       </c>
       <c r="AF10" s="26" t="n">
         <f aca="false">AE10/$P10/1000*100</f>
-        <v>0.718418403699993</v>
+        <v>0.704681756048467</v>
       </c>
       <c r="AG10" s="26" t="n">
         <f aca="false">-AA10+($Q$45 + $Q$46)*1000*Q10/100</f>
-        <v>180.372026452331</v>
+        <v>175.578760620807</v>
       </c>
       <c r="AH10" s="26" t="n">
         <f aca="false">AG10/P10/10</f>
-        <v>0.344609438971993</v>
+        <v>0.335451673870976</v>
       </c>
       <c r="AI10" s="26" t="n">
         <f aca="false">AG10/P10</f>
-        <v>3.44609438971993</v>
+        <v>3.35451673870976</v>
       </c>
       <c r="AK10" s="26" t="n">
         <f aca="false">-Q10*($Q$47)*10</f>
@@ -4100,11 +4101,11 @@
       </c>
       <c r="M11" s="23" t="n">
         <f aca="false">O11*$M$37/100</f>
-        <v>338.3484</v>
+        <v>322.968927272727</v>
       </c>
       <c r="N11" s="24" t="n">
         <f aca="false">M11/$P11/10</f>
-        <v>0.57868988164466</v>
+        <v>0.552385796115358</v>
       </c>
       <c r="O11" s="23" t="n">
         <v>2300</v>
@@ -4118,31 +4119,31 @@
       </c>
       <c r="R11" s="23" t="n">
         <f aca="false">H11+F11+B11+D11+J11+M11</f>
-        <v>535.3176</v>
+        <v>519.938127272727</v>
       </c>
       <c r="S11" s="26" t="n">
         <f aca="false">R11/$P11/1000*100</f>
-        <v>0.915573647123213</v>
+        <v>0.88926956159391</v>
       </c>
       <c r="T11" s="26" t="n">
         <f aca="false">R11/P11</f>
-        <v>9.15573647123213</v>
+        <v>8.8926956159391</v>
       </c>
       <c r="U11" s="2" t="n">
         <f aca="false">3/5*H11+M11/3</f>
-        <v>134.3828</v>
+        <v>129.256309090909</v>
       </c>
       <c r="V11" s="26" t="n">
         <f aca="false">U11/$P11/1000*100</f>
-        <v>0.229839912430731</v>
+        <v>0.221071883920964</v>
       </c>
       <c r="W11" s="2" t="n">
         <f aca="false">R11-U11</f>
-        <v>400.9348</v>
+        <v>390.681818181818</v>
       </c>
       <c r="X11" s="26" t="n">
         <f aca="false">W11/$P11/1000*100</f>
-        <v>0.685733734692482</v>
+        <v>0.668197677672946</v>
       </c>
       <c r="Y11" s="26"/>
       <c r="Z11" s="26"/>
@@ -4156,27 +4157,27 @@
       </c>
       <c r="AC11" s="2" t="n">
         <f aca="false">1000/100*Q11*($Q$41+$Q$47-$Q$49)-AA11</f>
-        <v>241.643959967125</v>
+        <v>236.289597867863</v>
       </c>
       <c r="AD11" s="26" t="n">
         <f aca="false">AC11/$P11/1000*100</f>
-        <v>0.413292672858872</v>
+        <v>0.404134907757855</v>
       </c>
       <c r="AE11" s="2" t="n">
         <f aca="false">AC11+Q11/100*1000 *($Q$46+$Q$43)</f>
-        <v>420.044872275312</v>
+        <v>412.013329126418</v>
       </c>
       <c r="AF11" s="26" t="n">
         <f aca="false">AE11/$P11/1000*100</f>
-        <v>0.718418403699993</v>
+        <v>0.704681756048467</v>
       </c>
       <c r="AG11" s="26" t="n">
         <f aca="false">-AA11+($Q$45 + $Q$46)*1000*Q11/100</f>
-        <v>201.486246778145</v>
+        <v>196.131884678882</v>
       </c>
       <c r="AH11" s="26" t="n">
         <f aca="false">AG11/P11/10</f>
-        <v>0.344609438971993</v>
+        <v>0.335451673870976</v>
       </c>
       <c r="AI11" s="26" t="n">
         <f aca="false">ROUND(AG11/P11 *100/1000, 2)</f>
@@ -4326,11 +4327,11 @@
       </c>
       <c r="M12" s="23" t="n">
         <f aca="false">O12*$M$37/100</f>
-        <v>220.662</v>
+        <v>210.631909090909</v>
       </c>
       <c r="N12" s="24" t="n">
         <f aca="false">M12/$P12/10</f>
-        <v>1.00346521145975</v>
+        <v>0.957853156393402</v>
       </c>
       <c r="O12" s="23" t="n">
         <v>1500</v>
@@ -4344,31 +4345,31 @@
       </c>
       <c r="R12" s="23" t="n">
         <f aca="false">H12+F12+B12+D12+J12+M12</f>
-        <v>368.1306</v>
+        <v>358.100509090909</v>
       </c>
       <c r="S12" s="26" t="n">
         <f aca="false">R12/$P12/1000*100</f>
-        <v>1.67408185538881</v>
+        <v>1.62846980032246</v>
       </c>
       <c r="T12" s="26" t="n">
         <f aca="false">R12/P12</f>
-        <v>16.7408185538881</v>
+        <v>16.2846980032246</v>
       </c>
       <c r="U12" s="2" t="n">
         <f aca="false">3/5*H12+M12/3</f>
-        <v>101.154</v>
+        <v>97.8106363636364</v>
       </c>
       <c r="V12" s="26" t="n">
         <f aca="false">U12/$P12/1000*100</f>
-        <v>0.46</v>
+        <v>0.444795981644549</v>
       </c>
       <c r="W12" s="2" t="n">
         <f aca="false">R12-U12</f>
-        <v>266.9766</v>
+        <v>260.289872727273</v>
       </c>
       <c r="X12" s="26" t="n">
         <f aca="false">W12/$P12/1000*100</f>
-        <v>1.21408185538881</v>
+        <v>1.18367381867791</v>
       </c>
       <c r="Y12" s="26"/>
       <c r="Z12" s="26"/>
@@ -4382,27 +4383,27 @@
       </c>
       <c r="AC12" s="2" t="n">
         <f aca="false">1000/100*Q12*($Q$41+$Q$47-$Q$49)-AA12</f>
-        <v>90.8830587616661</v>
+        <v>88.8692662159524</v>
       </c>
       <c r="AD12" s="26" t="n">
         <f aca="false">AC12/$P12/1000*100</f>
-        <v>0.413292672858873</v>
+        <v>0.404134907757855</v>
       </c>
       <c r="AE12" s="2" t="n">
         <f aca="false">AC12+Q12/100*1000 *($Q$46+$Q$43)</f>
-        <v>157.980206973629</v>
+        <v>154.959518155058</v>
       </c>
       <c r="AF12" s="26" t="n">
         <f aca="false">AE12/$P12/1000*100</f>
-        <v>0.718418403699994</v>
+        <v>0.704681756048468</v>
       </c>
       <c r="AG12" s="26" t="n">
         <f aca="false">-AA12+($Q$45 + $Q$46)*1000*Q12/100</f>
-        <v>75.7796156299414</v>
+        <v>73.7658230842277</v>
       </c>
       <c r="AH12" s="26" t="n">
         <f aca="false">AG12/P12/10</f>
-        <v>0.344609438971994</v>
+        <v>0.335451673870976</v>
       </c>
       <c r="AI12" s="26" t="n">
         <f aca="false">ROUND(AG12/P12 *100/1000, 2)</f>
@@ -4552,11 +4553,11 @@
       </c>
       <c r="M13" s="23" t="n">
         <f aca="false">O13*$M$37/100</f>
-        <v>676.6968</v>
+        <v>645.937854545455</v>
       </c>
       <c r="N13" s="24" t="n">
         <f aca="false">M13/$P13/10</f>
-        <v>0.297353728254231</v>
+        <v>0.28383764969722</v>
       </c>
       <c r="O13" s="23" t="n">
         <v>4600</v>
@@ -4570,31 +4571,31 @@
       </c>
       <c r="R13" s="23" t="n">
         <f aca="false">H13+F13+B13+D13+J13+M13</f>
-        <v>1572.1664</v>
+        <v>1541.40745454545</v>
       </c>
       <c r="S13" s="26" t="n">
         <f aca="false">R13/$P13/1000*100</f>
-        <v>0.690840477561046</v>
+        <v>0.677324399004036</v>
       </c>
       <c r="T13" s="26" t="n">
         <f aca="false">R13/P13</f>
-        <v>6.90840477561046</v>
+        <v>6.77324399004036</v>
       </c>
       <c r="U13" s="2" t="n">
         <f aca="false">3/5*H13+M13/3</f>
-        <v>434.3656</v>
+        <v>424.112618181818</v>
       </c>
       <c r="V13" s="26" t="n">
         <f aca="false">U13/$P13/1000*100</f>
-        <v>0.190868688289033</v>
+        <v>0.186363328770029</v>
       </c>
       <c r="W13" s="2" t="n">
         <f aca="false">R13-U13</f>
-        <v>1137.8008</v>
+        <v>1117.29483636364</v>
       </c>
       <c r="X13" s="26" t="n">
         <f aca="false">W13/$P13/1000*100</f>
-        <v>0.499971789272014</v>
+        <v>0.490961070234007</v>
       </c>
       <c r="Y13" s="26"/>
       <c r="Z13" s="26"/>
@@ -4608,27 +4609,27 @@
       </c>
       <c r="AC13" s="2" t="n">
         <f aca="false">1000/100*Q13*($Q$41+$Q$47-$Q$49)-AA13</f>
-        <v>940.542534405121</v>
+        <v>919.701933631783</v>
       </c>
       <c r="AD13" s="26" t="n">
         <f aca="false">AC13/$P13/1000*100</f>
-        <v>0.413292672858872</v>
+        <v>0.404134907757855</v>
       </c>
       <c r="AE13" s="2" t="n">
         <f aca="false">AC13+Q13/100*1000 *($Q$46+$Q$43)</f>
-        <v>1634.92631385218</v>
+        <v>1603.66541269218</v>
       </c>
       <c r="AF13" s="26" t="n">
         <f aca="false">AE13/$P13/1000*100</f>
-        <v>0.718418403699993</v>
+        <v>0.704681756048467</v>
       </c>
       <c r="AG13" s="26" t="n">
         <f aca="false">-AA13+($Q$45 + $Q$46)*1000*Q13/100</f>
-        <v>784.238038551734</v>
+        <v>763.397437778396</v>
       </c>
       <c r="AH13" s="26" t="n">
         <f aca="false">AG13/P13/10</f>
-        <v>0.344609438971993</v>
+        <v>0.335451673870976</v>
       </c>
       <c r="AI13" s="26" t="n">
         <f aca="false">ROUND(AG13/P13 *100/1000, 2)</f>
@@ -4778,11 +4779,11 @@
       </c>
       <c r="M14" s="23" t="n">
         <f aca="false">O14*$M$37/100</f>
-        <v>617.8536</v>
+        <v>589.769345454546</v>
       </c>
       <c r="N14" s="24" t="n">
         <f aca="false">M14/$P14/10</f>
-        <v>0.17735760665507</v>
+        <v>0.169295897261657</v>
       </c>
       <c r="O14" s="23" t="n">
         <v>4200</v>
@@ -4796,31 +4797,31 @@
       </c>
       <c r="R14" s="23" t="n">
         <f aca="false">H14+F14+B14+D14+J14+M14</f>
-        <v>1894.3278</v>
+        <v>1866.24354545455</v>
       </c>
       <c r="S14" s="26" t="n">
         <f aca="false">R14/$P14/1000*100</f>
-        <v>0.543775167496254</v>
+        <v>0.535713458102842</v>
       </c>
       <c r="T14" s="26" t="n">
         <f aca="false">R14/P14</f>
-        <v>5.43775167496254</v>
+        <v>5.35713458102842</v>
       </c>
       <c r="U14" s="2" t="n">
         <f aca="false">3/5*H14+M14/3</f>
-        <v>525.7512</v>
+        <v>516.389781818182</v>
       </c>
       <c r="V14" s="26" t="n">
         <f aca="false">U14/$P14/1000*100</f>
-        <v>0.15091920566301</v>
+        <v>0.148231969198539</v>
       </c>
       <c r="W14" s="2" t="n">
         <f aca="false">R14-U14</f>
-        <v>1368.5766</v>
+        <v>1349.85376363636</v>
       </c>
       <c r="X14" s="26" t="n">
         <f aca="false">W14/$P14/1000*100</f>
-        <v>0.392855961833244</v>
+        <v>0.387481488904303</v>
       </c>
       <c r="Y14" s="26"/>
       <c r="Z14" s="26"/>
@@ -4834,27 +4835,27 @@
       </c>
       <c r="AC14" s="2" t="n">
         <f aca="false">1000/100*Q14*($Q$41+$Q$47-$Q$49)-AA14</f>
-        <v>1439.77115273154</v>
+        <v>1407.86861275973</v>
       </c>
       <c r="AD14" s="26" t="n">
         <f aca="false">AC14/$P14/1000*100</f>
-        <v>0.413292672858873</v>
+        <v>0.404134907757855</v>
       </c>
       <c r="AE14" s="2" t="n">
         <f aca="false">AC14+Q14/100*1000 *($Q$46+$Q$43)</f>
-        <v>2502.72545623352</v>
+        <v>2454.87164627581</v>
       </c>
       <c r="AF14" s="26" t="n">
         <f aca="false">AE14/$P14/1000*100</f>
-        <v>0.718418403699994</v>
+        <v>0.704681756048468</v>
       </c>
       <c r="AG14" s="26" t="n">
         <f aca="false">-AA14+($Q$45 + $Q$46)*1000*Q14/100</f>
-        <v>1200.50211816918</v>
+        <v>1168.59957819737</v>
       </c>
       <c r="AH14" s="26" t="n">
         <f aca="false">AG14/P14/10</f>
-        <v>0.344609438971994</v>
+        <v>0.335451673870976</v>
       </c>
       <c r="AI14" s="26" t="n">
         <f aca="false">ROUND(AG14/P14 *100/1000, 2)</f>
@@ -5004,11 +5005,11 @@
       </c>
       <c r="M15" s="23" t="n">
         <f aca="false">O15*$M$37/100</f>
-        <v>73.554</v>
+        <v>70.2106363636364</v>
       </c>
       <c r="N15" s="24" t="n">
         <f aca="false">M15/$P15/10</f>
-        <v>0.238046538722936</v>
+        <v>0.227226241508257</v>
       </c>
       <c r="O15" s="23" t="n">
         <v>500</v>
@@ -5022,31 +5023,31 @@
       </c>
       <c r="R15" s="23" t="n">
         <f aca="false">H15+F15+B15+D15+J15+M15</f>
-        <v>167.6546</v>
+        <v>164.311236363636</v>
       </c>
       <c r="S15" s="26" t="n">
         <f aca="false">R15/$P15/1000*100</f>
-        <v>0.542589080552769</v>
+        <v>0.53176878333809</v>
       </c>
       <c r="T15" s="26" t="n">
         <f aca="false">R15/P15</f>
-        <v>5.42589080552769</v>
+        <v>5.3176878333809</v>
       </c>
       <c r="U15" s="2" t="n">
         <f aca="false">3/5*H15+M15/3</f>
-        <v>41.918</v>
+        <v>40.8035454545455</v>
       </c>
       <c r="V15" s="26" t="n">
         <f aca="false">U15/$P15/1000*100</f>
-        <v>0.135661348263698</v>
+        <v>0.132054582525472</v>
       </c>
       <c r="W15" s="2" t="n">
         <f aca="false">R15-U15</f>
-        <v>125.7366</v>
+        <v>123.507690909091</v>
       </c>
       <c r="X15" s="26" t="n">
         <f aca="false">W15/$P15/1000*100</f>
-        <v>0.406927732289071</v>
+        <v>0.399714200812618</v>
       </c>
       <c r="Y15" s="26"/>
       <c r="Z15" s="26"/>
@@ -5060,27 +5061,27 @@
       </c>
       <c r="AC15" s="2" t="n">
         <f aca="false">1000/100*Q15*($Q$41+$Q$47-$Q$49)-AA15</f>
-        <v>127.703302986663</v>
+        <v>124.873645148099</v>
       </c>
       <c r="AD15" s="26" t="n">
         <f aca="false">AC15/$P15/1000*100</f>
-        <v>0.413292672858872</v>
+        <v>0.404134907757854</v>
       </c>
       <c r="AE15" s="2" t="n">
         <f aca="false">AC15+Q15/100*1000 *($Q$46+$Q$43)</f>
-        <v>221.984102559261</v>
+        <v>217.739615801415</v>
       </c>
       <c r="AF15" s="26" t="n">
         <f aca="false">AE15/$P15/1000*100</f>
-        <v>0.718418403699992</v>
+        <v>0.704681756048466</v>
       </c>
       <c r="AG15" s="26" t="n">
         <f aca="false">-AA15+($Q$45 + $Q$46)*1000*Q15/100</f>
-        <v>106.480870547956</v>
+        <v>103.651212709393</v>
       </c>
       <c r="AH15" s="26" t="n">
         <f aca="false">AG15/P15/10</f>
-        <v>0.344609438971993</v>
+        <v>0.335451673870975</v>
       </c>
       <c r="AI15" s="26" t="n">
         <f aca="false">ROUND(AG15/P15 *100/1000, 2)</f>
@@ -5228,13 +5229,13 @@
       <c r="L16" s="23" t="n">
         <v>720</v>
       </c>
-      <c r="M16" s="23" t="n">
+      <c r="M16" s="26" t="n">
         <f aca="false">O16*$M$37/100</f>
-        <v>426.6132</v>
+        <v>407.221690909091</v>
       </c>
       <c r="N16" s="24" t="n">
         <f aca="false">M16/$P16/10</f>
-        <v>0.167032696832898</v>
+        <v>0.159440301522312</v>
       </c>
       <c r="O16" s="23" t="n">
         <v>2900</v>
@@ -5248,31 +5249,31 @@
       </c>
       <c r="R16" s="23" t="n">
         <f aca="false">H16+F16+B16+D16+J16+M16</f>
-        <v>1057.918</v>
+        <v>1038.52649090909</v>
       </c>
       <c r="S16" s="26" t="n">
         <f aca="false">R16/$P16/1000*100</f>
-        <v>0.414208694358416</v>
+        <v>0.40661629904783</v>
       </c>
       <c r="T16" s="26" t="n">
         <f aca="false">R16/P16</f>
-        <v>4.14208694358416</v>
+        <v>4.0661629904783</v>
       </c>
       <c r="U16" s="2" t="n">
         <f aca="false">3/5*H16+M16/3</f>
-        <v>233.4044</v>
+        <v>226.940563636364</v>
       </c>
       <c r="V16" s="26" t="n">
         <f aca="false">U16/$P16/1000*100</f>
-        <v>0.0913852791818548</v>
+        <v>0.0888544807449928</v>
       </c>
       <c r="W16" s="2" t="n">
         <f aca="false">R16-U16</f>
-        <v>824.5136</v>
+        <v>811.585927272727</v>
       </c>
       <c r="X16" s="26" t="n">
         <f aca="false">W16/$P16/1000*100</f>
-        <v>0.322823415176561</v>
+        <v>0.317761818302837</v>
       </c>
       <c r="Y16" s="26"/>
       <c r="Z16" s="26"/>
@@ -5286,27 +5287,27 @@
       </c>
       <c r="AC16" s="2" t="n">
         <f aca="false">1000/100*Q16*($Q$41+$Q$47-$Q$49)-AA16</f>
-        <v>1055.57841696866</v>
+        <v>1032.1888438571</v>
       </c>
       <c r="AD16" s="26" t="n">
         <f aca="false">AC16/$P16/1000*100</f>
-        <v>0.413292672858872</v>
+        <v>0.404134907757855</v>
       </c>
       <c r="AE16" s="2" t="n">
         <f aca="false">AC16+Q16/100*1000 *($Q$46+$Q$43)</f>
-        <v>1834.89089233804</v>
+        <v>1799.80653267071</v>
       </c>
       <c r="AF16" s="26" t="n">
         <f aca="false">AE16/$P16/1000*100</f>
-        <v>0.718418403699993</v>
+        <v>0.704681756048467</v>
       </c>
       <c r="AG16" s="26" t="n">
         <f aca="false">-AA16+($Q$45 + $Q$46)*1000*Q16/100</f>
-        <v>880.156629795199</v>
+        <v>856.767056683644</v>
       </c>
       <c r="AH16" s="26" t="n">
         <f aca="false">AG16/P16/10</f>
-        <v>0.344609438971993</v>
+        <v>0.335451673870976</v>
       </c>
       <c r="AI16" s="26" t="n">
         <f aca="false">ROUND(AG16/P16 *100/1000, 2)</f>
@@ -5454,13 +5455,13 @@
       <c r="L17" s="23" t="n">
         <v>5380</v>
       </c>
-      <c r="M17" s="23" t="n">
+      <c r="M17" s="26" t="n">
         <f aca="false">O17*$M$37/100</f>
-        <v>9120.696</v>
+        <v>8706.11890909091</v>
       </c>
       <c r="N17" s="24" t="n">
         <f aca="false">M17/$P17/10</f>
-        <v>0.354245258835647</v>
+        <v>0.338143201615845</v>
       </c>
       <c r="O17" s="23" t="n">
         <v>62000</v>
@@ -5474,31 +5475,31 @@
       </c>
       <c r="R17" s="23" t="n">
         <f aca="false">H17+F17+B17+D17+J17+M17</f>
-        <v>22921.0652</v>
+        <v>22506.4881090909</v>
       </c>
       <c r="S17" s="26" t="n">
         <f aca="false">R17/$P17/1000*100</f>
-        <v>0.890247704184281</v>
+        <v>0.874145646964478</v>
       </c>
       <c r="T17" s="26" t="n">
         <f aca="false">R17/P17</f>
-        <v>8.90247704184281</v>
+        <v>8.74145646964478</v>
       </c>
       <c r="U17" s="2" t="n">
         <f aca="false">3/5*H17+M17/3</f>
-        <v>7042.232</v>
+        <v>6904.03963636364</v>
       </c>
       <c r="V17" s="26" t="n">
         <f aca="false">U17/$P17/1000*100</f>
-        <v>0.273518303605413</v>
+        <v>0.268150951198813</v>
       </c>
       <c r="W17" s="2" t="n">
         <f aca="false">R17-U17</f>
-        <v>15878.8332</v>
+        <v>15602.4484727273</v>
       </c>
       <c r="X17" s="26" t="n">
         <f aca="false">W17/$P17/1000*100</f>
-        <v>0.616729400578867</v>
+        <v>0.605994695765666</v>
       </c>
       <c r="Y17" s="26" t="n">
         <f aca="false">B17</f>
@@ -5518,31 +5519,31 @@
       </c>
       <c r="AC17" s="2" t="n">
         <f aca="false">1000/100*Q17*($Q$41+$Q$47-$Q$49)-AA17</f>
-        <v>6456.98032126972</v>
+        <v>6221.19680845624</v>
       </c>
       <c r="AD17" s="26" t="n">
         <f aca="false">AC17/$P17/1000*100</f>
-        <v>0.250787293557956</v>
+        <v>0.241629528456938</v>
       </c>
       <c r="AE17" s="2" t="n">
         <f aca="false">AC17+Q17/100*1000 *($Q$46+$Q$43)</f>
-        <v>14313.0036931191</v>
+        <v>13959.3284238989</v>
       </c>
       <c r="AF17" s="26" t="n">
         <f aca="false">AE17/$P17/1000*100</f>
-        <v>0.555913024399076</v>
+        <v>0.54217637674755</v>
       </c>
       <c r="AG17" s="26" t="n">
         <f aca="false">-AA17+($Q$45 + $Q$46)*1000*Q17/100</f>
-        <v>4688.60408770167</v>
+        <v>4452.82057488819</v>
       </c>
       <c r="AH17" s="26" t="n">
         <f aca="false">AG17/P17/10</f>
-        <v>0.182104059671077</v>
+        <v>0.17294629457006</v>
       </c>
       <c r="AI17" s="26" t="n">
         <f aca="false">ROUND(AG17/P17 *100/1000, 2)</f>
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="AK17" s="26" t="n">
         <f aca="false">-Q17*($Q$47)*10</f>
@@ -5686,13 +5687,13 @@
       <c r="L18" s="23" t="n">
         <v>6040</v>
       </c>
-      <c r="M18" s="23" t="n">
+      <c r="M18" s="26" t="n">
         <f aca="false">O18*$M$37/100</f>
-        <v>8488.1316</v>
+        <v>8102.30743636364</v>
       </c>
       <c r="N18" s="24" t="n">
         <f aca="false">M18/$P18/10</f>
-        <v>0.22759448054403</v>
+        <v>0.217249276882938</v>
       </c>
       <c r="O18" s="23" t="n">
         <v>57700</v>
@@ -5706,31 +5707,31 @@
       </c>
       <c r="R18" s="23" t="n">
         <f aca="false">H18+F18+B18+D18+J18+M18</f>
-        <v>23514.7052</v>
+        <v>23128.8810363636</v>
       </c>
       <c r="S18" s="26" t="n">
         <f aca="false">R18/$P18/1000*100</f>
-        <v>0.630505907229338</v>
+        <v>0.620160703568245</v>
       </c>
       <c r="T18" s="26" t="n">
         <f aca="false">R18/P18</f>
-        <v>6.30505907229338</v>
+        <v>6.20160703568245</v>
       </c>
       <c r="U18" s="2" t="n">
         <f aca="false">3/5*H18+M18/3</f>
-        <v>7835.7772</v>
+        <v>7707.16914545455</v>
       </c>
       <c r="V18" s="26" t="n">
         <f aca="false">U18/$P18/1000*100</f>
-        <v>0.210102732324833</v>
+        <v>0.206654331104469</v>
       </c>
       <c r="W18" s="2" t="n">
         <f aca="false">R18-U18</f>
-        <v>15678.928</v>
+        <v>15421.7118909091</v>
       </c>
       <c r="X18" s="26" t="n">
         <f aca="false">W18/$P18/1000*100</f>
-        <v>0.420403174904505</v>
+        <v>0.413506372463776</v>
       </c>
       <c r="Y18" s="26"/>
       <c r="Z18" s="26"/>
@@ -5744,27 +5745,27 @@
       </c>
       <c r="AC18" s="2" t="n">
         <f aca="false">1000/100*Q18*($Q$41+$Q$47-$Q$49)-AA18</f>
-        <v>15413.7419684182</v>
+        <v>15072.203302131</v>
       </c>
       <c r="AD18" s="26" t="n">
         <f aca="false">AC18/$P18/1000*100</f>
-        <v>0.413292672858872</v>
+        <v>0.404134907757854</v>
       </c>
       <c r="AE18" s="2" t="n">
         <f aca="false">AC18+Q18/100*1000 *($Q$46+$Q$43)</f>
-        <v>26793.3999976231</v>
+        <v>26281.0919981924</v>
       </c>
       <c r="AF18" s="26" t="n">
         <f aca="false">AE18/$P18/1000*100</f>
-        <v>0.718418403699992</v>
+        <v>0.704681756048466</v>
       </c>
       <c r="AG18" s="26" t="n">
         <f aca="false">-AA18+($Q$45 + $Q$46)*1000*Q18/100</f>
-        <v>12852.2021342717</v>
+        <v>12510.6634679846</v>
       </c>
       <c r="AH18" s="26" t="n">
         <f aca="false">AG18/P18/10</f>
-        <v>0.344609438971993</v>
+        <v>0.335451673870976</v>
       </c>
       <c r="AI18" s="26" t="n">
         <f aca="false">ROUND(AG18/P18 *100/1000, 2)</f>
@@ -5912,13 +5913,13 @@
       <c r="L19" s="23" t="n">
         <v>2540</v>
       </c>
-      <c r="M19" s="23" t="n">
+      <c r="M19" s="26" t="n">
         <f aca="false">O19*$M$37/100</f>
-        <v>926.7804</v>
+        <v>884.654018181818</v>
       </c>
       <c r="N19" s="24" t="n">
         <f aca="false">M19/$P19/10</f>
-        <v>0.512370232362714</v>
+        <v>0.489080676346227</v>
       </c>
       <c r="O19" s="23" t="n">
         <v>6300</v>
@@ -5932,31 +5933,31 @@
       </c>
       <c r="R19" s="23" t="n">
         <f aca="false">H19+F19+B19+D19+J19+M19</f>
-        <v>1805.164</v>
+        <v>1763.03761818182</v>
       </c>
       <c r="S19" s="26" t="n">
         <f aca="false">R19/$P19/1000*100</f>
-        <v>0.997984310126547</v>
+        <v>0.97469475411006</v>
       </c>
       <c r="T19" s="26" t="n">
         <f aca="false">R19/P19</f>
-        <v>9.97984310126547</v>
+        <v>9.7469475411006</v>
       </c>
       <c r="U19" s="2" t="n">
         <f aca="false">3/5*H19+M19/3</f>
-        <v>379.7268</v>
+        <v>365.684672727273</v>
       </c>
       <c r="V19" s="26" t="n">
         <f aca="false">U19/$P19/1000*100</f>
-        <v>0.209931833636479</v>
+        <v>0.20216864829765</v>
       </c>
       <c r="W19" s="2" t="n">
         <f aca="false">R19-U19</f>
-        <v>1425.4372</v>
+        <v>1397.35294545455</v>
       </c>
       <c r="X19" s="26" t="n">
         <f aca="false">W19/$P19/1000*100</f>
-        <v>0.788052476490068</v>
+        <v>0.77252610581241</v>
       </c>
       <c r="Y19" s="26"/>
       <c r="Z19" s="30" t="n">
@@ -5973,31 +5974,31 @@
       </c>
       <c r="AC19" s="2" t="n">
         <f aca="false">1000/100*Q19*($Q$41+$Q$47-$Q$49)-AA19</f>
-        <v>724.867919593859</v>
+        <v>708.303262501488</v>
       </c>
       <c r="AD19" s="26" t="n">
         <f aca="false">AC19/$P19/1000*100</f>
-        <v>0.400742985495358</v>
+        <v>0.391585220394341</v>
       </c>
       <c r="AE19" s="2" t="n">
         <f aca="false">AC19+Q19/100*1000 *($Q$46+$Q$43)</f>
-        <v>1276.78239279659</v>
+        <v>1251.93540715803</v>
       </c>
       <c r="AF19" s="26" t="n">
         <f aca="false">AE19/$P19/1000*100</f>
-        <v>0.70586871633648</v>
+        <v>0.692132068684954</v>
       </c>
       <c r="AG19" s="26" t="n">
         <f aca="false">-Z19+($Q$45 + $Q$46)*1000*Q19/100</f>
-        <v>600.632999306933</v>
+        <v>584.068342214562</v>
       </c>
       <c r="AH19" s="26" t="n">
         <f aca="false">AG19/P19/10</f>
-        <v>0.332059751608479</v>
+        <v>0.322901986507462</v>
       </c>
       <c r="AI19" s="26" t="n">
         <f aca="false">ROUND(AG19/P19 *100/1000, 2)</f>
-        <v>0.33</v>
+        <v>0.32</v>
       </c>
       <c r="AK19" s="26" t="n">
         <f aca="false">-Q19*($Q$47)*10</f>
@@ -6141,13 +6142,13 @@
       <c r="L20" s="23" t="n">
         <v>370</v>
       </c>
-      <c r="M20" s="23" t="n">
+      <c r="M20" s="26" t="n">
         <f aca="false">O20*$M$37/100</f>
-        <v>367.77</v>
+        <v>351.053181818182</v>
       </c>
       <c r="N20" s="24" t="n">
         <f aca="false">M20/$P20/10</f>
-        <v>0.246951465176869</v>
+        <v>0.23572639857792</v>
       </c>
       <c r="O20" s="23" t="n">
         <v>2500</v>
@@ -6161,31 +6162,31 @@
       </c>
       <c r="R20" s="23" t="n">
         <f aca="false">H20+F20+B20+D20+J20+M20</f>
-        <v>921.0058</v>
+        <v>904.288981818182</v>
       </c>
       <c r="S20" s="26" t="n">
         <f aca="false">R20/$P20/1000*100</f>
-        <v>0.61844014396605</v>
+        <v>0.607215077367101</v>
       </c>
       <c r="T20" s="26" t="n">
         <f aca="false">R20/P20</f>
-        <v>6.1844014396605</v>
+        <v>6.07215077367101</v>
       </c>
       <c r="U20" s="2" t="n">
         <f aca="false">3/5*H20+M20/3</f>
-        <v>247.39</v>
+        <v>241.817727272727</v>
       </c>
       <c r="V20" s="26" t="n">
         <f aca="false">U20/$P20/1000*100</f>
-        <v>0.166118288523005</v>
+        <v>0.162376599656689</v>
       </c>
       <c r="W20" s="2" t="n">
         <f aca="false">R20-U20</f>
-        <v>673.6158</v>
+        <v>662.471254545455</v>
       </c>
       <c r="X20" s="26" t="n">
         <f aca="false">W20/$P20/1000*100</f>
-        <v>0.452321855443045</v>
+        <v>0.444838477710412</v>
       </c>
       <c r="Y20" s="26"/>
       <c r="Z20" s="26"/>
@@ -6199,27 +6200,27 @@
       </c>
       <c r="AC20" s="2" t="n">
         <f aca="false">1000/100*Q20*($Q$41+$Q$47-$Q$49)-AA20</f>
-        <v>615.491980128349</v>
+        <v>601.85387002931</v>
       </c>
       <c r="AD20" s="26" t="n">
         <f aca="false">AC20/$P20/1000*100</f>
-        <v>0.413292672858874</v>
+        <v>0.404134907757856</v>
       </c>
       <c r="AE20" s="2" t="n">
         <f aca="false">AC20+Q20/100*1000 *($Q$46+$Q$43)</f>
-        <v>1069.89742352618</v>
+        <v>1049.44025837762</v>
       </c>
       <c r="AF20" s="26" t="n">
         <f aca="false">AE20/$P20/1000*100</f>
-        <v>0.718418403699996</v>
+        <v>0.70468175604847</v>
       </c>
       <c r="AG20" s="26" t="n">
         <f aca="false">-AA20+($Q$45 + $Q$46)*1000*Q20/100</f>
-        <v>513.206160894653</v>
+        <v>499.568050795614</v>
       </c>
       <c r="AH20" s="26" t="n">
         <f aca="false">AG20/P20/10</f>
-        <v>0.344609438971994</v>
+        <v>0.335451673870977</v>
       </c>
       <c r="AI20" s="26" t="n">
         <f aca="false">ROUND(AG20/P20 *100/1000, 2)</f>
@@ -6367,13 +6368,13 @@
       <c r="L21" s="23" t="n">
         <v>940</v>
       </c>
-      <c r="M21" s="23" t="n">
+      <c r="M21" s="26" t="n">
         <f aca="false">O21*$M$37/100</f>
-        <v>559.0104</v>
+        <v>533.600836363636</v>
       </c>
       <c r="N21" s="24" t="n">
         <f aca="false">M21/$P21/10</f>
-        <v>0.172810891520677</v>
+        <v>0.16495585099701</v>
       </c>
       <c r="O21" s="23" t="n">
         <v>3800</v>
@@ -6387,31 +6388,31 @@
       </c>
       <c r="R21" s="23" t="n">
         <f aca="false">H21+F21+B21+D21+J21+M21</f>
-        <v>1607.75</v>
+        <v>1582.34043636364</v>
       </c>
       <c r="S21" s="26" t="n">
         <f aca="false">R21/$P21/1000*100</f>
-        <v>0.497015280650177</v>
+        <v>0.48916024012651</v>
       </c>
       <c r="T21" s="26" t="n">
         <f aca="false">R21/P21</f>
-        <v>4.97015280650177</v>
+        <v>4.8916024012651</v>
       </c>
       <c r="U21" s="2" t="n">
         <f aca="false">3/5*H21+M21/3</f>
-        <v>384.9368</v>
+        <v>376.466945454545</v>
       </c>
       <c r="V21" s="26" t="n">
         <f aca="false">U21/$P21/1000*100</f>
-        <v>0.118998271923235</v>
+        <v>0.116379925082013</v>
       </c>
       <c r="W21" s="2" t="n">
         <f aca="false">R21-U21</f>
-        <v>1222.8132</v>
+        <v>1205.87349090909</v>
       </c>
       <c r="X21" s="26" t="n">
         <f aca="false">W21/$P21/1000*100</f>
-        <v>0.378017008726942</v>
+        <v>0.372780315044498</v>
       </c>
       <c r="Y21" s="26"/>
       <c r="Z21" s="30" t="n">
@@ -6428,31 +6429,31 @@
       </c>
       <c r="AC21" s="2" t="n">
         <f aca="false">1000/100*Q21*($Q$41+$Q$47-$Q$49)-AA21</f>
-        <v>1095.52327109061</v>
+        <v>1065.89964096419</v>
       </c>
       <c r="AD21" s="26" t="n">
         <f aca="false">AC21/$P21/1000*100</f>
-        <v>0.338666960684123</v>
+        <v>0.329509195583106</v>
       </c>
       <c r="AE21" s="2" t="n">
         <f aca="false">AC21+Q21/100*1000 *($Q$46+$Q$43)</f>
-        <v>2082.54703647278</v>
+        <v>2038.11159128314</v>
       </c>
       <c r="AF21" s="26" t="n">
         <f aca="false">AE21/$P21/1000*100</f>
-        <v>0.643792691525244</v>
+        <v>0.630056043873718</v>
       </c>
       <c r="AG21" s="26" t="n">
         <f aca="false">-Z21+($Q$45 + $Q$46)*1000*Q21/100</f>
-        <v>873.346059280994</v>
+        <v>843.722429154572</v>
       </c>
       <c r="AH21" s="26" t="n">
         <f aca="false">AG21/P21/10</f>
-        <v>0.269983726797244</v>
+        <v>0.260825961696227</v>
       </c>
       <c r="AI21" s="26" t="n">
         <f aca="false">ROUND(AG21/P21 *100/1000, 2)</f>
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="AK21" s="26" t="n">
         <f aca="false">-Q21*($Q$47)*10</f>
@@ -6599,13 +6600,13 @@
       <c r="L22" s="23" t="n">
         <v>7110</v>
       </c>
-      <c r="M22" s="23" t="n">
+      <c r="M22" s="26" t="n">
         <f aca="false">O22*$M$37/100</f>
-        <v>8311.602</v>
+        <v>7933.80190909091</v>
       </c>
       <c r="N22" s="24" t="n">
         <f aca="false">M22/$P22/10</f>
-        <v>0.458197003274568</v>
+        <v>0.437369866762087</v>
       </c>
       <c r="O22" s="23" t="n">
         <v>56500</v>
@@ -6619,31 +6620,31 @@
       </c>
       <c r="R22" s="23" t="n">
         <f aca="false">H22+F22+B22+D22+J22+M22</f>
-        <v>14491.1494</v>
+        <v>14113.3493090909</v>
       </c>
       <c r="S22" s="26" t="n">
         <f aca="false">R22/$P22/1000*100</f>
-        <v>0.798859381029559</v>
+        <v>0.778032244517079</v>
       </c>
       <c r="T22" s="26" t="n">
         <f aca="false">R22/P22</f>
-        <v>7.98859381029559</v>
+        <v>7.78032244517079</v>
       </c>
       <c r="U22" s="2" t="n">
         <f aca="false">3/5*H22+M22/3</f>
-        <v>4341.334</v>
+        <v>4215.40063636364</v>
       </c>
       <c r="V22" s="26" t="n">
         <f aca="false">U22/$P22/1000*100</f>
-        <v>0.239326453433886</v>
+        <v>0.232384074596392</v>
       </c>
       <c r="W22" s="2" t="n">
         <f aca="false">R22-U22</f>
-        <v>10149.8154</v>
+        <v>9897.94867272727</v>
       </c>
       <c r="X22" s="26" t="n">
         <f aca="false">W22/$P22/1000*100</f>
-        <v>0.559532927595674</v>
+        <v>0.545648169920687</v>
       </c>
       <c r="Y22" s="26" t="n">
         <f aca="false">B22</f>
@@ -6663,31 +6664,31 @@
       </c>
       <c r="AC22" s="2" t="n">
         <f aca="false">1000/100*Q22*($Q$41+$Q$47-$Q$49)-AA22</f>
-        <v>6485.54642712539</v>
+        <v>6319.42639974595</v>
       </c>
       <c r="AD22" s="26" t="n">
         <f aca="false">AC22/$P22/1000*100</f>
-        <v>0.357531308345483</v>
+        <v>0.348373543244465</v>
       </c>
       <c r="AE22" s="2" t="n">
         <f aca="false">AC22+Q22/100*1000 *($Q$46+$Q$43)</f>
-        <v>12020.4661594372</v>
+        <v>11771.286118368</v>
       </c>
       <c r="AF22" s="26" t="n">
         <f aca="false">AE22/$P22/1000*100</f>
-        <v>0.662657039186604</v>
+        <v>0.648920391535078</v>
       </c>
       <c r="AG22" s="26" t="n">
         <f aca="false">-AA22+($Q$45 + $Q$46)*1000*Q22/100</f>
-        <v>5239.64630106418</v>
+        <v>5073.52627368474</v>
       </c>
       <c r="AH22" s="26" t="n">
         <f aca="false">AG22/P22/10</f>
-        <v>0.288848074458604</v>
+        <v>0.279690309357586</v>
       </c>
       <c r="AI22" s="26" t="n">
         <f aca="false">ROUND(AG22/P22 *100/1000, 2)</f>
-        <v>0.29</v>
+        <v>0.28</v>
       </c>
       <c r="AK22" s="26" t="n">
         <f aca="false">-Q22*($Q$47)*10</f>
@@ -6831,13 +6832,13 @@
       <c r="L23" s="23" t="n">
         <v>180</v>
       </c>
-      <c r="M23" s="23" t="n">
+      <c r="M23" s="26" t="n">
         <f aca="false">O23*$M$37/100</f>
-        <v>73.554</v>
+        <v>70.2106363636364</v>
       </c>
       <c r="N23" s="24" t="n">
         <f aca="false">M23/$P23/10</f>
-        <v>0.222385487528345</v>
+        <v>0.212277056277056</v>
       </c>
       <c r="O23" s="23" t="n">
         <v>500</v>
@@ -6851,31 +6852,31 @@
       </c>
       <c r="R23" s="23" t="n">
         <f aca="false">H23+F23+B23+D23+J23+M23</f>
-        <v>182.5552</v>
+        <v>179.211836363636</v>
       </c>
       <c r="S23" s="26" t="n">
         <f aca="false">R23/$P23/1000*100</f>
-        <v>0.551943159486017</v>
+        <v>0.541834728234728</v>
       </c>
       <c r="T23" s="26" t="n">
         <f aca="false">R23/P23</f>
-        <v>5.51943159486017</v>
+        <v>5.41834728234728</v>
       </c>
       <c r="U23" s="2" t="n">
         <f aca="false">3/5*H23+M23/3</f>
-        <v>36.518</v>
+        <v>35.4035454545455</v>
       </c>
       <c r="V23" s="26" t="n">
         <f aca="false">U23/$P23/1000*100</f>
-        <v>0.110409674981104</v>
+        <v>0.107040197897341</v>
       </c>
       <c r="W23" s="2" t="n">
         <f aca="false">R23-U23</f>
-        <v>146.0372</v>
+        <v>143.808290909091</v>
       </c>
       <c r="X23" s="26" t="n">
         <f aca="false">W23/$P23/1000*100</f>
-        <v>0.441533484504913</v>
+        <v>0.434794530337387</v>
       </c>
       <c r="Y23" s="26"/>
       <c r="Z23" s="26"/>
@@ -6889,27 +6890,27 @@
       </c>
       <c r="AC23" s="2" t="n">
         <f aca="false">1000/100*Q23*($Q$41+$Q$47-$Q$49)-AA23</f>
-        <v>136.696551548072</v>
+        <v>133.66762074091</v>
       </c>
       <c r="AD23" s="26" t="n">
         <f aca="false">AC23/$P23/1000*100</f>
-        <v>0.413292672858872</v>
+        <v>0.404134907757855</v>
       </c>
       <c r="AE23" s="2" t="n">
         <f aca="false">AC23+Q23/100*1000 *($Q$46+$Q$43)</f>
-        <v>237.616887023773</v>
+        <v>233.07349081303</v>
       </c>
       <c r="AF23" s="26" t="n">
         <f aca="false">AE23/$P23/1000*100</f>
-        <v>0.718418403699992</v>
+        <v>0.704681756048466</v>
       </c>
       <c r="AG23" s="26" t="n">
         <f aca="false">-AA23+($Q$45 + $Q$46)*1000*Q23/100</f>
-        <v>113.979571939987</v>
+        <v>110.950641132825</v>
       </c>
       <c r="AH23" s="26" t="n">
         <f aca="false">AG23/P23/10</f>
-        <v>0.344609438971993</v>
+        <v>0.335451673870976</v>
       </c>
       <c r="AI23" s="26" t="n">
         <f aca="false">ROUND(AG23/P23 *100/1000, 2)</f>
@@ -7057,13 +7058,13 @@
       <c r="L24" s="23" t="n">
         <v>140</v>
       </c>
-      <c r="M24" s="23" t="n">
+      <c r="M24" s="26" t="n">
         <f aca="false">O24*$M$37/100</f>
-        <v>117.6864</v>
+        <v>112.337018181818</v>
       </c>
       <c r="N24" s="24" t="n">
         <f aca="false">M24/$P24/10</f>
-        <v>0.217873222748815</v>
+        <v>0.207969894442051</v>
       </c>
       <c r="O24" s="23" t="n">
         <v>800</v>
@@ -7077,31 +7078,31 @@
       </c>
       <c r="R24" s="23" t="n">
         <f aca="false">H24+F24+B24+D24+J24+M24</f>
-        <v>246.454</v>
+        <v>241.104618181818</v>
       </c>
       <c r="S24" s="26" t="n">
         <f aca="false">R24/$P24/1000*100</f>
-        <v>0.456261107819905</v>
+        <v>0.446357779513141</v>
       </c>
       <c r="T24" s="26" t="n">
         <f aca="false">R24/P24</f>
-        <v>4.56261107819905</v>
+        <v>4.46357779513141</v>
       </c>
       <c r="U24" s="2" t="n">
         <f aca="false">3/5*H24+M24/3</f>
-        <v>57.8288</v>
+        <v>56.0456727272727</v>
       </c>
       <c r="V24" s="26" t="n">
         <f aca="false">U24/$P24/1000*100</f>
-        <v>0.1070586492891</v>
+        <v>0.103757539853511</v>
       </c>
       <c r="W24" s="2" t="n">
         <f aca="false">R24-U24</f>
-        <v>188.6252</v>
+        <v>185.058945454545</v>
       </c>
       <c r="X24" s="26" t="n">
         <f aca="false">W24/$P24/1000*100</f>
-        <v>0.349202458530806</v>
+        <v>0.342600239659629</v>
       </c>
       <c r="Y24" s="26"/>
       <c r="Z24" s="26"/>
@@ -7115,27 +7116,27 @@
       </c>
       <c r="AC24" s="2" t="n">
         <f aca="false">1000/100*Q24*($Q$41+$Q$47-$Q$49)-AA24</f>
-        <v>223.244170171449</v>
+        <v>218.297511774483</v>
       </c>
       <c r="AD24" s="26" t="n">
         <f aca="false">AC24/$P24/1000*100</f>
-        <v>0.413292672858873</v>
+        <v>0.404134907757855</v>
       </c>
       <c r="AE24" s="2" t="n">
         <f aca="false">AC24+Q24/100*1000 *($Q$46+$Q$43)</f>
-        <v>388.060884942589</v>
+        <v>380.640897347141</v>
       </c>
       <c r="AF24" s="26" t="n">
         <f aca="false">AE24/$P24/1000*100</f>
-        <v>0.718418403699994</v>
+        <v>0.704681756048468</v>
       </c>
       <c r="AG24" s="26" t="n">
         <f aca="false">-AA24+($Q$45 + $Q$46)*1000*Q24/100</f>
-        <v>186.144234555112</v>
+        <v>181.197576158147</v>
       </c>
       <c r="AH24" s="26" t="n">
         <f aca="false">AG24/P24/10</f>
-        <v>0.344609438971994</v>
+        <v>0.335451673870976</v>
       </c>
       <c r="AI24" s="26" t="n">
         <f aca="false">ROUND(AG24/P24 *100/1000, 2)</f>
@@ -7283,13 +7284,13 @@
       <c r="L25" s="23" t="n">
         <v>210</v>
       </c>
-      <c r="M25" s="23" t="n">
+      <c r="M25" s="26" t="n">
         <f aca="false">O25*$M$37/100</f>
-        <v>264.7944</v>
+        <v>252.758290909091</v>
       </c>
       <c r="N25" s="24" t="n">
         <f aca="false">M25/$P25/10</f>
-        <v>0.524657023974638</v>
+        <v>0.500808977430337</v>
       </c>
       <c r="O25" s="23" t="n">
         <v>1800</v>
@@ -7303,31 +7304,31 @@
       </c>
       <c r="R25" s="23" t="n">
         <f aca="false">H25+F25+B25+D25+J25+M25</f>
-        <v>563.7958</v>
+        <v>551.759690909091</v>
       </c>
       <c r="S25" s="26" t="n">
         <f aca="false">R25/$P25/1000*100</f>
-        <v>1.11709094511591</v>
+        <v>1.09324289857161</v>
       </c>
       <c r="T25" s="26" t="n">
         <f aca="false">R25/P25</f>
-        <v>11.1709094511591</v>
+        <v>10.9324289857161</v>
       </c>
       <c r="U25" s="2" t="n">
         <f aca="false">3/5*H25+M25/3</f>
-        <v>213.0648</v>
+        <v>209.052763636364</v>
       </c>
       <c r="V25" s="26" t="n">
         <f aca="false">U25/$P25/1000*100</f>
-        <v>0.422161283931048</v>
+        <v>0.414211935082948</v>
       </c>
       <c r="W25" s="2" t="n">
         <f aca="false">R25-U25</f>
-        <v>350.731</v>
+        <v>342.706927272727</v>
       </c>
       <c r="X25" s="26" t="n">
         <f aca="false">W25/$P25/1000*100</f>
-        <v>0.694929661184862</v>
+        <v>0.679030963488661</v>
       </c>
       <c r="Y25" s="26"/>
       <c r="Z25" s="26"/>
@@ -7341,27 +7342,27 @@
       </c>
       <c r="AC25" s="2" t="n">
         <f aca="false">1000/100*Q25*($Q$41+$Q$47-$Q$49)-AA25</f>
-        <v>208.588811991873</v>
+        <v>203.966887945389</v>
       </c>
       <c r="AD25" s="26" t="n">
         <f aca="false">AC25/$P25/1000*100</f>
-        <v>0.413292672858872</v>
+        <v>0.404134907757855</v>
       </c>
       <c r="AE25" s="2" t="n">
         <f aca="false">AC25+Q25/100*1000 *($Q$46+$Q$43)</f>
-        <v>362.585768347386</v>
+        <v>355.652882277661</v>
       </c>
       <c r="AF25" s="26" t="n">
         <f aca="false">AE25/$P25/1000*100</f>
-        <v>0.718418403699993</v>
+        <v>0.704681756048467</v>
       </c>
       <c r="AG25" s="26" t="n">
         <f aca="false">-AA25+($Q$45 + $Q$46)*1000*Q25/100</f>
-        <v>173.924383849165</v>
+        <v>169.302459802681</v>
       </c>
       <c r="AH25" s="26" t="n">
         <f aca="false">AG25/P25/10</f>
-        <v>0.344609438971993</v>
+        <v>0.335451673870976</v>
       </c>
       <c r="AI25" s="26" t="n">
         <f aca="false">ROUND(AG25/P25 *100/1000, 2)</f>
@@ -7509,13 +7510,13 @@
       <c r="L26" s="23" t="n">
         <v>270</v>
       </c>
-      <c r="M26" s="23" t="n">
+      <c r="M26" s="26" t="n">
         <f aca="false">O26*$M$37/100</f>
-        <v>132.3972</v>
+        <v>126.379145454545</v>
       </c>
       <c r="N26" s="24" t="n">
         <f aca="false">M26/$P26/10</f>
-        <v>0.965627598278754</v>
+        <v>0.921735434720629</v>
       </c>
       <c r="O26" s="23" t="n">
         <v>900</v>
@@ -7529,31 +7530,31 @@
       </c>
       <c r="R26" s="23" t="n">
         <f aca="false">H26+F26+B26+D26+J26+M26</f>
-        <v>221.399</v>
+        <v>215.380945454545</v>
       </c>
       <c r="S26" s="26" t="n">
         <f aca="false">R26/$P26/1000*100</f>
-        <v>1.61475457661731</v>
+        <v>1.57086241305919</v>
       </c>
       <c r="T26" s="26" t="n">
         <f aca="false">R26/P26</f>
-        <v>16.1475457661731</v>
+        <v>15.7086241305919</v>
       </c>
       <c r="U26" s="2" t="n">
         <f aca="false">3/5*H26+M26/3</f>
-        <v>49.5324</v>
+        <v>47.5263818181818</v>
       </c>
       <c r="V26" s="26" t="n">
         <f aca="false">U26/$P26/1000*100</f>
-        <v>0.361260301947342</v>
+        <v>0.3466295807613</v>
       </c>
       <c r="W26" s="2" t="n">
         <f aca="false">R26-U26</f>
-        <v>171.8666</v>
+        <v>167.854563636364</v>
       </c>
       <c r="X26" s="26" t="n">
         <f aca="false">W26/$P26/1000*100</f>
-        <v>1.25349427466997</v>
+        <v>1.22423283229789</v>
       </c>
       <c r="Y26" s="26"/>
       <c r="Z26" s="26"/>
@@ -7567,27 +7568,27 @@
       </c>
       <c r="AC26" s="2" t="n">
         <f aca="false">1000/100*Q26*($Q$41+$Q$47-$Q$49)-AA26</f>
-        <v>56.66655837568</v>
+        <v>55.4109372026795</v>
       </c>
       <c r="AD26" s="26" t="n">
         <f aca="false">AC26/$P26/1000*100</f>
-        <v>0.413292672858872</v>
+        <v>0.404134907757855</v>
       </c>
       <c r="AE26" s="2" t="n">
         <f aca="false">AC26+Q26/100*1000 *($Q$46+$Q$43)</f>
-        <v>98.5023473313061</v>
+        <v>96.6189155718054</v>
       </c>
       <c r="AF26" s="26" t="n">
         <f aca="false">AE26/$P26/1000*100</f>
-        <v>0.718418403699994</v>
+        <v>0.704681756048467</v>
       </c>
       <c r="AG26" s="26" t="n">
         <f aca="false">-AA26+($Q$45 + $Q$46)*1000*Q26/100</f>
-        <v>47.24940017745</v>
+        <v>45.9937790044495</v>
       </c>
       <c r="AH26" s="26" t="n">
         <f aca="false">AG26/P26/10</f>
-        <v>0.344609438971993</v>
+        <v>0.335451673870976</v>
       </c>
       <c r="AI26" s="26" t="n">
         <f aca="false">ROUND(AG26/P26 *100/1000, 2)</f>
@@ -7735,13 +7736,13 @@
       <c r="L27" s="23" t="n">
         <v>1980</v>
       </c>
-      <c r="M27" s="23" t="n">
+      <c r="M27" s="26" t="n">
         <f aca="false">O27*$M$37/100</f>
-        <v>1618.188</v>
+        <v>1544.634</v>
       </c>
       <c r="N27" s="24" t="n">
         <f aca="false">M27/$P27/10</f>
-        <v>0.193295873170592</v>
+        <v>0.184509697117383</v>
       </c>
       <c r="O27" s="23" t="n">
         <v>11000</v>
@@ -7755,31 +7756,31 @@
       </c>
       <c r="R27" s="23" t="n">
         <f aca="false">H27+F27+B27+D27+J27+M27</f>
-        <v>5939.2012</v>
+        <v>5865.6472</v>
       </c>
       <c r="S27" s="26" t="n">
         <f aca="false">R27/$P27/1000*100</f>
-        <v>0.709449756078915</v>
+        <v>0.700663580025706</v>
       </c>
       <c r="T27" s="26" t="n">
         <f aca="false">R27/P27</f>
-        <v>7.09449756078915</v>
+        <v>7.00663580025706</v>
       </c>
       <c r="U27" s="2" t="n">
         <f aca="false">3/5*H27+M27/3</f>
-        <v>1087.196</v>
+        <v>1062.678</v>
       </c>
       <c r="V27" s="26" t="n">
         <f aca="false">U27/$P27/1000*100</f>
-        <v>0.129867790471549</v>
+        <v>0.126939065120479</v>
       </c>
       <c r="W27" s="2" t="n">
         <f aca="false">R27-U27</f>
-        <v>4852.0052</v>
+        <v>4802.9692</v>
       </c>
       <c r="X27" s="26" t="n">
         <f aca="false">W27/$P27/1000*100</f>
-        <v>0.579581965607366</v>
+        <v>0.573724514905227</v>
       </c>
       <c r="Y27" s="26"/>
       <c r="Z27" s="26"/>
@@ -7793,27 +7794,27 @@
       </c>
       <c r="AC27" s="2" t="n">
         <f aca="false">1000/100*Q27*($Q$41+$Q$47-$Q$49)-AA27</f>
-        <v>3459.90440839842</v>
+        <v>3383.23962838935</v>
       </c>
       <c r="AD27" s="26" t="n">
         <f aca="false">AC27/$P27/1000*100</f>
-        <v>0.413292672858873</v>
+        <v>0.404134907757855</v>
       </c>
       <c r="AE27" s="2" t="n">
         <f aca="false">AC27+Q27/100*1000 *($Q$46+$Q$43)</f>
-        <v>6014.28277167872</v>
+        <v>5899.28560166511</v>
       </c>
       <c r="AF27" s="26" t="n">
         <f aca="false">AE27/$P27/1000*100</f>
-        <v>0.718418403699994</v>
+        <v>0.704681756048468</v>
       </c>
       <c r="AG27" s="26" t="n">
         <f aca="false">-AA27+($Q$45 + $Q$46)*1000*Q27/100</f>
-        <v>2884.91859492038</v>
+        <v>2808.25381491131</v>
       </c>
       <c r="AH27" s="26" t="n">
         <f aca="false">AG27/P27/10</f>
-        <v>0.344609438971994</v>
+        <v>0.335451673870976</v>
       </c>
       <c r="AI27" s="26" t="n">
         <f aca="false">ROUND(AG27/P27 *100/1000, 2)</f>
@@ -7961,13 +7962,13 @@
       <c r="L28" s="23" t="n">
         <v>1190</v>
       </c>
-      <c r="M28" s="23" t="n">
+      <c r="M28" s="26" t="n">
         <f aca="false">O28*$M$37/100</f>
-        <v>1176.864</v>
+        <v>1123.37018181818</v>
       </c>
       <c r="N28" s="24" t="n">
         <f aca="false">M28/$P28/10</f>
-        <v>0.214791088333689</v>
+        <v>0.205027857045794</v>
       </c>
       <c r="O28" s="23" t="n">
         <v>8000</v>
@@ -7981,31 +7982,31 @@
       </c>
       <c r="R28" s="23" t="n">
         <f aca="false">H28+F28+B28+D28+J28+M28</f>
-        <v>3001.5386</v>
+        <v>2948.04478181818</v>
       </c>
       <c r="S28" s="26" t="n">
         <f aca="false">R28/$P28/1000*100</f>
-        <v>0.547814991850866</v>
+        <v>0.538051760562971</v>
       </c>
       <c r="T28" s="26" t="n">
         <f aca="false">R28/P28</f>
-        <v>5.47814991850866</v>
+        <v>5.38051760562971</v>
       </c>
       <c r="U28" s="2" t="n">
         <f aca="false">3/5*H28+M28/3</f>
-        <v>728.288</v>
+        <v>710.456727272727</v>
       </c>
       <c r="V28" s="26" t="n">
         <f aca="false">U28/$P28/1000*100</f>
-        <v>0.132920857584535</v>
+        <v>0.129666447155236</v>
       </c>
       <c r="W28" s="2" t="n">
         <f aca="false">R28-U28</f>
-        <v>2273.2506</v>
+        <v>2237.58805454545</v>
       </c>
       <c r="X28" s="26" t="n">
         <f aca="false">W28/$P28/1000*100</f>
-        <v>0.414894134266332</v>
+        <v>0.408385313407735</v>
       </c>
       <c r="Y28" s="26"/>
       <c r="Z28" s="26"/>
@@ -8019,27 +8020,27 @@
       </c>
       <c r="AC28" s="2" t="n">
         <f aca="false">1000/100*Q28*($Q$41+$Q$47-$Q$49)-AA28</f>
-        <v>2264.47601678777</v>
+        <v>2214.29961444514</v>
       </c>
       <c r="AD28" s="26" t="n">
         <f aca="false">AC28/$P28/1000*100</f>
-        <v>0.413292672858872</v>
+        <v>0.404134907757855</v>
       </c>
       <c r="AE28" s="2" t="n">
         <f aca="false">AC28+Q28/100*1000 *($Q$46+$Q$43)</f>
-        <v>3936.29345989667</v>
+        <v>3861.02885638271</v>
       </c>
       <c r="AF28" s="26" t="n">
         <f aca="false">AE28/$P28/1000*100</f>
-        <v>0.718418403699992</v>
+        <v>0.704681756048466</v>
       </c>
       <c r="AG28" s="26" t="n">
         <f aca="false">-AA28+($Q$45 + $Q$46)*1000*Q28/100</f>
-        <v>1888.15302316584</v>
+        <v>1837.9766208232</v>
       </c>
       <c r="AH28" s="26" t="n">
         <f aca="false">AG28/P28/10</f>
-        <v>0.344609438971993</v>
+        <v>0.335451673870976</v>
       </c>
       <c r="AI28" s="26" t="n">
         <f aca="false">ROUND(AG28/P28 *100/1000, 2)</f>
@@ -8187,13 +8188,13 @@
       <c r="L29" s="23" t="n">
         <v>1950</v>
       </c>
-      <c r="M29" s="23" t="n">
+      <c r="M29" s="26" t="n">
         <f aca="false">O29*$M$37/100</f>
-        <v>941.4912</v>
+        <v>898.696145454545</v>
       </c>
       <c r="N29" s="24" t="n">
         <f aca="false">M29/$P29/10</f>
-        <v>0.444361628318584</v>
+        <v>0.424163372485921</v>
       </c>
       <c r="O29" s="23" t="n">
         <v>6400</v>
@@ -8207,31 +8208,31 @@
       </c>
       <c r="R29" s="23" t="n">
         <f aca="false">H29+F29+B29+D29+J29+M29</f>
-        <v>1972.4042</v>
+        <v>1929.60914545455</v>
       </c>
       <c r="S29" s="26" t="n">
         <f aca="false">R29/$P29/1000*100</f>
-        <v>0.930928235988201</v>
+        <v>0.910729980155538</v>
       </c>
       <c r="T29" s="26" t="n">
         <f aca="false">R29/P29</f>
-        <v>9.30928235988201</v>
+        <v>9.10729980155538</v>
       </c>
       <c r="U29" s="2" t="n">
         <f aca="false">3/5*H29+M29/3</f>
-        <v>511.8304</v>
+        <v>497.565381818182</v>
       </c>
       <c r="V29" s="26" t="n">
         <f aca="false">U29/$P29/1000*100</f>
-        <v>0.24157187020649</v>
+        <v>0.234839118262269</v>
       </c>
       <c r="W29" s="2" t="n">
         <f aca="false">R29-U29</f>
-        <v>1460.5738</v>
+        <v>1432.04376363636</v>
       </c>
       <c r="X29" s="26" t="n">
         <f aca="false">W29/$P29/1000*100</f>
-        <v>0.689356365781711</v>
+        <v>0.675890861893269</v>
       </c>
       <c r="Y29" s="26"/>
       <c r="Z29" s="26"/>
@@ -8245,27 +8246,27 @@
       </c>
       <c r="AC29" s="2" t="n">
         <f aca="false">1000/100*Q29*($Q$41+$Q$47-$Q$49)-AA29</f>
-        <v>875.663850619736</v>
+        <v>856.260835811956</v>
       </c>
       <c r="AD29" s="26" t="n">
         <f aca="false">AC29/$P29/1000*100</f>
-        <v>0.413292672858873</v>
+        <v>0.404134907757855</v>
       </c>
       <c r="AE29" s="2" t="n">
         <f aca="false">AC29+Q29/100*1000 *($Q$46+$Q$43)</f>
-        <v>1522.14899283936</v>
+        <v>1493.04447062769</v>
       </c>
       <c r="AF29" s="26" t="n">
         <f aca="false">AE29/$P29/1000*100</f>
-        <v>0.718418403699994</v>
+        <v>0.704681756048468</v>
       </c>
       <c r="AG29" s="26" t="n">
         <f aca="false">-AA29+($Q$45 + $Q$46)*1000*Q29/100</f>
-        <v>730.141248821911</v>
+        <v>710.738234014131</v>
       </c>
       <c r="AH29" s="26" t="n">
         <f aca="false">AG29/P29/10</f>
-        <v>0.344609438971994</v>
+        <v>0.335451673870976</v>
       </c>
       <c r="AI29" s="26" t="n">
         <f aca="false">ROUND(AG29/P29 *100/1000, 2)</f>
@@ -8413,13 +8414,13 @@
       <c r="L30" s="23" t="n">
         <v>620</v>
       </c>
-      <c r="M30" s="23" t="n">
+      <c r="M30" s="26" t="n">
         <f aca="false">O30*$M$37/100</f>
-        <v>470.7456</v>
+        <v>449.348072727273</v>
       </c>
       <c r="N30" s="24" t="n">
         <f aca="false">M30/$P30/10</f>
-        <v>0.218634168090956</v>
+        <v>0.208696251359549</v>
       </c>
       <c r="O30" s="23" t="n">
         <v>3200</v>
@@ -8433,31 +8434,31 @@
       </c>
       <c r="R30" s="23" t="n">
         <f aca="false">H30+F30+B30+D30+J30+M30</f>
-        <v>903.3164</v>
+        <v>881.918872727273</v>
       </c>
       <c r="S30" s="26" t="n">
         <f aca="false">R30/$P30/1000*100</f>
-        <v>0.419538344356097</v>
+        <v>0.40960042762469</v>
       </c>
       <c r="T30" s="26" t="n">
         <f aca="false">R30/P30</f>
-        <v>4.19538344356097</v>
+        <v>4.0960042762469</v>
       </c>
       <c r="U30" s="2" t="n">
         <f aca="false">3/5*H30+M30/3</f>
-        <v>229.5152</v>
+        <v>222.382690909091</v>
       </c>
       <c r="V30" s="26" t="n">
         <f aca="false">U30/$P30/1000*100</f>
-        <v>0.106596566842535</v>
+        <v>0.103283927932066</v>
       </c>
       <c r="W30" s="2" t="n">
         <f aca="false">R30-U30</f>
-        <v>673.8012</v>
+        <v>659.536181818182</v>
       </c>
       <c r="X30" s="26" t="n">
         <f aca="false">W30/$P30/1000*100</f>
-        <v>0.312941777513562</v>
+        <v>0.306316499692624</v>
       </c>
       <c r="Y30" s="26"/>
       <c r="Z30" s="26"/>
@@ -8471,27 +8472,27 @@
       </c>
       <c r="AC30" s="2" t="n">
         <f aca="false">1000/100*Q30*($Q$41+$Q$47-$Q$49)-AA30</f>
-        <v>889.868719785896</v>
+        <v>870.150952591593</v>
       </c>
       <c r="AD30" s="26" t="n">
         <f aca="false">AC30/$P30/1000*100</f>
-        <v>0.413292672858873</v>
+        <v>0.404134907757855</v>
       </c>
       <c r="AE30" s="2" t="n">
         <f aca="false">AC30+Q30/100*1000 *($Q$46+$Q$43)</f>
-        <v>1546.84103337453</v>
+        <v>1517.26438258308</v>
       </c>
       <c r="AF30" s="26" t="n">
         <f aca="false">AE30/$P30/1000*100</f>
-        <v>0.718418403699994</v>
+        <v>0.704681756048468</v>
       </c>
       <c r="AG30" s="26" t="n">
         <f aca="false">-AA30+($Q$45 + $Q$46)*1000*Q30/100</f>
-        <v>741.985475239379</v>
+        <v>722.267708045077</v>
       </c>
       <c r="AH30" s="26" t="n">
         <f aca="false">AG30/P30/10</f>
-        <v>0.344609438971994</v>
+        <v>0.335451673870976</v>
       </c>
       <c r="AI30" s="26" t="n">
         <f aca="false">ROUND(AG30/P30 *100/1000, 2)</f>
@@ -8639,13 +8640,13 @@
       <c r="L31" s="23" t="n">
         <v>50</v>
       </c>
-      <c r="M31" s="23" t="n">
+      <c r="M31" s="26" t="n">
         <f aca="false">O31*$M$37/100</f>
-        <v>191.2404</v>
+        <v>182.547654545455</v>
       </c>
       <c r="N31" s="24" t="n">
         <f aca="false">M31/$P31/10</f>
-        <v>0.196551213796789</v>
+        <v>0.187617067715117</v>
       </c>
       <c r="O31" s="23" t="n">
         <v>1300</v>
@@ -8659,31 +8660,31 @@
       </c>
       <c r="R31" s="23" t="n">
         <f aca="false">H31+F31+B31+D31+J31+M31</f>
-        <v>334.9074</v>
+        <v>326.214654545455</v>
       </c>
       <c r="S31" s="26" t="n">
         <f aca="false">R31/$P31/1000*100</f>
-        <v>0.344207897387408</v>
+        <v>0.335273751305736</v>
       </c>
       <c r="T31" s="26" t="n">
         <f aca="false">R31/P31</f>
-        <v>3.44207897387408</v>
+        <v>3.35273751305736</v>
       </c>
       <c r="U31" s="2" t="n">
         <f aca="false">3/5*H31+M31/3</f>
-        <v>75.1468</v>
+        <v>72.2492181818182</v>
       </c>
       <c r="V31" s="26" t="n">
         <f aca="false">U31/$P31/1000*100</f>
-        <v>0.0772336533125039</v>
+        <v>0.0742556046186131</v>
       </c>
       <c r="W31" s="2" t="n">
         <f aca="false">R31-U31</f>
-        <v>259.7606</v>
+        <v>253.965436363636</v>
       </c>
       <c r="X31" s="26" t="n">
         <f aca="false">W31/$P31/1000*100</f>
-        <v>0.266974244074904</v>
+        <v>0.261018146687122</v>
       </c>
       <c r="Y31" s="26"/>
       <c r="Z31" s="26"/>
@@ -8697,27 +8698,27 @@
       </c>
       <c r="AC31" s="2" t="n">
         <f aca="false">1000/100*Q31*($Q$41+$Q$47-$Q$49)-AA31</f>
-        <v>402.125504838226</v>
+        <v>393.215182550238</v>
       </c>
       <c r="AD31" s="26" t="n">
         <f aca="false">AC31/$P31/1000*100</f>
-        <v>0.413292672858872</v>
+        <v>0.404134907757855</v>
       </c>
       <c r="AE31" s="2" t="n">
         <f aca="false">AC31+Q31/100*1000 *($Q$46+$Q$43)</f>
-        <v>699.006738432019</v>
+        <v>685.641255000038</v>
       </c>
       <c r="AF31" s="26" t="n">
         <f aca="false">AE31/$P31/1000*100</f>
-        <v>0.718418403699993</v>
+        <v>0.704681756048467</v>
       </c>
       <c r="AG31" s="26" t="n">
         <f aca="false">-AA31+($Q$45 + $Q$46)*1000*Q31/100</f>
-        <v>335.29809193097</v>
+        <v>326.387769642982</v>
       </c>
       <c r="AH31" s="26" t="n">
         <f aca="false">AG31/P31/10</f>
-        <v>0.344609438971993</v>
+        <v>0.335451673870976</v>
       </c>
       <c r="AI31" s="26" t="n">
         <f aca="false">ROUND(AG31/P31 *100/1000, 2)</f>
@@ -8866,13 +8867,13 @@
       <c r="L32" s="23" t="n">
         <v>30</v>
       </c>
-      <c r="M32" s="23" t="n">
+      <c r="M32" s="26" t="n">
         <f aca="false">O32*$M$37/100</f>
-        <v>161.8188</v>
+        <v>154.4634</v>
       </c>
       <c r="N32" s="24" t="n">
         <f aca="false">M32/$P32/10</f>
-        <v>0.314388296322201</v>
+        <v>0.300097919216646</v>
       </c>
       <c r="O32" s="23" t="n">
         <v>1100</v>
@@ -8886,31 +8887,31 @@
       </c>
       <c r="R32" s="23" t="n">
         <f aca="false">H32+F32+B32+D32+J32+M32</f>
-        <v>291.219</v>
+        <v>283.8636</v>
       </c>
       <c r="S32" s="26" t="n">
         <f aca="false">R32/$P32/1000*100</f>
-        <v>0.565792387946611</v>
+        <v>0.551502010841056</v>
       </c>
       <c r="T32" s="26" t="n">
         <f aca="false">R32/P32</f>
-        <v>5.65792387946611</v>
+        <v>5.51502010841056</v>
       </c>
       <c r="U32" s="2" t="n">
         <f aca="false">3/5*H32+M32/3</f>
-        <v>98.9396</v>
+        <v>96.4878</v>
       </c>
       <c r="V32" s="26" t="n">
         <f aca="false">U32/$P32/1000*100</f>
-        <v>0.192223970779662</v>
+        <v>0.187460511744477</v>
       </c>
       <c r="W32" s="2" t="n">
         <f aca="false">R32-U32</f>
-        <v>192.2794</v>
+        <v>187.3758</v>
       </c>
       <c r="X32" s="26" t="n">
         <f aca="false">W32/$P32/1000*100</f>
-        <v>0.373568417166949</v>
+        <v>0.364041499096579</v>
       </c>
       <c r="Y32" s="26"/>
       <c r="Z32" s="26"/>
@@ -8924,27 +8925,27 @@
       </c>
       <c r="AC32" s="2" t="n">
         <f aca="false">1000/100*Q32*($Q$41+$Q$47-$Q$49)-AA32</f>
-        <v>212.72587164719</v>
+        <v>208.012278372046</v>
       </c>
       <c r="AD32" s="26" t="n">
         <f aca="false">AC32/$P32/1000*100</f>
-        <v>0.413292672858872</v>
+        <v>0.404134907757855</v>
       </c>
       <c r="AE32" s="2" t="n">
         <f aca="false">AC32+Q32/100*1000 *($Q$46+$Q$43)</f>
-        <v>369.777136568424</v>
+        <v>362.706746655707</v>
       </c>
       <c r="AF32" s="26" t="n">
         <f aca="false">AE32/$P32/1000*100</f>
-        <v>0.718418403699994</v>
+        <v>0.704681756048468</v>
       </c>
       <c r="AG32" s="26" t="n">
         <f aca="false">-AA32+($Q$45 + $Q$46)*1000*Q32/100</f>
-        <v>177.373924333275</v>
+        <v>172.66033105813</v>
       </c>
       <c r="AH32" s="26" t="n">
         <f aca="false">AG32/P32/10</f>
-        <v>0.344609438971994</v>
+        <v>0.335451673870976</v>
       </c>
       <c r="AI32" s="26" t="n">
         <f aca="false">ROUND(AG32/P32 *100/1000, 2)</f>
@@ -9092,13 +9093,13 @@
       <c r="L33" s="23" t="n">
         <v>9330</v>
       </c>
-      <c r="M33" s="23" t="n">
+      <c r="M33" s="26" t="n">
         <f aca="false">O33*$M$37/100</f>
-        <v>4545.6372</v>
+        <v>4339.01732727273</v>
       </c>
       <c r="N33" s="24" t="n">
         <f aca="false">M33/$P33/10</f>
-        <v>0.374689323469409</v>
+        <v>0.357657990584436</v>
       </c>
       <c r="O33" s="23" t="n">
         <v>30900</v>
@@ -9112,31 +9113,31 @@
       </c>
       <c r="R33" s="23" t="n">
         <f aca="false">H33+F33+B33+D33+J33+M33</f>
-        <v>10631.2994</v>
+        <v>10424.6795272727</v>
       </c>
       <c r="S33" s="26" t="n">
         <f aca="false">R33/$P33/1000*100</f>
-        <v>0.876320349496157</v>
+        <v>0.859289016611184</v>
       </c>
       <c r="T33" s="26" t="n">
         <f aca="false">R33/P33</f>
-        <v>8.76320349496157</v>
+        <v>8.59289016611184</v>
       </c>
       <c r="U33" s="2" t="n">
         <f aca="false">3/5*H33+M33/3</f>
-        <v>2805.8124</v>
+        <v>2736.93910909091</v>
       </c>
       <c r="V33" s="26" t="n">
         <f aca="false">U33/$P33/1000*100</f>
-        <v>0.23127845529293</v>
+        <v>0.225601344331272</v>
       </c>
       <c r="W33" s="2" t="n">
         <f aca="false">R33-U33</f>
-        <v>7825.487</v>
+        <v>7687.74041818182</v>
       </c>
       <c r="X33" s="26" t="n">
         <f aca="false">W33/$P33/1000*100</f>
-        <v>0.645041894203227</v>
+        <v>0.633687672279912</v>
       </c>
       <c r="Y33" s="26" t="n">
         <f aca="false">B33</f>
@@ -9156,31 +9157,31 @@
       </c>
       <c r="AC33" s="2" t="n">
         <f aca="false">1000/100*Q33*($Q$41+$Q$47-$Q$49)-AA33</f>
-        <v>4086.36338395562</v>
+        <v>3975.26366719136</v>
       </c>
       <c r="AD33" s="26" t="n">
         <f aca="false">AC33/$P33/1000*100</f>
-        <v>0.336832145729645</v>
+        <v>0.327674380628628</v>
       </c>
       <c r="AE33" s="2" t="n">
         <f aca="false">AC33+Q33/100*1000 *($Q$46+$Q$43)</f>
-        <v>7788.07246908739</v>
+        <v>7621.42289394099</v>
       </c>
       <c r="AF33" s="26" t="n">
         <f aca="false">AE33/$P33/1000*100</f>
-        <v>0.641957876570766</v>
+        <v>0.62822122891924</v>
       </c>
       <c r="AG33" s="26" t="n">
         <f aca="false">-AA33+($Q$45 + $Q$46)*1000*Q33/100</f>
-        <v>3253.11556124848</v>
+        <v>3142.01584448421</v>
       </c>
       <c r="AH33" s="26" t="n">
         <f aca="false">AG33/P33/10</f>
-        <v>0.268148911842766</v>
+        <v>0.258991146741749</v>
       </c>
       <c r="AI33" s="26" t="n">
         <f aca="false">ROUND(AG33/P33 *100/1000, 2)</f>
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="AK33" s="26" t="n">
         <f aca="false">-Q33*($Q$47)*10</f>
@@ -9324,13 +9325,13 @@
       <c r="L34" s="23" t="n">
         <v>1160</v>
       </c>
-      <c r="M34" s="23" t="n">
+      <c r="M34" s="26" t="n">
         <f aca="false">O34*$M$37/100</f>
-        <v>1044.4668</v>
+        <v>996.991036363636</v>
       </c>
       <c r="N34" s="24" t="n">
         <f aca="false">M34/$P34/10</f>
-        <v>0.188976041165338</v>
+        <v>0.180386221112368</v>
       </c>
       <c r="O34" s="23" t="n">
         <v>7100</v>
@@ -9344,31 +9345,31 @@
       </c>
       <c r="R34" s="23" t="n">
         <f aca="false">H34+F34+B34+D34+J34+M34</f>
-        <v>3063.2412</v>
+        <v>3015.76543636364</v>
       </c>
       <c r="S34" s="26" t="n">
         <f aca="false">R34/$P34/1000*100</f>
-        <v>0.554234174902026</v>
+        <v>0.545644354849056</v>
       </c>
       <c r="T34" s="26" t="n">
         <f aca="false">R34/P34</f>
-        <v>5.54234174902026</v>
+        <v>5.45644354849056</v>
       </c>
       <c r="U34" s="2" t="n">
         <f aca="false">3/5*H34+M34/3</f>
-        <v>775.3556</v>
+        <v>759.530345454546</v>
       </c>
       <c r="V34" s="26" t="n">
         <f aca="false">U34/$P34/1000*100</f>
-        <v>0.140285580913989</v>
+        <v>0.137422307562999</v>
       </c>
       <c r="W34" s="2" t="n">
         <f aca="false">R34-U34</f>
-        <v>2287.8856</v>
+        <v>2256.23509090909</v>
       </c>
       <c r="X34" s="26" t="n">
         <f aca="false">W34/$P34/1000*100</f>
-        <v>0.413948593988037</v>
+        <v>0.408222047286057</v>
       </c>
       <c r="Y34" s="26"/>
       <c r="Z34" s="26"/>
@@ -9382,27 +9383,27 @@
       </c>
       <c r="AC34" s="2" t="n">
         <f aca="false">1000/100*Q34*($Q$41+$Q$47-$Q$49)-AA34</f>
-        <v>2284.26033703753</v>
+        <v>2233.64555247951</v>
       </c>
       <c r="AD34" s="26" t="n">
         <f aca="false">AC34/$P34/1000*100</f>
-        <v>0.413292672858872</v>
+        <v>0.404134907757855</v>
       </c>
       <c r="AE34" s="2" t="n">
         <f aca="false">AC34+Q34/100*1000 *($Q$46+$Q$43)</f>
-        <v>3970.68414888178</v>
+        <v>3894.76197204475</v>
       </c>
       <c r="AF34" s="26" t="n">
         <f aca="false">AE34/$P34/1000*100</f>
-        <v>0.718418403699993</v>
+        <v>0.704681756048466</v>
       </c>
       <c r="AG34" s="26" t="n">
         <f aca="false">-AA34+($Q$45 + $Q$46)*1000*Q34/100</f>
-        <v>1904.64947700943</v>
+        <v>1854.0346924514</v>
       </c>
       <c r="AH34" s="26" t="n">
         <f aca="false">AG34/P34/10</f>
-        <v>0.344609438971993</v>
+        <v>0.335451673870976</v>
       </c>
       <c r="AI34" s="26" t="n">
         <f aca="false">ROUND(AG34/P34 *100/1000, 2)</f>
@@ -9548,13 +9549,13 @@
         <v>0.0721194560782395</v>
       </c>
       <c r="L35" s="23"/>
-      <c r="M35" s="23" t="n">
+      <c r="M35" s="26" t="n">
         <f aca="false">SUM(M8:M34)</f>
-        <v>44000.0028</v>
+        <v>42000.0026727273</v>
       </c>
       <c r="N35" s="24" t="n">
         <f aca="false">M35/$P35/10</f>
-        <v>0.302206248333573</v>
+        <v>0.288469600682047</v>
       </c>
       <c r="O35" s="23"/>
       <c r="P35" s="2" t="n">
@@ -9566,28 +9567,28 @@
       </c>
       <c r="R35" s="23" t="n">
         <f aca="false">H35+F35+B35+D35+J35+M35</f>
-        <v>104594.9028</v>
+        <v>102594.902672727</v>
       </c>
       <c r="S35" s="26" t="n">
         <f aca="false">R35/$P35/1000*100</f>
-        <v>0.718391617238778</v>
+        <v>0.704654969587251</v>
       </c>
       <c r="T35" s="26"/>
       <c r="U35" s="2" t="n">
         <f aca="false">3/5*H35+M35/3</f>
-        <v>30425.0676</v>
+        <v>29758.4008909091</v>
       </c>
       <c r="V35" s="26" t="n">
         <f aca="false">U35/$P35/1000*100</f>
-        <v>0.20896920339949</v>
+        <v>0.204390320848982</v>
       </c>
       <c r="W35" s="2" t="n">
         <f aca="false">R35-U35</f>
-        <v>74169.8352</v>
+        <v>72836.5017818182</v>
       </c>
       <c r="X35" s="26" t="n">
         <f aca="false">W35/$P35/1000*100</f>
-        <v>0.509422413839287</v>
+        <v>0.50026464873827</v>
       </c>
       <c r="Y35" s="23" t="n">
         <f aca="false">SUM(Y8:Y34)</f>
@@ -9607,28 +9608,28 @@
       </c>
       <c r="AC35" s="2" t="n">
         <f aca="false">1000/100*Q35*($Q$41+$Q$47-$Q$49)-AA35</f>
-        <v>53624.214821376</v>
+        <v>52290.8814031942</v>
       </c>
       <c r="AD35" s="26" t="n">
         <f aca="false">AC35/$P35/1000*100</f>
-        <v>0.368308448857681</v>
+        <v>0.359150683756664</v>
       </c>
       <c r="AE35" s="2" t="n">
         <f aca="false">AC35+Q35/100*1000 *($Q$46+$Q$43)</f>
-        <v>98049.282421376</v>
+        <v>96049.2822941033</v>
       </c>
       <c r="AF35" s="26" t="n">
         <f aca="false">AE35/$P35/1000*100</f>
-        <v>0.673434179698802</v>
+        <v>0.659697532047276</v>
       </c>
       <c r="AG35" s="26" t="n">
         <f aca="false">SUM(AG8:AG34)</f>
-        <v>43624.214821376</v>
+        <v>42290.8814031942</v>
       </c>
       <c r="AH35" s="23"/>
       <c r="AI35" s="36" t="n">
         <f aca="false">ROUND(AG35/P35 *100/1000, 2)</f>
-        <v>0.3</v>
+        <v>0.29</v>
       </c>
       <c r="AK35" s="26" t="n">
         <f aca="false">-Q35*($Q$47)*10</f>
@@ -9677,9 +9678,9 @@
         <f aca="false">SUM(L8:L34)</f>
         <v>45000</v>
       </c>
-      <c r="M36" s="1" t="n">
+      <c r="M36" s="2" t="n">
         <f aca="false">SUM(M8:M34)</f>
-        <v>44000.0028</v>
+        <v>42000.0026727273</v>
       </c>
       <c r="O36" s="1" t="n">
         <f aca="false">SUM(O8:O34)</f>
@@ -9692,7 +9693,7 @@
       <c r="Q36" s="2"/>
       <c r="R36" s="1" t="n">
         <f aca="false">SUM(R8:R34)</f>
-        <v>104598.8028</v>
+        <v>102598.802672727</v>
       </c>
       <c r="T36" s="2"/>
       <c r="Y36" s="2"/>
@@ -9703,8 +9704,9 @@
         <v>23.334</v>
       </c>
       <c r="K37" s="38"/>
-      <c r="M37" s="37" t="n">
-        <v>14.7108</v>
+      <c r="M37" s="38" t="n">
+        <f aca="false">14.7108*42/44</f>
+        <v>14.0421272727273</v>
       </c>
       <c r="N37" s="38"/>
     </row>
@@ -9714,7 +9716,7 @@
       </c>
       <c r="C38" s="40" t="n">
         <f aca="false">SUM(B35:M35)</f>
-        <v>104595.318985369</v>
+        <v>102595.318858096</v>
       </c>
       <c r="D38" s="40"/>
       <c r="E38" s="40"/>
@@ -9822,7 +9824,7 @@
       </c>
       <c r="Q43" s="46" t="n">
         <f aca="false">U35/1000</f>
-        <v>30.4250676</v>
+        <v>29.7584008909091</v>
       </c>
       <c r="R43" s="41"/>
       <c r="S43" s="41"/>
@@ -9848,7 +9850,7 @@
       </c>
       <c r="Q44" s="47" t="n">
         <f aca="false">R36/1000 -Q43</f>
-        <v>74.1737352</v>
+        <v>72.8404017818182</v>
       </c>
       <c r="R44" s="41"/>
       <c r="S44" s="41"/>
@@ -9874,7 +9876,7 @@
       </c>
       <c r="Q45" s="47" t="n">
         <f aca="false">Q44-Q46-Q47</f>
-        <v>36.1737352</v>
+        <v>34.8404017818182</v>
       </c>
       <c r="R45" s="41"/>
       <c r="S45" s="41"/>
@@ -9992,7 +9994,7 @@
       </c>
       <c r="Q49" s="47" t="n">
         <f aca="false">Q41-Q45</f>
-        <v>98.7862648</v>
+        <v>100.119598218182</v>
       </c>
       <c r="R49" s="41"/>
       <c r="S49" s="41"/>
@@ -10024,9 +10026,9 @@
       <c r="P50" s="45" t="s">
         <v>212</v>
       </c>
-      <c r="Q50" s="47" t="n">
+      <c r="Q50" s="45" t="n">
         <f aca="false">Q49/Q48</f>
-        <v>0.477689868471954</v>
+        <v>0.48413732213821</v>
       </c>
       <c r="R50" s="41"/>
       <c r="S50" s="41"/>

</xml_diff>